<commit_message>
Sync updated Master produk.xlsx DOI Min & DOI Max data values
</commit_message>
<xml_diff>
--- a/Master produk.xlsx
+++ b/Master produk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Argo\Project AI\DOI BULANAN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F84342B2-D06A-4952-BB74-14BCCB728294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4AD3A7F-E849-4CF6-8169-FC03A91F7171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7A4E4CA0-3C41-4699-9069-61742CAEF447}"/>
   </bookViews>
@@ -4200,7 +4200,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -4241,7 +4241,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -8074,7 +8074,7 @@
         <v>31.531882744630686</v>
       </c>
       <c r="M2" s="1">
-        <v>61.531882744630686</v>
+        <v>68.992082882567104</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -8114,7 +8114,7 @@
         <v>32.601499693858898</v>
       </c>
       <c r="M3" s="1">
-        <v>62.601499693858898</v>
+        <v>67.724444914043858</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
@@ -8154,7 +8154,7 @@
         <v>30.504473852092975</v>
       </c>
       <c r="M4" s="1">
-        <v>60.504473852092971</v>
+        <v>63.057629500816489</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -8194,7 +8194,7 @@
         <v>32.714140659424864</v>
       </c>
       <c r="M5" s="1">
-        <v>62.714140659424864</v>
+        <v>67.395120661156312</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -8234,7 +8234,7 @@
         <v>43.815214223258515</v>
       </c>
       <c r="M6" s="1">
-        <v>73.815214223258522</v>
+        <v>74.857498903232369</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -8274,7 +8274,7 @@
         <v>36.581038702563127</v>
       </c>
       <c r="M7" s="1">
-        <v>66.58103870256312</v>
+        <v>68.367113374611563</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -8313,7 +8313,7 @@
         <v>45</v>
       </c>
       <c r="M8" s="1">
-        <v>95</v>
+        <v>85.544968055479714</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -8352,7 +8352,7 @@
         <v>30</v>
       </c>
       <c r="M9" s="1">
-        <v>60</v>
+        <v>64.407659718853708</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -8391,7 +8391,7 @@
         <v>30</v>
       </c>
       <c r="M10" s="1">
-        <v>60</v>
+        <v>63.017912665437635</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -8431,7 +8431,7 @@
         <v>42.069893198288234</v>
       </c>
       <c r="M11" s="1">
-        <v>72.069893198288241</v>
+        <v>72.716749707397014</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
@@ -8474,7 +8474,7 @@
         <v>44.406049495875358</v>
       </c>
       <c r="M12" s="1">
-        <v>74.406049495875351</v>
+        <v>79.854510724204886</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -8513,7 +8513,7 @@
         <v>30</v>
       </c>
       <c r="M13" s="1">
-        <v>60</v>
+        <v>60.384379826708212</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
@@ -8553,7 +8553,7 @@
         <v>30.909068114288583</v>
       </c>
       <c r="M14" s="1">
-        <v>60.909068114288587</v>
+        <v>61.929237523829954</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -8593,7 +8593,7 @@
         <v>31.39723675452402</v>
       </c>
       <c r="M15" s="1">
-        <v>61.397236754524016</v>
+        <v>61.872064771143869</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
@@ -8633,7 +8633,7 @@
         <v>34.898587536684573</v>
       </c>
       <c r="M16" s="1">
-        <v>64.898587536684573</v>
+        <v>66.13137238016138</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -8672,7 +8672,7 @@
         <v>36.313250647764363</v>
       </c>
       <c r="M17" s="1">
-        <v>66.313250647764363</v>
+        <v>66.596219559607931</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
@@ -8712,7 +8712,7 @@
         <v>38.42278148735199</v>
       </c>
       <c r="M18" s="1">
-        <v>68.422781487351983</v>
+        <v>73.65562157688197</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
@@ -8752,7 +8752,7 @@
         <v>44.834118578266924</v>
       </c>
       <c r="M19" s="1">
-        <v>74.834118578266924</v>
+        <v>74.861427705264632</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
@@ -8792,7 +8792,7 @@
         <v>30.445754549841567</v>
       </c>
       <c r="M20" s="1">
-        <v>60.445754549841567</v>
+        <v>75.088995988007127</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
@@ -8832,7 +8832,7 @@
         <v>33.821892709822492</v>
       </c>
       <c r="M21" s="1">
-        <v>63.821892709822492</v>
+        <v>67.800439372909821</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
@@ -8872,7 +8872,7 @@
         <v>31.538898172883417</v>
       </c>
       <c r="M22" s="1">
-        <v>61.538898172883421</v>
+        <v>65.886286039203739</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
@@ -8912,7 +8912,7 @@
         <v>30.492933262791926</v>
       </c>
       <c r="M23" s="1">
-        <v>60.492933262791922</v>
+        <v>62.630620973341777</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
@@ -8952,7 +8952,7 @@
         <v>41.84002633311389</v>
       </c>
       <c r="M24" s="1">
-        <v>86.840026333113883</v>
+        <v>85.911981414409297</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
@@ -8992,7 +8992,7 @@
         <v>30.013555947001613</v>
       </c>
       <c r="M25" s="1">
-        <v>60.013555947001613</v>
+        <v>72.976720821025481</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
@@ -9032,7 +9032,7 @@
         <v>34.151901469317188</v>
       </c>
       <c r="M26" s="1">
-        <v>86.151901469317181</v>
+        <v>84.376667051225624</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
@@ -9071,7 +9071,7 @@
         <v>30</v>
       </c>
       <c r="M27" s="1">
-        <v>60</v>
+        <v>64.98063129482918</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
@@ -9111,7 +9111,7 @@
         <v>40.772475337260786</v>
       </c>
       <c r="M28" s="1">
-        <v>70.772475337260786</v>
+        <v>82.745246773257662</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
@@ -9190,7 +9190,7 @@
         <v>31.683238335006983</v>
       </c>
       <c r="M30" s="1">
-        <v>73.68323833500699</v>
+        <v>77.541785261196992</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
@@ -9229,7 +9229,7 @@
         <v>35.626787416587227</v>
       </c>
       <c r="M31" s="1">
-        <v>221.62678741658723</v>
+        <v>225.84906391878553</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
@@ -9269,7 +9269,7 @@
         <v>35.50668245643714</v>
       </c>
       <c r="M32" s="1">
-        <v>65.506682456437147</v>
+        <v>66.258264246220136</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
@@ -9309,7 +9309,7 @@
         <v>35.923527755739244</v>
       </c>
       <c r="M33" s="1">
-        <v>65.923527755739244</v>
+        <v>73.336831516805347</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
@@ -9388,7 +9388,7 @@
         <v>37.179123463682025</v>
       </c>
       <c r="M35" s="1">
-        <v>67.179123463682032</v>
+        <v>67.805500548982621</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
@@ -9428,7 +9428,7 @@
         <v>31.884614329978895</v>
       </c>
       <c r="M36" s="1">
-        <v>61.884614329978895</v>
+        <v>76.857434946044918</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
@@ -9468,7 +9468,7 @@
         <v>35.067074492425533</v>
       </c>
       <c r="M37" s="1">
-        <v>91.067074492425533</v>
+        <v>92.38971544490019</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
@@ -9507,7 +9507,7 @@
         <v>30</v>
       </c>
       <c r="M38" s="1">
-        <v>60</v>
+        <v>63.93672177227922</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
@@ -9547,7 +9547,7 @@
         <v>36.001221415484828</v>
       </c>
       <c r="M39" s="1">
-        <v>66.001221415484821</v>
+        <v>73.166163442663475</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
@@ -9629,7 +9629,7 @@
         <v>36.61000326904216</v>
       </c>
       <c r="M41" s="1">
-        <v>66.610003269042153</v>
+        <v>80.863776631194128</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
@@ -9669,7 +9669,7 @@
         <v>32.569679489066132</v>
       </c>
       <c r="M42" s="1">
-        <v>62.569679489066132</v>
+        <v>64.98861209756555</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
@@ -9709,7 +9709,7 @@
         <v>42.134124507647456</v>
       </c>
       <c r="M43" s="1">
-        <v>72.134124507647456</v>
+        <v>83.696549391066526</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
@@ -9748,7 +9748,7 @@
         <v>43.279690364636387</v>
       </c>
       <c r="M44" s="1">
-        <v>73.279690364636394</v>
+        <v>74.128695294342421</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
@@ -9788,7 +9788,7 @@
         <v>35.291408807842139</v>
       </c>
       <c r="M45" s="1">
-        <v>65.291408807842146</v>
+        <v>70.852834450485261</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
@@ -9828,7 +9828,7 @@
         <v>39.614393182176855</v>
       </c>
       <c r="M46" s="1">
-        <v>86.614393182176855</v>
+        <v>85.727869991936331</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.3">
@@ -9868,7 +9868,7 @@
         <v>35.634830180077508</v>
       </c>
       <c r="M47" s="1">
-        <v>65.6348301800775</v>
+        <v>73.113495812350592</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.3">
@@ -9908,7 +9908,7 @@
         <v>41.764830508474574</v>
       </c>
       <c r="M48" s="1">
-        <v>297.76483050847457</v>
+        <v>290.84487583658824</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.3">
@@ -9948,7 +9948,7 @@
         <v>38.162488653027026</v>
       </c>
       <c r="M49" s="1">
-        <v>102.16248865302703</v>
+        <v>101.59010813034628</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.3">
@@ -9988,7 +9988,7 @@
         <v>36.751023720810117</v>
       </c>
       <c r="M50" s="1">
-        <v>68.75102372081011</v>
+        <v>68.977967812647407</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.3">
@@ -10028,7 +10028,7 @@
         <v>35.899570473364925</v>
       </c>
       <c r="M51" s="1">
-        <v>65.899570473364918</v>
+        <v>74.592313654013424</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.3">
@@ -10068,7 +10068,7 @@
         <v>34.204425711275036</v>
       </c>
       <c r="M52" s="1">
-        <v>64.204425711275036</v>
+        <v>70.719143961905829</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.3">
@@ -10108,7 +10108,7 @@
         <v>42.438486962908556</v>
       </c>
       <c r="M53" s="1">
-        <v>123.43848696290856</v>
+        <v>119.34018894276268</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.3">
@@ -10148,7 +10148,7 @@
         <v>31.787990739929391</v>
       </c>
       <c r="M54" s="1">
-        <v>61.787990739929391</v>
+        <v>62.762107509652537</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.3">
@@ -10188,7 +10188,7 @@
         <v>38.885029557746435</v>
       </c>
       <c r="M55" s="1">
-        <v>111.88502955774644</v>
+        <v>107.63100443189037</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.3">
@@ -10228,7 +10228,7 @@
         <v>32.137857281742171</v>
       </c>
       <c r="M56" s="1">
-        <v>62.137857281742171</v>
+        <v>66.430115507285763</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.3">
@@ -10268,7 +10268,7 @@
         <v>42.044576188510753</v>
       </c>
       <c r="M57" s="1">
-        <v>88.044576188510746</v>
+        <v>85.264603532813254</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.3">
@@ -10308,7 +10308,7 @@
         <v>35.347981507077826</v>
       </c>
       <c r="M58" s="1">
-        <v>65.347981507077833</v>
+        <v>68.924930599308738</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.3">
@@ -10348,7 +10348,7 @@
         <v>34.684808172334684</v>
       </c>
       <c r="M59" s="1">
-        <v>64.684808172334684</v>
+        <v>66.772701611132277</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.3">
@@ -10388,7 +10388,7 @@
         <v>40.631173211274401</v>
       </c>
       <c r="M60" s="1">
-        <v>258.63117321127442</v>
+        <v>246.30171474799118</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.3">
@@ -10428,7 +10428,7 @@
         <v>36.089721553798547</v>
       </c>
       <c r="M61" s="1">
-        <v>111.08972155379854</v>
+        <v>108.0688537167664</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.3">
@@ -10468,7 +10468,7 @@
         <v>39.838576840718183</v>
       </c>
       <c r="M62" s="1">
-        <v>239.83857684071819</v>
+        <v>227.91466492094148</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.3">
@@ -10508,7 +10508,7 @@
         <v>41.140577675999111</v>
       </c>
       <c r="M63" s="1">
-        <v>169.14057767599911</v>
+        <v>186.5182059350403</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.3">
@@ -10548,7 +10548,7 @@
         <v>37.821011673151752</v>
       </c>
       <c r="M64" s="1">
-        <v>94.821011673151759</v>
+        <v>90.470850170579695</v>
       </c>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.3">
@@ -10588,7 +10588,7 @@
         <v>39.293075547227666</v>
       </c>
       <c r="M65" s="1">
-        <v>169.29307554722766</v>
+        <v>151.56193378027729</v>
       </c>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.3">
@@ -10628,7 +10628,7 @@
         <v>40.012763241863432</v>
       </c>
       <c r="M66" s="1">
-        <v>93.012763241863439</v>
+        <v>91.69909507855553</v>
       </c>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.3">
@@ -10668,7 +10668,7 @@
         <v>40.958864426419467</v>
       </c>
       <c r="M67" s="1">
-        <v>93.958864426419467</v>
+        <v>93.747703257984625</v>
       </c>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.3">
@@ -10747,7 +10747,7 @@
         <v>43.106222865412448</v>
       </c>
       <c r="M69" s="1">
-        <v>73.106222865412448</v>
+        <v>76.120230525031559</v>
       </c>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.3">
@@ -10787,7 +10787,7 @@
         <v>39.080678164279462</v>
       </c>
       <c r="M70" s="1">
-        <v>69.080678164279462</v>
+        <v>70.985503722359937</v>
       </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.3">
@@ -10827,7 +10827,7 @@
         <v>41.635049683830175</v>
       </c>
       <c r="M71" s="1">
-        <v>71.635049683830175</v>
+        <v>73.984711537239065</v>
       </c>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.3">
@@ -10867,7 +10867,7 @@
         <v>42.375941891249759</v>
       </c>
       <c r="M72" s="1">
-        <v>72.375941891249767</v>
+        <v>73.27085845590409</v>
       </c>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.3">
@@ -10906,7 +10906,7 @@
         <v>30</v>
       </c>
       <c r="M73" s="1">
-        <v>60</v>
+        <v>68.210662637599825</v>
       </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.3">
@@ -10946,7 +10946,7 @@
         <v>35.291401837516744</v>
       </c>
       <c r="M74" s="1">
-        <v>65.291401837516744</v>
+        <v>89.891587079875492</v>
       </c>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.3">
@@ -10986,7 +10986,7 @@
         <v>37.192887931034484</v>
       </c>
       <c r="M75" s="1">
-        <v>83.192887931034477</v>
+        <v>81.656340497130913</v>
       </c>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.3">
@@ -11025,7 +11025,7 @@
         <v>30</v>
       </c>
       <c r="M76" s="1">
-        <v>60</v>
+        <v>63.03267500487479</v>
       </c>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.3">
@@ -11065,7 +11065,7 @@
         <v>31.300211416490491</v>
       </c>
       <c r="M77" s="1">
-        <v>107.3002114164905</v>
+        <v>160.61195230717874</v>
       </c>
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.3">
@@ -11108,7 +11108,7 @@
         <v>34.911838790931981</v>
       </c>
       <c r="M78" s="1">
-        <v>64.911838790931981</v>
+        <v>76.476702810938235</v>
       </c>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.3">
@@ -11150,7 +11150,7 @@
         <v>45</v>
       </c>
       <c r="M79" s="1">
-        <v>115</v>
+        <v>97.047128129602356</v>
       </c>
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.3">
@@ -11193,7 +11193,7 @@
         <v>36.929176708388397</v>
       </c>
       <c r="M80" s="1">
-        <v>596.92917670838835</v>
+        <v>605.60136605750074</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.3">
@@ -11236,7 +11236,7 @@
         <v>30.800751387007999</v>
       </c>
       <c r="M81" s="1">
-        <v>186.80075138700801</v>
+        <v>167.00474758110886</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.3">
@@ -11278,7 +11278,7 @@
         <v>30</v>
       </c>
       <c r="M82" s="1">
-        <v>95</v>
+        <v>109.15449090825814</v>
       </c>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.3">
@@ -11321,7 +11321,7 @@
         <v>38.271724137931031</v>
       </c>
       <c r="M83" s="1">
-        <v>530.27172413793107</v>
+        <v>588.53323767646373</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.3">
@@ -11364,7 +11364,7 @@
         <v>35.877462195190006</v>
       </c>
       <c r="M84" s="1">
-        <v>136.87746219518999</v>
+        <v>152.59612118166336</v>
       </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.3">
@@ -11407,7 +11407,7 @@
         <v>34.432377693194127</v>
       </c>
       <c r="M85" s="1">
-        <v>95.432377693194127</v>
+        <v>100.95636802802325</v>
       </c>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.3">
@@ -11446,7 +11446,7 @@
         <v>30</v>
       </c>
       <c r="M86" s="1">
-        <v>60</v>
+        <v>61.267421664623782</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.3">
@@ -11486,7 +11486,7 @@
         <v>30.318637463469816</v>
       </c>
       <c r="M87" s="1">
-        <v>60.318637463469813</v>
+        <v>64.508759608982302</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.3">
@@ -11525,7 +11525,7 @@
         <v>30</v>
       </c>
       <c r="M88" s="1">
-        <v>60</v>
+        <v>62.179467446513776</v>
       </c>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.3">
@@ -11565,7 +11565,7 @@
         <v>31.531002806838472</v>
       </c>
       <c r="M89" s="1">
-        <v>61.531002806838472</v>
+        <v>71.337263881853232</v>
       </c>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.3">
@@ -11604,7 +11604,7 @@
         <v>30</v>
       </c>
       <c r="M90" s="1">
-        <v>121</v>
+        <v>109.05154639175257</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.3">
@@ -11643,7 +11643,7 @@
         <v>30</v>
       </c>
       <c r="M91" s="1">
-        <v>165</v>
+        <v>164.19607843137257</v>
       </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.3">
@@ -11682,7 +11682,7 @@
         <v>30</v>
       </c>
       <c r="M92" s="1">
-        <v>60</v>
+        <v>71.485766478916133</v>
       </c>
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.3">
@@ -11722,7 +11722,7 @@
         <v>35.033303182304081</v>
       </c>
       <c r="M93" s="1">
-        <v>65.033303182304081</v>
+        <v>77.089682700423822</v>
       </c>
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.3">
@@ -11762,7 +11762,7 @@
         <v>36.443840672579064</v>
       </c>
       <c r="M94" s="1">
-        <v>75.443840672579057</v>
+        <v>76.459812169599758</v>
       </c>
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.3">
@@ -11802,7 +11802,7 @@
         <v>31.565762004175365</v>
       </c>
       <c r="M95" s="1">
-        <v>130.56576200417535</v>
+        <v>142.44691902494426</v>
       </c>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.3">
@@ -11842,7 +11842,7 @@
         <v>30.875106202209011</v>
       </c>
       <c r="M96" s="1">
-        <v>62.875106202209011</v>
+        <v>64.039960742320673</v>
       </c>
     </row>
     <row r="97" spans="1:13" x14ac:dyDescent="0.3">
@@ -11885,7 +11885,7 @@
         <v>34.449881168740376</v>
       </c>
       <c r="M97" s="1">
-        <v>77.449881168740376</v>
+        <v>81.967459890843713</v>
       </c>
     </row>
     <row r="98" spans="1:13" x14ac:dyDescent="0.3">
@@ -11928,7 +11928,7 @@
         <v>35.023775864284787</v>
       </c>
       <c r="M98" s="1">
-        <v>250.0237758642848</v>
+        <v>252.77553230456579</v>
       </c>
     </row>
     <row r="99" spans="1:13" x14ac:dyDescent="0.3">
@@ -11968,7 +11968,7 @@
         <v>44.615254510309271</v>
       </c>
       <c r="M99" s="1">
-        <v>74.615254510309271</v>
+        <v>77.619360123853482</v>
       </c>
     </row>
     <row r="100" spans="1:13" x14ac:dyDescent="0.3">
@@ -12008,7 +12008,7 @@
         <v>33.594126749919027</v>
       </c>
       <c r="M100" s="1">
-        <v>72.594126749919027</v>
+        <v>69.824311910435895</v>
       </c>
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.3">
@@ -12125,7 +12125,7 @@
         <v>30</v>
       </c>
       <c r="M103" s="1">
-        <v>69</v>
+        <v>66.729500471253544</v>
       </c>
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.3">
@@ -12165,7 +12165,7 @@
         <v>36.854384553499607</v>
       </c>
       <c r="M104" s="1">
-        <v>66.854384553499614</v>
+        <v>84.778540192448858</v>
       </c>
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.3">
@@ -12204,7 +12204,7 @@
         <v>30.774870854857522</v>
       </c>
       <c r="M105" s="1">
-        <v>68.774870854857525</v>
+        <v>67.687448040427881</v>
       </c>
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.3">
@@ -12243,7 +12243,7 @@
         <v>33.505948215535341</v>
       </c>
       <c r="M106" s="1">
-        <v>107.50594821553534</v>
+        <v>115.93848634615716</v>
       </c>
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.3">
@@ -12282,7 +12282,7 @@
         <v>33.376792698826591</v>
       </c>
       <c r="M107" s="1">
-        <v>72.376792698826591</v>
+        <v>74.037579064501585</v>
       </c>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.3">
@@ -12321,7 +12321,7 @@
         <v>42.430939226519335</v>
       </c>
       <c r="M108" s="1">
-        <v>188.43093922651934</v>
+        <v>205.55208912384992</v>
       </c>
     </row>
     <row r="109" spans="1:13" x14ac:dyDescent="0.3">
@@ -12360,7 +12360,7 @@
         <v>31.954848640328368</v>
       </c>
       <c r="M109" s="1">
-        <v>217.95484864032838</v>
+        <v>228.33621375408785</v>
       </c>
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.3">
@@ -12400,7 +12400,7 @@
         <v>32.52365124009205</v>
       </c>
       <c r="M110" s="1">
-        <v>62.52365124009205</v>
+        <v>83.785488967248455</v>
       </c>
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.3">
@@ -12440,7 +12440,7 @@
         <v>32.359169843286736</v>
       </c>
       <c r="M111" s="1">
-        <v>62.359169843286736</v>
+        <v>76.778271075937425</v>
       </c>
     </row>
     <row r="112" spans="1:13" x14ac:dyDescent="0.3">
@@ -12480,7 +12480,7 @@
         <v>35.328083989501316</v>
       </c>
       <c r="M112" s="1">
-        <v>104.32808398950132</v>
+        <v>111.74647777188474</v>
       </c>
     </row>
     <row r="113" spans="1:13" x14ac:dyDescent="0.3">
@@ -12520,7 +12520,7 @@
         <v>35.119906868451686</v>
       </c>
       <c r="M113" s="1">
-        <v>158.11990686845169</v>
+        <v>167.2036556221905</v>
       </c>
     </row>
     <row r="114" spans="1:13" x14ac:dyDescent="0.3">
@@ -12559,7 +12559,7 @@
         <v>39.83259220507454</v>
       </c>
       <c r="M114" s="1">
-        <v>168.83259220507455</v>
+        <v>179.97981757313795</v>
       </c>
     </row>
     <row r="115" spans="1:13" x14ac:dyDescent="0.3">
@@ -12599,7 +12599,7 @@
         <v>33.566263558159832</v>
       </c>
       <c r="M115" s="1">
-        <v>63.566263558159832</v>
+        <v>90.664323100095103</v>
       </c>
     </row>
     <row r="116" spans="1:13" x14ac:dyDescent="0.3">
@@ -12639,7 +12639,7 @@
         <v>32.580816110227872</v>
       </c>
       <c r="M116" s="1">
-        <v>62.580816110227872</v>
+        <v>63.443335712946116</v>
       </c>
     </row>
     <row r="117" spans="1:13" x14ac:dyDescent="0.3">
@@ -12677,7 +12677,7 @@
         <v>30</v>
       </c>
       <c r="M117" s="1">
-        <v>60</v>
+        <v>74.575378538512183</v>
       </c>
     </row>
     <row r="118" spans="1:13" x14ac:dyDescent="0.3">
@@ -12716,7 +12716,7 @@
         <v>31.298926220990648</v>
       </c>
       <c r="M118" s="1">
-        <v>136.29892622099064</v>
+        <v>137.06305741429142</v>
       </c>
     </row>
     <row r="119" spans="1:13" x14ac:dyDescent="0.3">
@@ -12756,7 +12756,7 @@
         <v>39.772614928324273</v>
       </c>
       <c r="M119" s="1">
-        <v>188.77261492832429</v>
+        <v>192.09431447308907</v>
       </c>
     </row>
     <row r="120" spans="1:13" x14ac:dyDescent="0.3">
@@ -12795,7 +12795,7 @@
         <v>38.571428571428569</v>
       </c>
       <c r="M120" s="1">
-        <v>279.57142857142856</v>
+        <v>270.25637373593503</v>
       </c>
     </row>
     <row r="121" spans="1:13" x14ac:dyDescent="0.3">
@@ -12835,7 +12835,7 @@
         <v>32.898540405838382</v>
       </c>
       <c r="M121" s="1">
-        <v>62.898540405838382</v>
+        <v>73.714407616416537</v>
       </c>
     </row>
     <row r="122" spans="1:13" x14ac:dyDescent="0.3">
@@ -12875,7 +12875,7 @@
         <v>32.945582211819783</v>
       </c>
       <c r="M122" s="1">
-        <v>62.945582211819783</v>
+        <v>77.271738075848617</v>
       </c>
     </row>
     <row r="123" spans="1:13" x14ac:dyDescent="0.3">
@@ -12914,7 +12914,7 @@
         <v>30</v>
       </c>
       <c r="M123" s="1">
-        <v>163</v>
+        <v>160.11815252416756</v>
       </c>
     </row>
     <row r="124" spans="1:13" x14ac:dyDescent="0.3">
@@ -12954,7 +12954,7 @@
         <v>34.348437939769212</v>
       </c>
       <c r="M124" s="1">
-        <v>299.34843793976921</v>
+        <v>293.29875669114324</v>
       </c>
     </row>
     <row r="125" spans="1:13" x14ac:dyDescent="0.3">
@@ -12993,7 +12993,7 @@
         <v>34.078629475071388</v>
       </c>
       <c r="M125" s="1">
-        <v>85.078629475071381</v>
+        <v>86.872613066684892</v>
       </c>
     </row>
     <row r="126" spans="1:13" x14ac:dyDescent="0.3">
@@ -13031,7 +13031,7 @@
         <v>30</v>
       </c>
       <c r="M126" s="1">
-        <v>60</v>
+        <v>92.448214843343393</v>
       </c>
     </row>
     <row r="127" spans="1:13" x14ac:dyDescent="0.3">
@@ -13070,7 +13070,7 @@
         <v>33.192660550458726</v>
       </c>
       <c r="M127" s="1">
-        <v>238.19266055045873</v>
+        <v>251.41183863265056</v>
       </c>
     </row>
     <row r="128" spans="1:13" x14ac:dyDescent="0.3">
@@ -13109,7 +13109,7 @@
         <v>40.543130990415335</v>
       </c>
       <c r="M128" s="1">
-        <v>434.54313099041531</v>
+        <v>400.28035726778751</v>
       </c>
     </row>
     <row r="129" spans="1:13" x14ac:dyDescent="0.3">
@@ -13149,7 +13149,7 @@
         <v>33.857965451055662</v>
       </c>
       <c r="M129" s="1">
-        <v>698.85796545105563</v>
+        <v>895.79826395851831</v>
       </c>
     </row>
     <row r="130" spans="1:13" x14ac:dyDescent="0.3">
@@ -13188,7 +13188,7 @@
         <v>44.20774647887324</v>
       </c>
       <c r="M130" s="1">
-        <v>494.20774647887322</v>
+        <v>453.53466955579637</v>
       </c>
     </row>
     <row r="131" spans="1:13" x14ac:dyDescent="0.3">
@@ -13227,7 +13227,7 @@
         <v>30</v>
       </c>
       <c r="M131" s="1">
-        <v>60</v>
+        <v>61.817520523745195</v>
       </c>
     </row>
     <row r="132" spans="1:13" x14ac:dyDescent="0.3">
@@ -13266,7 +13266,7 @@
         <v>34.816901408450704</v>
       </c>
       <c r="M132" s="1">
-        <v>163.81690140845069</v>
+        <v>164.61803777208706</v>
       </c>
     </row>
     <row r="133" spans="1:13" x14ac:dyDescent="0.3">
@@ -13305,7 +13305,7 @@
         <v>30</v>
       </c>
       <c r="M133" s="1">
-        <v>63</v>
+        <v>64.338544798556825</v>
       </c>
     </row>
     <row r="134" spans="1:13" x14ac:dyDescent="0.3">
@@ -13344,7 +13344,7 @@
         <v>32.253829321663019</v>
       </c>
       <c r="M134" s="1">
-        <v>66.253829321663019</v>
+        <v>66.738781609404626</v>
       </c>
     </row>
     <row r="135" spans="1:13" x14ac:dyDescent="0.3">
@@ -13382,7 +13382,7 @@
         <v>30</v>
       </c>
       <c r="M135" s="1">
-        <v>60</v>
+        <v>248.51731952088053</v>
       </c>
     </row>
     <row r="136" spans="1:13" x14ac:dyDescent="0.3">
@@ -13420,7 +13420,7 @@
         <v>30</v>
       </c>
       <c r="M136" s="1">
-        <v>60</v>
+        <v>81.835355552142545</v>
       </c>
     </row>
     <row r="137" spans="1:13" x14ac:dyDescent="0.3">
@@ -13458,7 +13458,7 @@
         <v>30</v>
       </c>
       <c r="M137" s="1">
-        <v>60</v>
+        <v>501.36871508379892</v>
       </c>
     </row>
     <row r="138" spans="1:13" x14ac:dyDescent="0.3">
@@ -13535,7 +13535,7 @@
         <v>30</v>
       </c>
       <c r="M139" s="1">
-        <v>60</v>
+        <v>120.64965586704719</v>
       </c>
     </row>
     <row r="140" spans="1:13" x14ac:dyDescent="0.3">
@@ -13573,7 +13573,7 @@
         <v>30</v>
       </c>
       <c r="M140" s="1">
-        <v>60</v>
+        <v>250.74694224605926</v>
       </c>
     </row>
     <row r="141" spans="1:13" x14ac:dyDescent="0.3">
@@ -13654,7 +13654,7 @@
         <v>30</v>
       </c>
       <c r="M142" s="1">
-        <v>60</v>
+        <v>62.842275597296698</v>
       </c>
     </row>
     <row r="143" spans="1:13" x14ac:dyDescent="0.3">
@@ -13694,7 +13694,7 @@
         <v>30.323016958336979</v>
       </c>
       <c r="M143" s="1">
-        <v>60.323016958336979</v>
+        <v>69.256915688393761</v>
       </c>
     </row>
     <row r="144" spans="1:13" x14ac:dyDescent="0.3">
@@ -13733,7 +13733,7 @@
         <v>30</v>
       </c>
       <c r="M144" s="1">
-        <v>60</v>
+        <v>62.193160800583783</v>
       </c>
     </row>
     <row r="145" spans="1:13" x14ac:dyDescent="0.3">
@@ -13772,7 +13772,7 @@
         <v>30</v>
       </c>
       <c r="M145" s="1">
-        <v>60</v>
+        <v>60.021830616803975</v>
       </c>
     </row>
     <row r="146" spans="1:13" x14ac:dyDescent="0.3">
@@ -13815,7 +13815,7 @@
         <v>35.772558714462299</v>
       </c>
       <c r="M146" s="1">
-        <v>86.772558714462292</v>
+        <v>85.516079595353943</v>
       </c>
     </row>
     <row r="147" spans="1:13" x14ac:dyDescent="0.3">
@@ -13858,7 +13858,7 @@
         <v>32.307263089370402</v>
       </c>
       <c r="M147" s="1">
-        <v>67.307263089370394</v>
+        <v>68.437772534132847</v>
       </c>
     </row>
     <row r="148" spans="1:13" x14ac:dyDescent="0.3">
@@ -13898,7 +13898,7 @@
         <v>43.500131616882058</v>
       </c>
       <c r="M148" s="1">
-        <v>73.500131616882058</v>
+        <v>87.288533913431436</v>
       </c>
     </row>
     <row r="149" spans="1:13" x14ac:dyDescent="0.3">
@@ -13938,7 +13938,7 @@
         <v>39.00584795321636</v>
       </c>
       <c r="M149" s="1">
-        <v>121.00584795321636</v>
+        <v>118.16959165872076</v>
       </c>
     </row>
     <row r="150" spans="1:13" x14ac:dyDescent="0.3">
@@ -13977,7 +13977,7 @@
         <v>30</v>
       </c>
       <c r="M150" s="1">
-        <v>123</v>
+        <v>124.85898468976629</v>
       </c>
     </row>
     <row r="151" spans="1:13" x14ac:dyDescent="0.3">
@@ -14017,7 +14017,7 @@
         <v>31.887258543833575</v>
       </c>
       <c r="M151" s="1">
-        <v>61.887258543833575</v>
+        <v>67.5264683707926</v>
       </c>
     </row>
     <row r="152" spans="1:13" x14ac:dyDescent="0.3">
@@ -14056,7 +14056,7 @@
         <v>30</v>
       </c>
       <c r="M152" s="1">
-        <v>60</v>
+        <v>65.747238034891197</v>
       </c>
     </row>
     <row r="153" spans="1:13" x14ac:dyDescent="0.3">
@@ -14095,7 +14095,7 @@
         <v>30</v>
       </c>
       <c r="M153" s="1">
-        <v>60</v>
+        <v>69.658617400471911</v>
       </c>
     </row>
     <row r="154" spans="1:13" x14ac:dyDescent="0.3">
@@ -14177,7 +14177,7 @@
         <v>36.321073547520427</v>
       </c>
       <c r="M155" s="1">
-        <v>66.321073547520427</v>
+        <v>67.454364925161144</v>
       </c>
     </row>
     <row r="156" spans="1:13" x14ac:dyDescent="0.3">
@@ -14217,7 +14217,7 @@
         <v>31.336825902930883</v>
       </c>
       <c r="M156" s="1">
-        <v>93.336825902930883</v>
+        <v>61.340846673841298</v>
       </c>
     </row>
     <row r="157" spans="1:13" x14ac:dyDescent="0.3">
@@ -14295,7 +14295,7 @@
         <v>30</v>
       </c>
       <c r="M158" s="1">
-        <v>60</v>
+        <v>60.684058431099764</v>
       </c>
     </row>
     <row r="159" spans="1:13" x14ac:dyDescent="0.3">
@@ -14335,7 +14335,7 @@
         <v>36.619708413841572</v>
       </c>
       <c r="M159" s="1">
-        <v>127.61970841384158</v>
+        <v>141.75955438060282</v>
       </c>
     </row>
     <row r="160" spans="1:13" x14ac:dyDescent="0.3">
@@ -14375,7 +14375,7 @@
         <v>39.434577779882105</v>
       </c>
       <c r="M160" s="1">
-        <v>69.434577779882105</v>
+        <v>69.92781236494389</v>
       </c>
     </row>
     <row r="161" spans="1:13" x14ac:dyDescent="0.3">
@@ -14417,7 +14417,7 @@
         <v>30</v>
       </c>
       <c r="M161" s="1">
-        <v>60</v>
+        <v>60.382587342557031</v>
       </c>
     </row>
     <row r="162" spans="1:13" x14ac:dyDescent="0.3">
@@ -14460,7 +14460,7 @@
         <v>34.013510365711632</v>
       </c>
       <c r="M162" s="1">
-        <v>64.013510365711625</v>
+        <v>66.176440036652423</v>
       </c>
     </row>
     <row r="163" spans="1:13" x14ac:dyDescent="0.3">
@@ -14500,7 +14500,7 @@
         <v>31.310018949126409</v>
       </c>
       <c r="M163" s="1">
-        <v>61.310018949126409</v>
+        <v>61.339162139334292</v>
       </c>
     </row>
     <row r="164" spans="1:13" x14ac:dyDescent="0.3">
@@ -14540,7 +14540,7 @@
         <v>31.434307074622726</v>
       </c>
       <c r="M164" s="1">
-        <v>61.434307074622723</v>
+        <v>63.257711475801848</v>
       </c>
     </row>
     <row r="165" spans="1:13" x14ac:dyDescent="0.3">
@@ -14579,7 +14579,7 @@
         <v>30</v>
       </c>
       <c r="M165" s="1">
-        <v>60</v>
+        <v>60.122308908867744</v>
       </c>
     </row>
     <row r="166" spans="1:13" x14ac:dyDescent="0.3">
@@ -14618,7 +14618,7 @@
         <v>30</v>
       </c>
       <c r="M166" s="1">
-        <v>60</v>
+        <v>61.763981528989234</v>
       </c>
     </row>
     <row r="167" spans="1:13" x14ac:dyDescent="0.3">
@@ -14657,7 +14657,7 @@
         <v>30</v>
       </c>
       <c r="M167" s="1">
-        <v>60</v>
+        <v>63.854641093078456</v>
       </c>
     </row>
     <row r="168" spans="1:13" x14ac:dyDescent="0.3">
@@ -14696,7 +14696,7 @@
         <v>30</v>
       </c>
       <c r="M168" s="1">
-        <v>60</v>
+        <v>64.454601934853997</v>
       </c>
     </row>
     <row r="169" spans="1:13" x14ac:dyDescent="0.3">
@@ -14735,7 +14735,7 @@
         <v>30</v>
       </c>
       <c r="M169" s="1">
-        <v>60</v>
+        <v>60.199501246882789</v>
       </c>
     </row>
     <row r="170" spans="1:13" x14ac:dyDescent="0.3">
@@ -14774,7 +14774,7 @@
         <v>30</v>
       </c>
       <c r="M170" s="1">
-        <v>60</v>
+        <v>61.292034067598195</v>
       </c>
     </row>
     <row r="171" spans="1:13" x14ac:dyDescent="0.3">
@@ -14814,7 +14814,7 @@
         <v>35.958196245403514</v>
       </c>
       <c r="M171" s="1">
-        <v>68.958196245403514</v>
+        <v>73.989046840379274</v>
       </c>
     </row>
     <row r="172" spans="1:13" x14ac:dyDescent="0.3">
@@ -14854,7 +14854,7 @@
         <v>31.960053690162155</v>
       </c>
       <c r="M172" s="1">
-        <v>61.960053690162155</v>
+        <v>65.988205251663828</v>
       </c>
     </row>
     <row r="173" spans="1:13" x14ac:dyDescent="0.3">
@@ -14893,7 +14893,7 @@
         <v>30</v>
       </c>
       <c r="M173" s="1">
-        <v>60</v>
+        <v>61.942437498762843</v>
       </c>
     </row>
     <row r="174" spans="1:13" x14ac:dyDescent="0.3">
@@ -14933,7 +14933,7 @@
         <v>36.998809462187474</v>
       </c>
       <c r="M174" s="1">
-        <v>67.998809462187467</v>
+        <v>90.980738822413812</v>
       </c>
     </row>
     <row r="175" spans="1:13" x14ac:dyDescent="0.3">
@@ -14972,7 +14972,7 @@
         <v>30</v>
       </c>
       <c r="M175" s="1">
-        <v>72</v>
+        <v>67.881976943271326</v>
       </c>
     </row>
     <row r="176" spans="1:13" x14ac:dyDescent="0.3">
@@ -15011,7 +15011,7 @@
         <v>30</v>
       </c>
       <c r="M176" s="1">
-        <v>60</v>
+        <v>62.747119466343236</v>
       </c>
     </row>
     <row r="177" spans="1:13" x14ac:dyDescent="0.3">
@@ -15050,7 +15050,7 @@
         <v>30</v>
       </c>
       <c r="M177" s="1">
-        <v>60</v>
+        <v>60.954428202923481</v>
       </c>
     </row>
     <row r="178" spans="1:13" x14ac:dyDescent="0.3">
@@ -15089,7 +15089,7 @@
         <v>30</v>
       </c>
       <c r="M178" s="1">
-        <v>60</v>
+        <v>61.42275240034914</v>
       </c>
     </row>
     <row r="179" spans="1:13" x14ac:dyDescent="0.3">
@@ -15128,7 +15128,7 @@
         <v>30</v>
       </c>
       <c r="M179" s="1">
-        <v>60</v>
+        <v>71.55444401692958</v>
       </c>
     </row>
     <row r="180" spans="1:13" x14ac:dyDescent="0.3">
@@ -15167,7 +15167,7 @@
         <v>30</v>
       </c>
       <c r="M180" s="1">
-        <v>60</v>
+        <v>61.195840554592721</v>
       </c>
     </row>
     <row r="181" spans="1:13" x14ac:dyDescent="0.3">
@@ -15205,7 +15205,7 @@
         <v>30</v>
       </c>
       <c r="M181" s="1">
-        <v>60</v>
+        <v>72.088854247856602</v>
       </c>
     </row>
     <row r="182" spans="1:13" x14ac:dyDescent="0.3">
@@ -15244,7 +15244,7 @@
         <v>30</v>
       </c>
       <c r="M182" s="1">
-        <v>60</v>
+        <v>66.400404448938303</v>
       </c>
     </row>
     <row r="183" spans="1:13" x14ac:dyDescent="0.3">
@@ -15283,7 +15283,7 @@
         <v>30</v>
       </c>
       <c r="M183" s="1">
-        <v>60</v>
+        <v>85.045871559633028</v>
       </c>
     </row>
     <row r="184" spans="1:13" x14ac:dyDescent="0.3">
@@ -15323,7 +15323,7 @@
         <v>41.983590144318825</v>
       </c>
       <c r="M184" s="1">
-        <v>71.983590144318825</v>
+        <v>72.649617935406511</v>
       </c>
     </row>
     <row r="185" spans="1:13" x14ac:dyDescent="0.3">
@@ -15363,7 +15363,7 @@
         <v>38.384520884520882</v>
       </c>
       <c r="M185" s="1">
-        <v>75.384520884520882</v>
+        <v>97.420270310562216</v>
       </c>
     </row>
     <row r="186" spans="1:13" x14ac:dyDescent="0.3">
@@ -15402,7 +15402,7 @@
         <v>30</v>
       </c>
       <c r="M186" s="1">
-        <v>72</v>
+        <v>76.035805626598489</v>
       </c>
     </row>
     <row r="187" spans="1:13" x14ac:dyDescent="0.3">
@@ -15442,7 +15442,7 @@
         <v>33.851040525739315</v>
       </c>
       <c r="M187" s="1">
-        <v>72.851040525739307</v>
+        <v>91.451040525739302</v>
       </c>
     </row>
     <row r="188" spans="1:13" x14ac:dyDescent="0.3">
@@ -15481,7 +15481,7 @@
         <v>45</v>
       </c>
       <c r="M188" s="1">
-        <v>75</v>
+        <v>90.529277855065146</v>
       </c>
     </row>
     <row r="189" spans="1:13" x14ac:dyDescent="0.3">
@@ -15520,7 +15520,7 @@
         <v>30</v>
       </c>
       <c r="M189" s="1">
-        <v>357</v>
+        <v>749.99999999999989</v>
       </c>
     </row>
     <row r="190" spans="1:13" x14ac:dyDescent="0.3">
@@ -15560,7 +15560,7 @@
         <v>33.069932832872382</v>
       </c>
       <c r="M190" s="1">
-        <v>175.06993283287238</v>
+        <v>236.45976334134696</v>
       </c>
     </row>
     <row r="191" spans="1:13" x14ac:dyDescent="0.3">
@@ -15599,7 +15599,7 @@
         <v>45</v>
       </c>
       <c r="M191" s="1">
-        <v>75</v>
+        <v>75.372911862309465</v>
       </c>
     </row>
     <row r="192" spans="1:13" x14ac:dyDescent="0.3">
@@ -15639,7 +15639,7 @@
         <v>38.912523256239652</v>
       </c>
       <c r="M192" s="1">
-        <v>68.912523256239652</v>
+        <v>69.266414297036476</v>
       </c>
     </row>
     <row r="193" spans="1:13" x14ac:dyDescent="0.3">
@@ -15679,7 +15679,7 @@
         <v>40.416254708834451</v>
       </c>
       <c r="M193" s="1">
-        <v>70.416254708834458</v>
+        <v>75.234436527016257</v>
       </c>
     </row>
     <row r="194" spans="1:13" x14ac:dyDescent="0.3">
@@ -15721,7 +15721,7 @@
         <v>30</v>
       </c>
       <c r="M194" s="1">
-        <v>60</v>
+        <v>60.014130946773435</v>
       </c>
     </row>
     <row r="195" spans="1:13" x14ac:dyDescent="0.3">
@@ -15764,7 +15764,7 @@
         <v>36.997411561691109</v>
       </c>
       <c r="M195" s="1">
-        <v>286.99741156169114</v>
+        <v>317.52191715068511</v>
       </c>
     </row>
     <row r="196" spans="1:13" x14ac:dyDescent="0.3">
@@ -15803,7 +15803,7 @@
         <v>34.552473753366208</v>
       </c>
       <c r="M196" s="1">
-        <v>64.552473753366201</v>
+        <v>67.980614273155368</v>
       </c>
     </row>
     <row r="197" spans="1:13" x14ac:dyDescent="0.3">
@@ -15842,7 +15842,7 @@
         <v>38.010057732108493</v>
       </c>
       <c r="M197" s="1">
-        <v>68.010057732108493</v>
+        <v>70.919232819095939</v>
       </c>
     </row>
     <row r="198" spans="1:13" x14ac:dyDescent="0.3">
@@ -15880,7 +15880,7 @@
         <v>30</v>
       </c>
       <c r="M198" s="1">
-        <v>60</v>
+        <v>64.98698088332236</v>
       </c>
     </row>
     <row r="199" spans="1:13" x14ac:dyDescent="0.3">
@@ -15922,7 +15922,7 @@
         <v>30</v>
       </c>
       <c r="M199" s="1">
-        <v>60</v>
+        <v>60.000676696817266</v>
       </c>
     </row>
     <row r="200" spans="1:13" x14ac:dyDescent="0.3">
@@ -16004,7 +16004,7 @@
         <v>37.807017770798367</v>
       </c>
       <c r="M201" s="1">
-        <v>67.807017770798367</v>
+        <v>68.441164778341701</v>
       </c>
     </row>
     <row r="202" spans="1:13" x14ac:dyDescent="0.3">
@@ -16044,7 +16044,7 @@
         <v>34.234285214246121</v>
       </c>
       <c r="M202" s="1">
-        <v>64.234285214246114</v>
+        <v>64.597282440380582</v>
       </c>
     </row>
     <row r="203" spans="1:13" x14ac:dyDescent="0.3">
@@ -16084,7 +16084,7 @@
         <v>35.012439593075506</v>
       </c>
       <c r="M203" s="1">
-        <v>72.012439593075499</v>
+        <v>68.82485703032782</v>
       </c>
     </row>
     <row r="204" spans="1:13" x14ac:dyDescent="0.3">
@@ -16126,7 +16126,7 @@
         <v>30</v>
       </c>
       <c r="M204" s="1">
-        <v>60</v>
+        <v>100.39554317548746</v>
       </c>
     </row>
     <row r="205" spans="1:13" x14ac:dyDescent="0.3">
@@ -16166,7 +16166,7 @@
         <v>36.789508928571422</v>
       </c>
       <c r="M205" s="1">
-        <v>70.789508928571422</v>
+        <v>68.878985288510421</v>
       </c>
     </row>
     <row r="206" spans="1:13" x14ac:dyDescent="0.3">
@@ -16206,7 +16206,7 @@
         <v>40.452894307265659</v>
       </c>
       <c r="M206" s="1">
-        <v>70.452894307265666</v>
+        <v>71.085482318307072</v>
       </c>
     </row>
     <row r="207" spans="1:13" x14ac:dyDescent="0.3">
@@ -16246,7 +16246,7 @@
         <v>40.118428436252941</v>
       </c>
       <c r="M207" s="1">
-        <v>70.118428436252941</v>
+        <v>70.301027637471222</v>
       </c>
     </row>
     <row r="208" spans="1:13" x14ac:dyDescent="0.3">
@@ -16286,7 +16286,7 @@
         <v>32.356176234319975</v>
       </c>
       <c r="M208" s="1">
-        <v>62.356176234319975</v>
+        <v>80.664602362007273</v>
       </c>
     </row>
     <row r="209" spans="1:13" x14ac:dyDescent="0.3">
@@ -16329,7 +16329,7 @@
         <v>36.925824629241042</v>
       </c>
       <c r="M209" s="1">
-        <v>66.925824629241049</v>
+        <v>71.720484605097312</v>
       </c>
     </row>
     <row r="210" spans="1:13" x14ac:dyDescent="0.3">
@@ -16369,7 +16369,7 @@
         <v>37.194321477637004</v>
       </c>
       <c r="M210" s="1">
-        <v>67.194321477637004</v>
+        <v>87.679720921842801</v>
       </c>
     </row>
     <row r="211" spans="1:13" x14ac:dyDescent="0.3">
@@ -16409,7 +16409,7 @@
         <v>38.555670783444896</v>
       </c>
       <c r="M211" s="1">
-        <v>68.555670783444896</v>
+        <v>74.164464188391179</v>
       </c>
     </row>
     <row r="212" spans="1:13" x14ac:dyDescent="0.3">
@@ -16448,7 +16448,7 @@
         <v>32.805430637963163</v>
       </c>
       <c r="M212" s="1">
-        <v>62.805430637963163</v>
+        <v>66.570206110928666</v>
       </c>
     </row>
     <row r="213" spans="1:13" x14ac:dyDescent="0.3">
@@ -16487,7 +16487,7 @@
         <v>33.928054943892128</v>
       </c>
       <c r="M213" s="1">
-        <v>63.928054943892128</v>
+        <v>66.6217123948893</v>
       </c>
     </row>
     <row r="214" spans="1:13" x14ac:dyDescent="0.3">
@@ -16526,7 +16526,7 @@
         <v>45</v>
       </c>
       <c r="M214" s="1">
-        <v>75</v>
+        <v>78.037337435323735</v>
       </c>
     </row>
     <row r="215" spans="1:13" x14ac:dyDescent="0.3">
@@ -16565,7 +16565,7 @@
         <v>45</v>
       </c>
       <c r="M215" s="1">
-        <v>75</v>
+        <v>78.923622987093665</v>
       </c>
     </row>
     <row r="216" spans="1:13" x14ac:dyDescent="0.3">
@@ -16605,7 +16605,7 @@
         <v>36.985219264956086</v>
       </c>
       <c r="M216" s="1">
-        <v>66.985219264956086</v>
+        <v>67.709966089110353</v>
       </c>
     </row>
     <row r="217" spans="1:13" x14ac:dyDescent="0.3">
@@ -16645,7 +16645,7 @@
         <v>36.383472210291217</v>
       </c>
       <c r="M217" s="1">
-        <v>66.383472210291217</v>
+        <v>66.417135311620243</v>
       </c>
     </row>
     <row r="218" spans="1:13" x14ac:dyDescent="0.3">
@@ -16685,7 +16685,7 @@
         <v>39.786536430109877</v>
       </c>
       <c r="M218" s="1">
-        <v>69.786536430109877</v>
+        <v>79.401739419977233</v>
       </c>
     </row>
     <row r="219" spans="1:13" x14ac:dyDescent="0.3">
@@ -16725,7 +16725,7 @@
         <v>39.831619849429295</v>
       </c>
       <c r="M219" s="1">
-        <v>69.831619849429302</v>
+        <v>74.318302114886535</v>
       </c>
     </row>
     <row r="220" spans="1:13" x14ac:dyDescent="0.3">
@@ -16767,7 +16767,7 @@
         <v>30</v>
       </c>
       <c r="M220" s="1">
-        <v>60</v>
+        <v>60.001898553934758</v>
       </c>
     </row>
     <row r="221" spans="1:13" x14ac:dyDescent="0.3">
@@ -16885,7 +16885,7 @@
         <v>37.578570265429086</v>
       </c>
       <c r="M223" s="1">
-        <v>67.578570265429079</v>
+        <v>77.906191601403293</v>
       </c>
     </row>
     <row r="224" spans="1:13" x14ac:dyDescent="0.3">
@@ -16925,7 +16925,7 @@
         <v>37.769244852617369</v>
       </c>
       <c r="M224" s="1">
-        <v>67.769244852617362</v>
+        <v>82.334491495422625</v>
       </c>
     </row>
     <row r="225" spans="1:13" x14ac:dyDescent="0.3">
@@ -16963,7 +16963,7 @@
         <v>30</v>
       </c>
       <c r="M225" s="1">
-        <v>60</v>
+        <v>60.167336878972627</v>
       </c>
     </row>
     <row r="226" spans="1:13" x14ac:dyDescent="0.3">
@@ -17002,7 +17002,7 @@
         <v>30</v>
       </c>
       <c r="M226" s="1">
-        <v>60</v>
+        <v>67.338609943111535</v>
       </c>
     </row>
     <row r="227" spans="1:13" x14ac:dyDescent="0.3">
@@ -17040,7 +17040,7 @@
         <v>30</v>
       </c>
       <c r="M227" s="1">
-        <v>60</v>
+        <v>60.149160969546301</v>
       </c>
     </row>
     <row r="228" spans="1:13" x14ac:dyDescent="0.3">
@@ -17079,7 +17079,7 @@
         <v>30</v>
       </c>
       <c r="M228" s="1">
-        <v>60</v>
+        <v>60.218960571085461</v>
       </c>
     </row>
     <row r="229" spans="1:13" x14ac:dyDescent="0.3">
@@ -17119,7 +17119,7 @@
         <v>42.156229188303065</v>
       </c>
       <c r="M229" s="1">
-        <v>72.156229188303058</v>
+        <v>72.230825602574569</v>
       </c>
     </row>
     <row r="230" spans="1:13" x14ac:dyDescent="0.3">
@@ -17159,7 +17159,7 @@
         <v>36.104647898745554</v>
       </c>
       <c r="M230" s="1">
-        <v>66.104647898745554</v>
+        <v>66.177894255151244</v>
       </c>
     </row>
     <row r="231" spans="1:13" x14ac:dyDescent="0.3">
@@ -17199,7 +17199,7 @@
         <v>36.529550827423165</v>
       </c>
       <c r="M231" s="1">
-        <v>66.529550827423165</v>
+        <v>69.224863327423151</v>
       </c>
     </row>
     <row r="232" spans="1:13" x14ac:dyDescent="0.3">
@@ -17238,7 +17238,7 @@
         <v>40.238764044943821</v>
       </c>
       <c r="M232" s="1">
-        <v>70.238764044943821</v>
+        <v>70.875937216599752</v>
       </c>
     </row>
     <row r="233" spans="1:13" x14ac:dyDescent="0.3">
@@ -17276,7 +17276,7 @@
         <v>45</v>
       </c>
       <c r="M233" s="1">
-        <v>75</v>
+        <v>79.358381502890168</v>
       </c>
     </row>
     <row r="234" spans="1:13" x14ac:dyDescent="0.3">
@@ -17314,7 +17314,7 @@
         <v>30</v>
       </c>
       <c r="M234" s="1">
-        <v>60</v>
+        <v>60.043032075628958</v>
       </c>
     </row>
     <row r="235" spans="1:13" x14ac:dyDescent="0.3">
@@ -17352,7 +17352,7 @@
         <v>30</v>
       </c>
       <c r="M235" s="1">
-        <v>60</v>
+        <v>60.094814727296885</v>
       </c>
     </row>
     <row r="236" spans="1:13" x14ac:dyDescent="0.3">
@@ -17391,7 +17391,7 @@
         <v>30</v>
       </c>
       <c r="M236" s="1">
-        <v>139</v>
+        <v>236.07476635514016</v>
       </c>
     </row>
     <row r="237" spans="1:13" x14ac:dyDescent="0.3">
@@ -17430,7 +17430,7 @@
         <v>30</v>
       </c>
       <c r="M237" s="1">
-        <v>122</v>
+        <v>220.90909090909091</v>
       </c>
     </row>
     <row r="238" spans="1:13" x14ac:dyDescent="0.3">
@@ -17469,7 +17469,7 @@
         <v>30</v>
       </c>
       <c r="M238" s="1">
-        <v>153</v>
+        <v>316.73602080624187</v>
       </c>
     </row>
     <row r="239" spans="1:13" x14ac:dyDescent="0.3">
@@ -17507,7 +17507,7 @@
         <v>30</v>
       </c>
       <c r="M239" s="1">
-        <v>192</v>
+        <v>332.46913580246905</v>
       </c>
     </row>
     <row r="240" spans="1:13" x14ac:dyDescent="0.3">
@@ -17550,7 +17550,7 @@
         <v>38.112747366415334</v>
       </c>
       <c r="M240" s="1">
-        <v>68.112747366415334</v>
+        <v>69.287469450228329</v>
       </c>
     </row>
     <row r="241" spans="1:13" x14ac:dyDescent="0.3">
@@ -17590,7 +17590,7 @@
         <v>34.232722207434712</v>
       </c>
       <c r="M241" s="1">
-        <v>64.232722207434705</v>
+        <v>66.98351279868541</v>
       </c>
     </row>
     <row r="242" spans="1:13" x14ac:dyDescent="0.3">
@@ -17630,7 +17630,7 @@
         <v>32.530783728300385</v>
       </c>
       <c r="M242" s="1">
-        <v>62.530783728300385</v>
+        <v>69.91122157119743</v>
       </c>
     </row>
     <row r="243" spans="1:13" x14ac:dyDescent="0.3">
@@ -17670,7 +17670,7 @@
         <v>41.559981403745709</v>
       </c>
       <c r="M243" s="1">
-        <v>71.559981403745709</v>
+        <v>73.604267848234528</v>
       </c>
     </row>
     <row r="244" spans="1:13" x14ac:dyDescent="0.3">
@@ -17710,7 +17710,7 @@
         <v>33.197862218828924</v>
       </c>
       <c r="M244" s="1">
-        <v>63.197862218828924</v>
+        <v>65.057516283922979</v>
       </c>
     </row>
     <row r="245" spans="1:13" x14ac:dyDescent="0.3">
@@ -17750,7 +17750,7 @@
         <v>31.401592816914903</v>
       </c>
       <c r="M245" s="1">
-        <v>61.401592816914899</v>
+        <v>62.847822303404271</v>
       </c>
     </row>
     <row r="246" spans="1:13" x14ac:dyDescent="0.3">
@@ -17829,7 +17829,7 @@
         <v>32.606880601738794</v>
       </c>
       <c r="M247" s="1">
-        <v>62.606880601738794</v>
+        <v>64.736442092980553</v>
       </c>
     </row>
     <row r="248" spans="1:13" x14ac:dyDescent="0.3">
@@ -17871,7 +17871,7 @@
         <v>30</v>
       </c>
       <c r="M248" s="1">
-        <v>60</v>
+        <v>60.008941877794328</v>
       </c>
     </row>
     <row r="249" spans="1:13" x14ac:dyDescent="0.3">
@@ -17911,7 +17911,7 @@
         <v>32.068538950183886</v>
       </c>
       <c r="M249" s="1">
-        <v>62.068538950183886</v>
+        <v>62.755141076714281</v>
       </c>
     </row>
     <row r="250" spans="1:13" x14ac:dyDescent="0.3">
@@ -17951,7 +17951,7 @@
         <v>34.526055126183437</v>
       </c>
       <c r="M250" s="1">
-        <v>64.526055126183437</v>
+        <v>65.086567820292373</v>
       </c>
     </row>
     <row r="251" spans="1:13" x14ac:dyDescent="0.3">
@@ -17991,7 +17991,7 @@
         <v>32.888475480764122</v>
       </c>
       <c r="M251" s="1">
-        <v>62.888475480764122</v>
+        <v>63.840709687235602</v>
       </c>
     </row>
     <row r="252" spans="1:13" x14ac:dyDescent="0.3">
@@ -18031,7 +18031,7 @@
         <v>34.088384419094083</v>
       </c>
       <c r="M252" s="1">
-        <v>64.088384419094083</v>
+        <v>64.157473047752788</v>
       </c>
     </row>
     <row r="253" spans="1:13" x14ac:dyDescent="0.3">
@@ -18070,7 +18070,7 @@
         <v>32.519634515810701</v>
       </c>
       <c r="M253" s="1">
-        <v>62.519634515810701</v>
+        <v>62.585364443865238</v>
       </c>
     </row>
     <row r="254" spans="1:13" x14ac:dyDescent="0.3">
@@ -18110,7 +18110,7 @@
         <v>31.90648737653644</v>
       </c>
       <c r="M254" s="1">
-        <v>61.90648737653644</v>
+        <v>62.426807225556701</v>
       </c>
     </row>
     <row r="255" spans="1:13" x14ac:dyDescent="0.3">
@@ -18149,7 +18149,7 @@
         <v>30</v>
       </c>
       <c r="M255" s="1">
-        <v>60</v>
+        <v>61.078765825183837</v>
       </c>
     </row>
     <row r="256" spans="1:13" x14ac:dyDescent="0.3">
@@ -18187,7 +18187,7 @@
         <v>30</v>
       </c>
       <c r="M256" s="1">
-        <v>60</v>
+        <v>60.995428954110437</v>
       </c>
     </row>
     <row r="257" spans="1:13" x14ac:dyDescent="0.3">
@@ -18226,7 +18226,7 @@
         <v>30</v>
       </c>
       <c r="M257" s="1">
-        <v>60</v>
+        <v>63.740163217720777</v>
       </c>
     </row>
     <row r="258" spans="1:13" x14ac:dyDescent="0.3">
@@ -18265,7 +18265,7 @@
         <v>30</v>
       </c>
       <c r="M258" s="1">
-        <v>60</v>
+        <v>62.392049039935102</v>
       </c>
     </row>
     <row r="259" spans="1:13" x14ac:dyDescent="0.3">
@@ -18305,7 +18305,7 @@
         <v>30.121370056293813</v>
       </c>
       <c r="M259" s="1">
-        <v>60.121370056293813</v>
+        <v>60.626895617285875</v>
       </c>
     </row>
     <row r="260" spans="1:13" x14ac:dyDescent="0.3">
@@ -18344,7 +18344,7 @@
         <v>30</v>
       </c>
       <c r="M260" s="1">
-        <v>60</v>
+        <v>64.508648784156435</v>
       </c>
     </row>
     <row r="261" spans="1:13" x14ac:dyDescent="0.3">
@@ -18384,7 +18384,7 @@
         <v>31.984290623465888</v>
       </c>
       <c r="M261" s="1">
-        <v>61.984290623465888</v>
+        <v>63.105012741086895</v>
       </c>
     </row>
     <row r="262" spans="1:13" x14ac:dyDescent="0.3">
@@ -18423,7 +18423,7 @@
         <v>30</v>
       </c>
       <c r="M262" s="1">
-        <v>60</v>
+        <v>65.744904458598739</v>
       </c>
     </row>
     <row r="263" spans="1:13" x14ac:dyDescent="0.3">
@@ -18541,7 +18541,7 @@
         <v>30.148200423429785</v>
       </c>
       <c r="M265" s="1">
-        <v>60.148200423429785</v>
+        <v>60.15143353044563</v>
       </c>
     </row>
     <row r="266" spans="1:13" x14ac:dyDescent="0.3">
@@ -18581,7 +18581,7 @@
         <v>38.991974905084362</v>
       </c>
       <c r="M266" s="1">
-        <v>68.991974905084362</v>
+        <v>69.872671553019586</v>
       </c>
     </row>
     <row r="267" spans="1:13" x14ac:dyDescent="0.3">
@@ -18621,7 +18621,7 @@
         <v>40.153295635271242</v>
       </c>
       <c r="M267" s="1">
-        <v>70.153295635271235</v>
+        <v>83.532687660537732</v>
       </c>
     </row>
     <row r="268" spans="1:13" x14ac:dyDescent="0.3">
@@ -18660,7 +18660,7 @@
         <v>30</v>
       </c>
       <c r="M268" s="1">
-        <v>60</v>
+        <v>60.00464991756963</v>
       </c>
     </row>
     <row r="269" spans="1:13" x14ac:dyDescent="0.3">
@@ -18700,7 +18700,7 @@
         <v>44.123663612223517</v>
       </c>
       <c r="M269" s="1">
-        <v>74.12366361222351</v>
+        <v>74.928917985213431</v>
       </c>
     </row>
     <row r="270" spans="1:13" x14ac:dyDescent="0.3">
@@ -18740,7 +18740,7 @@
         <v>43.794670102393709</v>
       </c>
       <c r="M270" s="1">
-        <v>77.794670102393709</v>
+        <v>76.116542242542749</v>
       </c>
     </row>
     <row r="271" spans="1:13" x14ac:dyDescent="0.3">
@@ -18780,7 +18780,7 @@
         <v>42.779059040590411</v>
       </c>
       <c r="M271" s="1">
-        <v>72.779059040590411</v>
+        <v>75.903863009681686</v>
       </c>
     </row>
     <row r="272" spans="1:13" x14ac:dyDescent="0.3">
@@ -18859,7 +18859,7 @@
         <v>35.046253215830099</v>
       </c>
       <c r="M273" s="1">
-        <v>65.046253215830092</v>
+        <v>65.059746550122952</v>
       </c>
     </row>
     <row r="274" spans="1:13" x14ac:dyDescent="0.3">
@@ -18898,7 +18898,7 @@
         <v>30</v>
       </c>
       <c r="M274" s="1">
-        <v>60</v>
+        <v>60.168944994857284</v>
       </c>
     </row>
     <row r="275" spans="1:13" x14ac:dyDescent="0.3">
@@ -18937,7 +18937,7 @@
         <v>30</v>
       </c>
       <c r="M275" s="1">
-        <v>60</v>
+        <v>60.255899973236524</v>
       </c>
     </row>
     <row r="276" spans="1:13" x14ac:dyDescent="0.3">
@@ -18977,7 +18977,7 @@
         <v>31.320204382451443</v>
       </c>
       <c r="M276" s="1">
-        <v>61.320204382451443</v>
+        <v>62.557584449223057</v>
       </c>
     </row>
     <row r="277" spans="1:13" x14ac:dyDescent="0.3">
@@ -19017,7 +19017,7 @@
         <v>30.178694134520981</v>
       </c>
       <c r="M277" s="1">
-        <v>60.178694134520981</v>
+        <v>60.379455517509122</v>
       </c>
     </row>
     <row r="278" spans="1:13" x14ac:dyDescent="0.3">
@@ -19057,7 +19057,7 @@
         <v>30.732176088349256</v>
       </c>
       <c r="M278" s="1">
-        <v>60.732176088349256</v>
+        <v>60.827177351147228</v>
       </c>
     </row>
     <row r="279" spans="1:13" x14ac:dyDescent="0.3">
@@ -19097,7 +19097,7 @@
         <v>32.194555288804473</v>
       </c>
       <c r="M279" s="1">
-        <v>62.194555288804473</v>
+        <v>62.286058040989452</v>
       </c>
     </row>
     <row r="280" spans="1:13" x14ac:dyDescent="0.3">
@@ -19137,7 +19137,7 @@
         <v>37.711722159489732</v>
       </c>
       <c r="M280" s="1">
-        <v>67.711722159489739</v>
+        <v>67.936967417828498</v>
       </c>
     </row>
     <row r="281" spans="1:13" x14ac:dyDescent="0.3">
@@ -19177,7 +19177,7 @@
         <v>34.095597686375321</v>
       </c>
       <c r="M281" s="1">
-        <v>64.095597686375328</v>
+        <v>67.047126826594592</v>
       </c>
     </row>
     <row r="282" spans="1:13" x14ac:dyDescent="0.3">
@@ -19220,7 +19220,7 @@
         <v>32.606911644022979</v>
       </c>
       <c r="M282" s="1">
-        <v>62.606911644022979</v>
+        <v>62.789650676258965</v>
       </c>
     </row>
     <row r="283" spans="1:13" x14ac:dyDescent="0.3">
@@ -19263,7 +19263,7 @@
         <v>35.416583416583428</v>
       </c>
       <c r="M283" s="1">
-        <v>65.416583416583421</v>
+        <v>66.563876786021737</v>
       </c>
     </row>
     <row r="284" spans="1:13" x14ac:dyDescent="0.3">
@@ -19302,7 +19302,7 @@
         <v>30</v>
       </c>
       <c r="M284" s="1">
-        <v>60</v>
+        <v>60.04989606545486</v>
       </c>
     </row>
     <row r="285" spans="1:13" x14ac:dyDescent="0.3">
@@ -19342,7 +19342,7 @@
         <v>30.004777510497963</v>
       </c>
       <c r="M285" s="1">
-        <v>60.004777510497959</v>
+        <v>60.451869306330906</v>
       </c>
     </row>
     <row r="286" spans="1:13" x14ac:dyDescent="0.3">
@@ -19382,7 +19382,7 @@
         <v>34.256622702486872</v>
       </c>
       <c r="M286" s="1">
-        <v>64.256622702486879</v>
+        <v>64.739862250938572</v>
       </c>
     </row>
     <row r="287" spans="1:13" x14ac:dyDescent="0.3">
@@ -19422,7 +19422,7 @@
         <v>32.999849480708448</v>
       </c>
       <c r="M287" s="1">
-        <v>62.999849480708448</v>
+        <v>63.615589457609943</v>
       </c>
     </row>
     <row r="288" spans="1:13" x14ac:dyDescent="0.3">
@@ -19462,7 +19462,7 @@
         <v>32.756308559741292</v>
       </c>
       <c r="M288" s="1">
-        <v>62.756308559741292</v>
+        <v>62.899777391415654</v>
       </c>
     </row>
     <row r="289" spans="1:13" x14ac:dyDescent="0.3">
@@ -19501,7 +19501,7 @@
         <v>30</v>
       </c>
       <c r="M289" s="1">
-        <v>60</v>
+        <v>60.045955002393498</v>
       </c>
     </row>
     <row r="290" spans="1:13" x14ac:dyDescent="0.3">
@@ -19541,7 +19541,7 @@
         <v>30.730545966482168</v>
       </c>
       <c r="M290" s="1">
-        <v>60.730545966482168</v>
+        <v>60.795946109877526</v>
       </c>
     </row>
     <row r="291" spans="1:13" x14ac:dyDescent="0.3">
@@ -19580,7 +19580,7 @@
         <v>30</v>
       </c>
       <c r="M291" s="1">
-        <v>60</v>
+        <v>63.228371705252357</v>
       </c>
     </row>
     <row r="292" spans="1:13" x14ac:dyDescent="0.3">
@@ -19701,7 +19701,7 @@
         <v>31.288523285126701</v>
       </c>
       <c r="M294" s="1">
-        <v>61.288523285126701</v>
+        <v>61.288652026678037</v>
       </c>
     </row>
     <row r="295" spans="1:13" x14ac:dyDescent="0.3">
@@ -19819,7 +19819,7 @@
         <v>35.688572163244324</v>
       </c>
       <c r="M297" s="1">
-        <v>65.688572163244316</v>
+        <v>74.30941184129523</v>
       </c>
     </row>
     <row r="298" spans="1:13" x14ac:dyDescent="0.3">
@@ -19900,7 +19900,7 @@
         <v>30</v>
       </c>
       <c r="M299" s="1">
-        <v>60</v>
+        <v>61.504224383182724</v>
       </c>
     </row>
     <row r="300" spans="1:13" x14ac:dyDescent="0.3">
@@ -19943,7 +19943,7 @@
         <v>39.246466737979688</v>
       </c>
       <c r="M300" s="1">
-        <v>69.246466737979688</v>
+        <v>69.368115601431725</v>
       </c>
     </row>
     <row r="301" spans="1:13" x14ac:dyDescent="0.3">
@@ -19986,7 +19986,7 @@
         <v>41.871869016012951</v>
       </c>
       <c r="M301" s="1">
-        <v>71.871869016012951</v>
+        <v>71.88586882934878</v>
       </c>
     </row>
     <row r="302" spans="1:13" x14ac:dyDescent="0.3">
@@ -20028,7 +20028,7 @@
         <v>30</v>
       </c>
       <c r="M302" s="1">
-        <v>60</v>
+        <v>61.140125903474001</v>
       </c>
     </row>
     <row r="303" spans="1:13" x14ac:dyDescent="0.3">
@@ -20068,7 +20068,7 @@
         <v>41.359546743472173</v>
       </c>
       <c r="M303" s="1">
-        <v>71.35954674347218</v>
+        <v>71.612308148292115</v>
       </c>
     </row>
     <row r="304" spans="1:13" x14ac:dyDescent="0.3">
@@ -20108,7 +20108,7 @@
         <v>40.688336185353585</v>
       </c>
       <c r="M304" s="1">
-        <v>70.688336185353592</v>
+        <v>71.702347109124645</v>
       </c>
     </row>
     <row r="305" spans="1:13" x14ac:dyDescent="0.3">
@@ -20148,7 +20148,7 @@
         <v>39.945649180147257</v>
       </c>
       <c r="M305" s="1">
-        <v>69.945649180147257</v>
+        <v>70.16027675486275</v>
       </c>
     </row>
     <row r="306" spans="1:13" x14ac:dyDescent="0.3">
@@ -20187,7 +20187,7 @@
         <v>45</v>
       </c>
       <c r="M306" s="1">
-        <v>75</v>
+        <v>75.142518242695417</v>
       </c>
     </row>
     <row r="307" spans="1:13" x14ac:dyDescent="0.3">
@@ -20227,7 +20227,7 @@
         <v>32.886407766990295</v>
       </c>
       <c r="M307" s="1">
-        <v>62.886407766990295</v>
+        <v>63.229805776409741</v>
       </c>
     </row>
     <row r="308" spans="1:13" x14ac:dyDescent="0.3">
@@ -20267,7 +20267,7 @@
         <v>33.523212222667581</v>
       </c>
       <c r="M308" s="1">
-        <v>63.523212222667581</v>
+        <v>64.164390667222605</v>
       </c>
     </row>
     <row r="309" spans="1:13" x14ac:dyDescent="0.3">
@@ -20307,7 +20307,7 @@
         <v>32.955304804822653</v>
       </c>
       <c r="M309" s="1">
-        <v>62.955304804822653</v>
+        <v>63.43335450317506</v>
       </c>
     </row>
     <row r="310" spans="1:13" x14ac:dyDescent="0.3">
@@ -20347,7 +20347,7 @@
         <v>33.805070422535202</v>
       </c>
       <c r="M310" s="1">
-        <v>63.805070422535202</v>
+        <v>64.131531964797333</v>
       </c>
     </row>
     <row r="311" spans="1:13" x14ac:dyDescent="0.3">
@@ -20387,7 +20387,7 @@
         <v>36.464383951436965</v>
       </c>
       <c r="M311" s="1">
-        <v>66.464383951436957</v>
+        <v>67.060995510902416</v>
       </c>
     </row>
     <row r="312" spans="1:13" x14ac:dyDescent="0.3">
@@ -20427,7 +20427,7 @@
         <v>35.560934839808084</v>
       </c>
       <c r="M312" s="1">
-        <v>65.560934839808084</v>
+        <v>65.974334366556093</v>
       </c>
     </row>
     <row r="313" spans="1:13" x14ac:dyDescent="0.3">
@@ -20467,7 +20467,7 @@
         <v>34.364033914931518</v>
       </c>
       <c r="M313" s="1">
-        <v>64.364033914931525</v>
+        <v>66.042014145966405</v>
       </c>
     </row>
     <row r="314" spans="1:13" x14ac:dyDescent="0.3">
@@ -20507,7 +20507,7 @@
         <v>34.56156716417911</v>
       </c>
       <c r="M314" s="1">
-        <v>64.56156716417911</v>
+        <v>64.753744680730478</v>
       </c>
     </row>
     <row r="315" spans="1:13" x14ac:dyDescent="0.3">
@@ -20549,7 +20549,7 @@
         <v>30</v>
       </c>
       <c r="M315" s="1">
-        <v>60</v>
+        <v>64.583359736391856</v>
       </c>
     </row>
     <row r="316" spans="1:13" x14ac:dyDescent="0.3">
@@ -20589,7 +20589,7 @@
         <v>39.034266371050762</v>
       </c>
       <c r="M316" s="1">
-        <v>69.034266371050762</v>
+        <v>70.375083994435627</v>
       </c>
     </row>
     <row r="317" spans="1:13" x14ac:dyDescent="0.3">
@@ -20629,7 +20629,7 @@
         <v>33.353197040151279</v>
       </c>
       <c r="M317" s="1">
-        <v>63.353197040151279</v>
+        <v>66.516438219167384</v>
       </c>
     </row>
     <row r="318" spans="1:13" x14ac:dyDescent="0.3">
@@ -20669,7 +20669,7 @@
         <v>31.915188371613898</v>
       </c>
       <c r="M318" s="1">
-        <v>61.915188371613894</v>
+        <v>65.322032134745925</v>
       </c>
     </row>
     <row r="319" spans="1:13" x14ac:dyDescent="0.3">
@@ -20709,7 +20709,7 @@
         <v>38.066447811627832</v>
       </c>
       <c r="M319" s="1">
-        <v>68.066447811627825</v>
+        <v>68.460478957966018</v>
       </c>
     </row>
     <row r="320" spans="1:13" x14ac:dyDescent="0.3">
@@ -20749,7 +20749,7 @@
         <v>38.403386496771709</v>
       </c>
       <c r="M320" s="1">
-        <v>68.403386496771702</v>
+        <v>73.617306660538347</v>
       </c>
     </row>
     <row r="321" spans="1:13" x14ac:dyDescent="0.3">
@@ -20828,7 +20828,7 @@
         <v>41.092516028810863</v>
       </c>
       <c r="M322" s="1">
-        <v>71.092516028810863</v>
+        <v>73.019188657052467</v>
       </c>
     </row>
     <row r="323" spans="1:13" x14ac:dyDescent="0.3">
@@ -20909,7 +20909,7 @@
         <v>30</v>
       </c>
       <c r="M324" s="1">
-        <v>60</v>
+        <v>83.60508601346298</v>
       </c>
     </row>
     <row r="325" spans="1:13" x14ac:dyDescent="0.3">
@@ -20949,7 +20949,7 @@
         <v>40.082029287731473</v>
       </c>
       <c r="M325" s="1">
-        <v>70.082029287731473</v>
+        <v>70.531318387257556</v>
       </c>
     </row>
     <row r="326" spans="1:13" x14ac:dyDescent="0.3">
@@ -20989,7 +20989,7 @@
         <v>41.306744331347453</v>
       </c>
       <c r="M326" s="1">
-        <v>71.30674433134746</v>
+        <v>71.569335769437515</v>
       </c>
     </row>
     <row r="327" spans="1:13" x14ac:dyDescent="0.3">
@@ -21031,7 +21031,7 @@
         <v>30</v>
       </c>
       <c r="M327" s="1">
-        <v>60</v>
+        <v>61.564625850340136</v>
       </c>
     </row>
     <row r="328" spans="1:13" x14ac:dyDescent="0.3">
@@ -21113,7 +21113,7 @@
         <v>40.879765379194495</v>
       </c>
       <c r="M329" s="1">
-        <v>71.879765379194495</v>
+        <v>71.792639732671759</v>
       </c>
     </row>
     <row r="330" spans="1:13" x14ac:dyDescent="0.3">
@@ -21156,7 +21156,7 @@
         <v>39.227536206504034</v>
       </c>
       <c r="M330" s="1">
-        <v>77.227536206504027</v>
+        <v>76.916109938266075</v>
       </c>
     </row>
     <row r="331" spans="1:13" x14ac:dyDescent="0.3">
@@ -21234,7 +21234,7 @@
         <v>30</v>
       </c>
       <c r="M332" s="1">
-        <v>60</v>
+        <v>65.410579345088166</v>
       </c>
     </row>
     <row r="333" spans="1:13" x14ac:dyDescent="0.3">
@@ -21273,7 +21273,7 @@
         <v>30</v>
       </c>
       <c r="M333" s="1">
-        <v>81</v>
+        <v>95.375302663438262</v>
       </c>
     </row>
     <row r="334" spans="1:13" x14ac:dyDescent="0.3">
@@ -21315,7 +21315,7 @@
         <v>30</v>
       </c>
       <c r="M334" s="1">
-        <v>312</v>
+        <v>334.72258064516126</v>
       </c>
     </row>
     <row r="335" spans="1:13" x14ac:dyDescent="0.3">
@@ -21357,7 +21357,7 @@
         <v>30</v>
       </c>
       <c r="M335" s="1">
-        <v>91</v>
+        <v>81.40833988985051</v>
       </c>
     </row>
     <row r="336" spans="1:13" x14ac:dyDescent="0.3">
@@ -21396,7 +21396,7 @@
         <v>30</v>
       </c>
       <c r="M336" s="1">
-        <v>90</v>
+        <v>96.735751295336783</v>
       </c>
     </row>
     <row r="337" spans="1:13" x14ac:dyDescent="0.3">
@@ -21436,7 +21436,7 @@
         <v>30.615835777126101</v>
       </c>
       <c r="M337" s="1">
-        <v>256.61583577712611</v>
+        <v>279.23462030751273</v>
       </c>
     </row>
     <row r="338" spans="1:13" x14ac:dyDescent="0.3">
@@ -21476,7 +21476,7 @@
         <v>30.848621138596279</v>
       </c>
       <c r="M338" s="1">
-        <v>70.848621138596286</v>
+        <v>70.307518120906366</v>
       </c>
     </row>
     <row r="339" spans="1:13" x14ac:dyDescent="0.3">
@@ -21515,7 +21515,7 @@
         <v>30</v>
       </c>
       <c r="M339" s="1">
-        <v>106</v>
+        <v>112.43928949400762</v>
       </c>
     </row>
     <row r="340" spans="1:13" x14ac:dyDescent="0.3">
@@ -21555,7 +21555,7 @@
         <v>35.926115956900965</v>
       </c>
       <c r="M340" s="1">
-        <v>151.92611595690096</v>
+        <v>154.81910488679023</v>
       </c>
     </row>
     <row r="341" spans="1:13" x14ac:dyDescent="0.3">
@@ -21597,7 +21597,7 @@
         <v>30</v>
       </c>
       <c r="M341" s="1">
-        <v>124</v>
+        <v>129.81818181818181</v>
       </c>
     </row>
     <row r="342" spans="1:13" x14ac:dyDescent="0.3">
@@ -21637,7 +21637,7 @@
         <v>35.744442368765171</v>
       </c>
       <c r="M342" s="1">
-        <v>176.74444236876516</v>
+        <v>181.83139889050429</v>
       </c>
     </row>
     <row r="343" spans="1:13" x14ac:dyDescent="0.3">
@@ -21679,7 +21679,7 @@
         <v>30</v>
       </c>
       <c r="M343" s="1">
-        <v>113</v>
+        <v>97.562326869806114</v>
       </c>
     </row>
     <row r="344" spans="1:13" x14ac:dyDescent="0.3">
@@ -21718,7 +21718,7 @@
         <v>30</v>
       </c>
       <c r="M344" s="1">
-        <v>165</v>
+        <v>167.84810126582278</v>
       </c>
     </row>
     <row r="345" spans="1:13" x14ac:dyDescent="0.3">
@@ -21757,7 +21757,7 @@
         <v>30</v>
       </c>
       <c r="M345" s="1">
-        <v>302</v>
+        <v>320.05875440658042</v>
       </c>
     </row>
     <row r="346" spans="1:13" x14ac:dyDescent="0.3">
@@ -21797,7 +21797,7 @@
         <v>31.95207941126133</v>
       </c>
       <c r="M346" s="1">
-        <v>61.95207941126133</v>
+        <v>90.956124605849112</v>
       </c>
     </row>
     <row r="347" spans="1:13" x14ac:dyDescent="0.3">
@@ -21836,7 +21836,7 @@
         <v>30</v>
       </c>
       <c r="M347" s="1">
-        <v>60</v>
+        <v>66.171143881456572</v>
       </c>
     </row>
     <row r="348" spans="1:13" x14ac:dyDescent="0.3">
@@ -21875,7 +21875,7 @@
         <v>32.753706938443145</v>
       </c>
       <c r="M348" s="1">
-        <v>62.753706938443145</v>
+        <v>64.024065244632069</v>
       </c>
     </row>
     <row r="349" spans="1:13" x14ac:dyDescent="0.3">
@@ -21917,7 +21917,7 @@
         <v>30</v>
       </c>
       <c r="M349" s="1">
-        <v>60</v>
+        <v>61.488443071425912</v>
       </c>
     </row>
     <row r="350" spans="1:13" x14ac:dyDescent="0.3">
@@ -21956,7 +21956,7 @@
         <v>30</v>
       </c>
       <c r="M350" s="1">
-        <v>109</v>
+        <v>109.13736861181587</v>
       </c>
     </row>
     <row r="351" spans="1:13" x14ac:dyDescent="0.3">
@@ -21995,7 +21995,7 @@
         <v>30</v>
       </c>
       <c r="M351" s="1">
-        <v>271</v>
+        <v>266.01426660722245</v>
       </c>
     </row>
     <row r="352" spans="1:13" x14ac:dyDescent="0.3">
@@ -22035,7 +22035,7 @@
         <v>35.138316656856979</v>
       </c>
       <c r="M352" s="1">
-        <v>65.138316656856972</v>
+        <v>84.072585961260302</v>
       </c>
     </row>
     <row r="353" spans="1:13" x14ac:dyDescent="0.3">
@@ -22074,7 +22074,7 @@
         <v>30</v>
       </c>
       <c r="M353" s="1">
-        <v>141</v>
+        <v>145.33980582524271</v>
       </c>
     </row>
     <row r="354" spans="1:13" x14ac:dyDescent="0.3">
@@ -22113,7 +22113,7 @@
         <v>30</v>
       </c>
       <c r="M354" s="1">
-        <v>234</v>
+        <v>232.3512123438648</v>
       </c>
     </row>
     <row r="355" spans="1:13" x14ac:dyDescent="0.3">
@@ -22155,7 +22155,7 @@
         <v>30</v>
       </c>
       <c r="M355" s="1">
-        <v>134</v>
+        <v>119.99999999999999</v>
       </c>
     </row>
     <row r="356" spans="1:13" x14ac:dyDescent="0.3">
@@ -22194,7 +22194,7 @@
         <v>30</v>
       </c>
       <c r="M356" s="1">
-        <v>130</v>
+        <v>134.45803224013343</v>
       </c>
     </row>
     <row r="357" spans="1:13" x14ac:dyDescent="0.3">
@@ -22233,7 +22233,7 @@
         <v>30</v>
       </c>
       <c r="M357" s="1">
-        <v>250</v>
+        <v>253.86473429951693</v>
       </c>
     </row>
     <row r="358" spans="1:13" x14ac:dyDescent="0.3">
@@ -22273,7 +22273,7 @@
         <v>32.587859424920126</v>
       </c>
       <c r="M358" s="1">
-        <v>1566.5878594249202</v>
+        <v>1271.830544450738</v>
       </c>
     </row>
     <row r="359" spans="1:13" x14ac:dyDescent="0.3">
@@ -22316,7 +22316,7 @@
         <v>31.452631578947376</v>
       </c>
       <c r="M359" s="1">
-        <v>418.45263157894738</v>
+        <v>313.75677904438521</v>
       </c>
     </row>
     <row r="360" spans="1:13" x14ac:dyDescent="0.3">
@@ -22359,7 +22359,7 @@
         <v>32.064777327935218</v>
       </c>
       <c r="M360" s="1">
-        <v>199.06477732793522</v>
+        <v>180.7229242927915</v>
       </c>
     </row>
     <row r="361" spans="1:13" x14ac:dyDescent="0.3">
@@ -22401,7 +22401,7 @@
         <v>30</v>
       </c>
       <c r="M361" s="1">
-        <v>335</v>
+        <v>344.9387755102041</v>
       </c>
     </row>
     <row r="362" spans="1:13" x14ac:dyDescent="0.3">
@@ -22443,7 +22443,7 @@
         <v>30</v>
       </c>
       <c r="M362" s="1">
-        <v>371</v>
+        <v>349.10334346504561</v>
       </c>
     </row>
     <row r="363" spans="1:13" x14ac:dyDescent="0.3">
@@ -22560,7 +22560,7 @@
         <v>30</v>
       </c>
       <c r="M365" s="1">
-        <v>174</v>
+        <v>221.90163934426232</v>
       </c>
     </row>
     <row r="366" spans="1:13" x14ac:dyDescent="0.3">
@@ -22603,7 +22603,7 @@
         <v>36.273764258555133</v>
       </c>
       <c r="M366" s="1">
-        <v>456.27376425855516</v>
+        <v>386.02059970159314</v>
       </c>
     </row>
     <row r="367" spans="1:13" x14ac:dyDescent="0.3">
@@ -22646,7 +22646,7 @@
         <v>33.690139605496213</v>
       </c>
       <c r="M367" s="1">
-        <v>63.690139605496213</v>
+        <v>65.598207596877586</v>
       </c>
     </row>
     <row r="368" spans="1:13" x14ac:dyDescent="0.3">
@@ -22688,7 +22688,7 @@
         <v>30</v>
       </c>
       <c r="M368" s="1">
-        <v>60</v>
+        <v>62.548346285920836</v>
       </c>
     </row>
     <row r="369" spans="1:13" x14ac:dyDescent="0.3">
@@ -22727,7 +22727,7 @@
         <v>30</v>
       </c>
       <c r="M369" s="1">
-        <v>60</v>
+        <v>74.35260027451578</v>
       </c>
     </row>
     <row r="370" spans="1:13" x14ac:dyDescent="0.3">
@@ -22806,7 +22806,7 @@
         <v>37.241379310344826</v>
       </c>
       <c r="M371" s="1">
-        <v>1115.2413793103449</v>
+        <v>876.23466790094858</v>
       </c>
     </row>
     <row r="372" spans="1:13" x14ac:dyDescent="0.3">
@@ -22845,7 +22845,7 @@
         <v>30</v>
       </c>
       <c r="M372" s="1">
-        <v>60</v>
+        <v>68.771952885236345</v>
       </c>
     </row>
     <row r="373" spans="1:13" x14ac:dyDescent="0.3">
@@ -22884,7 +22884,7 @@
         <v>30</v>
       </c>
       <c r="M373" s="1">
-        <v>152</v>
+        <v>137.44031093836759</v>
       </c>
     </row>
     <row r="374" spans="1:13" x14ac:dyDescent="0.3">
@@ -22923,7 +22923,7 @@
         <v>30</v>
       </c>
       <c r="M374" s="1">
-        <v>114</v>
+        <v>113.95582329317271</v>
       </c>
     </row>
     <row r="375" spans="1:13" x14ac:dyDescent="0.3">
@@ -22962,7 +22962,7 @@
         <v>30</v>
       </c>
       <c r="M375" s="1">
-        <v>100</v>
+        <v>98.99289099526068</v>
       </c>
     </row>
     <row r="376" spans="1:13" x14ac:dyDescent="0.3">
@@ -23001,7 +23001,7 @@
         <v>30</v>
       </c>
       <c r="M376" s="1">
-        <v>119</v>
+        <v>123.5288888888889</v>
       </c>
     </row>
     <row r="377" spans="1:13" x14ac:dyDescent="0.3">
@@ -23041,7 +23041,7 @@
         <v>36.023725834797894</v>
       </c>
       <c r="M377" s="1">
-        <v>66.023725834797887</v>
+        <v>74.170478217861515</v>
       </c>
     </row>
     <row r="378" spans="1:13" x14ac:dyDescent="0.3">
@@ -23081,7 +23081,7 @@
         <v>30.199632778602925</v>
       </c>
       <c r="M378" s="1">
-        <v>60.199632778602925</v>
+        <v>70.870522871573144</v>
       </c>
     </row>
     <row r="379" spans="1:13" x14ac:dyDescent="0.3">
@@ -23120,7 +23120,7 @@
         <v>30</v>
       </c>
       <c r="M379" s="1">
-        <v>166</v>
+        <v>156.31578947368422</v>
       </c>
     </row>
     <row r="380" spans="1:13" x14ac:dyDescent="0.3">
@@ -23160,7 +23160,7 @@
         <v>43.260116703828452</v>
       </c>
       <c r="M380" s="1">
-        <v>100.26011670382846</v>
+        <v>101.56533216705029</v>
       </c>
     </row>
     <row r="381" spans="1:13" x14ac:dyDescent="0.3">
@@ -23202,7 +23202,7 @@
         <v>30</v>
       </c>
       <c r="M381" s="1">
-        <v>507</v>
+        <v>698.22393822393826</v>
       </c>
     </row>
     <row r="382" spans="1:13" x14ac:dyDescent="0.3">
@@ -23241,7 +23241,7 @@
         <v>30</v>
       </c>
       <c r="M382" s="1">
-        <v>372</v>
+        <v>473.13253012048187</v>
       </c>
     </row>
     <row r="383" spans="1:13" x14ac:dyDescent="0.3">
@@ -23281,7 +23281,7 @@
         <v>33.606871919001094</v>
       </c>
       <c r="M383" s="1">
-        <v>63.606871919001094</v>
+        <v>74.61576855295506</v>
       </c>
     </row>
     <row r="384" spans="1:13" x14ac:dyDescent="0.3">
@@ -23321,7 +23321,7 @@
         <v>31.445128576602677</v>
       </c>
       <c r="M384" s="1">
-        <v>99.445128576602684</v>
+        <v>96.673916803781339</v>
       </c>
     </row>
     <row r="385" spans="1:13" x14ac:dyDescent="0.3">
@@ -23360,7 +23360,7 @@
         <v>30</v>
       </c>
       <c r="M385" s="1">
-        <v>114</v>
+        <v>105.68401287553648</v>
       </c>
     </row>
     <row r="386" spans="1:13" x14ac:dyDescent="0.3">
@@ -23399,7 +23399,7 @@
         <v>30</v>
       </c>
       <c r="M386" s="1">
-        <v>87</v>
+        <v>90.369078222548666</v>
       </c>
     </row>
     <row r="387" spans="1:13" x14ac:dyDescent="0.3">
@@ -23438,7 +23438,7 @@
         <v>30</v>
       </c>
       <c r="M387" s="1">
-        <v>60</v>
+        <v>66.77227209944752</v>
       </c>
     </row>
     <row r="388" spans="1:13" x14ac:dyDescent="0.3">
@@ -23477,7 +23477,7 @@
         <v>30</v>
       </c>
       <c r="M388" s="1">
-        <v>134</v>
+        <v>131.98500535523027</v>
       </c>
     </row>
     <row r="389" spans="1:13" x14ac:dyDescent="0.3">
@@ -23516,7 +23516,7 @@
         <v>30</v>
       </c>
       <c r="M389" s="1">
-        <v>60</v>
+        <v>72.651567064594076</v>
       </c>
     </row>
     <row r="390" spans="1:13" x14ac:dyDescent="0.3">
@@ -23555,7 +23555,7 @@
         <v>30</v>
       </c>
       <c r="M390" s="1">
-        <v>69</v>
+        <v>99.592476489028215</v>
       </c>
     </row>
     <row r="391" spans="1:13" x14ac:dyDescent="0.3">
@@ -23595,7 +23595,7 @@
         <v>40.845556514236407</v>
       </c>
       <c r="M391" s="1">
-        <v>568.84555651423636</v>
+        <v>540.23356141019724</v>
       </c>
     </row>
     <row r="392" spans="1:13" x14ac:dyDescent="0.3">
@@ -23673,7 +23673,7 @@
         <v>30</v>
       </c>
       <c r="M393" s="1">
-        <v>63</v>
+        <v>61.019842270157369</v>
       </c>
     </row>
     <row r="394" spans="1:13" x14ac:dyDescent="0.3">
@@ -23713,7 +23713,7 @@
         <v>32.331378299120232</v>
       </c>
       <c r="M394" s="1">
-        <v>121.33137829912023</v>
+        <v>132.81032132141587</v>
       </c>
     </row>
     <row r="395" spans="1:13" x14ac:dyDescent="0.3">
@@ -23752,7 +23752,7 @@
         <v>30</v>
       </c>
       <c r="M395" s="1">
-        <v>114</v>
+        <v>106.17032531076437</v>
       </c>
     </row>
     <row r="396" spans="1:13" x14ac:dyDescent="0.3">
@@ -23792,7 +23792,7 @@
         <v>35.241193945395395</v>
       </c>
       <c r="M396" s="1">
-        <v>152.24119394539539</v>
+        <v>140.30390774243074</v>
       </c>
     </row>
     <row r="397" spans="1:13" x14ac:dyDescent="0.3">
@@ -23832,7 +23832,7 @@
         <v>33.467336683417088</v>
       </c>
       <c r="M397" s="1">
-        <v>165.4673366834171</v>
+        <v>177.74549853782946</v>
       </c>
     </row>
     <row r="398" spans="1:13" x14ac:dyDescent="0.3">
@@ -23872,7 +23872,7 @@
         <v>34.117647058823522</v>
       </c>
       <c r="M398" s="1">
-        <v>756.11764705882354</v>
+        <v>867.45098039215691</v>
       </c>
     </row>
     <row r="399" spans="1:13" x14ac:dyDescent="0.3">
@@ -23911,7 +23911,7 @@
         <v>30</v>
       </c>
       <c r="M399" s="1">
-        <v>331</v>
+        <v>536.59630606860151</v>
       </c>
     </row>
     <row r="400" spans="1:13" x14ac:dyDescent="0.3">
@@ -23951,7 +23951,7 @@
         <v>31.26558941546471</v>
       </c>
       <c r="M400" s="1">
-        <v>61.26558941546471</v>
+        <v>85.13187876813538</v>
       </c>
     </row>
     <row r="401" spans="1:13" x14ac:dyDescent="0.3">
@@ -23993,7 +23993,7 @@
         <v>30</v>
       </c>
       <c r="M401" s="1">
-        <v>1489</v>
+        <v>1110.6081081081079</v>
       </c>
     </row>
     <row r="402" spans="1:13" x14ac:dyDescent="0.3">
@@ -24033,7 +24033,7 @@
         <v>35.09906939049268</v>
       </c>
       <c r="M402" s="1">
-        <v>67.099069390492673</v>
+        <v>66.180950571949992</v>
       </c>
     </row>
     <row r="403" spans="1:13" x14ac:dyDescent="0.3">
@@ -24072,7 +24072,7 @@
         <v>30</v>
       </c>
       <c r="M403" s="1">
-        <v>201</v>
+        <v>191.01562499999994</v>
       </c>
     </row>
     <row r="404" spans="1:13" x14ac:dyDescent="0.3">
@@ -24112,7 +24112,7 @@
         <v>30.278422273781903</v>
       </c>
       <c r="M404" s="1">
-        <v>60.278422273781899</v>
+        <v>60.328009050641406</v>
       </c>
     </row>
     <row r="405" spans="1:13" x14ac:dyDescent="0.3">
@@ -24155,7 +24155,7 @@
         <v>33.340540540540545</v>
       </c>
       <c r="M405" s="1">
-        <v>163.34054054054053</v>
+        <v>156.62821177341726</v>
       </c>
     </row>
     <row r="406" spans="1:13" x14ac:dyDescent="0.3">
@@ -24198,7 +24198,7 @@
         <v>36.651120464111017</v>
       </c>
       <c r="M406" s="1">
-        <v>326.65112046411105</v>
+        <v>340.07969189268249</v>
       </c>
     </row>
     <row r="407" spans="1:13" x14ac:dyDescent="0.3">
@@ -24238,7 +24238,7 @@
         <v>35.834609494640127</v>
       </c>
       <c r="M407" s="1">
-        <v>65.834609494640119</v>
+        <v>87.680451279629978</v>
       </c>
     </row>
     <row r="408" spans="1:13" x14ac:dyDescent="0.3">
@@ -24280,7 +24280,7 @@
         <v>30</v>
       </c>
       <c r="M408" s="1">
-        <v>96</v>
+        <v>94.111182934712346</v>
       </c>
     </row>
     <row r="409" spans="1:13" x14ac:dyDescent="0.3">
@@ -24323,7 +24323,7 @@
         <v>30.102389078498295</v>
       </c>
       <c r="M409" s="1">
-        <v>62.102389078498291</v>
+        <v>89.13710542058125</v>
       </c>
     </row>
     <row r="410" spans="1:13" x14ac:dyDescent="0.3">
@@ -24366,7 +24366,7 @@
         <v>35.248202670318385</v>
       </c>
       <c r="M410" s="1">
-        <v>102.24820267031839</v>
+        <v>81.54607501074392</v>
       </c>
     </row>
     <row r="411" spans="1:13" x14ac:dyDescent="0.3">
@@ -24408,7 +24408,7 @@
         <v>30</v>
       </c>
       <c r="M411" s="1">
-        <v>92</v>
+        <v>84.822335025380724</v>
       </c>
     </row>
     <row r="412" spans="1:13" x14ac:dyDescent="0.3">
@@ -24451,7 +24451,7 @@
         <v>35.297397769516742</v>
       </c>
       <c r="M412" s="1">
-        <v>193.29739776951675</v>
+        <v>168.84578486629093</v>
       </c>
     </row>
     <row r="413" spans="1:13" x14ac:dyDescent="0.3">
@@ -24490,7 +24490,7 @@
         <v>30</v>
       </c>
       <c r="M413" s="1">
-        <v>60</v>
+        <v>60.423662848882472</v>
       </c>
     </row>
     <row r="414" spans="1:13" x14ac:dyDescent="0.3">
@@ -24529,7 +24529,7 @@
         <v>30</v>
       </c>
       <c r="M414" s="1">
-        <v>252</v>
+        <v>283.62831858407083</v>
       </c>
     </row>
     <row r="415" spans="1:13" x14ac:dyDescent="0.3">
@@ -24571,7 +24571,7 @@
         <v>30</v>
       </c>
       <c r="M415" s="1">
-        <v>612</v>
+        <v>13774.800000000003</v>
       </c>
     </row>
     <row r="416" spans="1:13" x14ac:dyDescent="0.3">
@@ -24613,7 +24613,7 @@
         <v>30</v>
       </c>
       <c r="M416" s="1">
-        <v>162</v>
+        <v>138.38411329752643</v>
       </c>
     </row>
     <row r="417" spans="1:13" x14ac:dyDescent="0.3">
@@ -24656,7 +24656,7 @@
         <v>32.349194944315627</v>
       </c>
       <c r="M417" s="1">
-        <v>228.34919494431563</v>
+        <v>197.88317999107898</v>
       </c>
     </row>
     <row r="418" spans="1:13" x14ac:dyDescent="0.3">
@@ -24695,7 +24695,7 @@
         <v>30</v>
       </c>
       <c r="M418" s="1">
-        <v>818</v>
+        <v>1428.963730569948</v>
       </c>
     </row>
     <row r="419" spans="1:13" x14ac:dyDescent="0.3">
@@ -24735,7 +24735,7 @@
         <v>39.211618257261421</v>
       </c>
       <c r="M419" s="1">
-        <v>371.21161825726142</v>
+        <v>332.28854133418457</v>
       </c>
     </row>
     <row r="420" spans="1:13" x14ac:dyDescent="0.3">
@@ -24777,7 +24777,7 @@
         <v>45</v>
       </c>
       <c r="M420" s="1">
-        <v>128</v>
+        <v>132.11328356583707</v>
       </c>
     </row>
     <row r="421" spans="1:13" x14ac:dyDescent="0.3">
@@ -24819,7 +24819,7 @@
         <v>30</v>
       </c>
       <c r="M421" s="1">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="422" spans="1:13" x14ac:dyDescent="0.3">
@@ -24861,7 +24861,7 @@
         <v>30</v>
       </c>
       <c r="M422" s="1">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resync updated Max DOI for PAR001 (96 Hari) in Master data
</commit_message>
<xml_diff>
--- a/Master produk.xlsx
+++ b/Master produk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Argo\Project AI\DOI BULANAN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4AD3A7F-E849-4CF6-8169-FC03A91F7171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3CAAB9-805C-4734-8792-99F24DAF9A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7A4E4CA0-3C41-4699-9069-61742CAEF447}"/>
   </bookViews>
@@ -14217,7 +14217,7 @@
         <v>31.336825902930883</v>
       </c>
       <c r="M156" s="1">
-        <v>61.340846673841298</v>
+        <v>96</v>
       </c>
     </row>
     <row r="157" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
feat: Add brand logos, glassmorphism UI, multi-select popover search, connected cascading filters, 6-month avg sales & Rupiah defaults
</commit_message>
<xml_diff>
--- a/Master produk.xlsx
+++ b/Master produk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Argo\Project AI\DOI BULANAN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3CAAB9-805C-4734-8792-99F24DAF9A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE0C36B-B01A-4112-8227-76DD97418F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7A4E4CA0-3C41-4699-9069-61742CAEF447}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3067" uniqueCount="1384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3421" uniqueCount="1386">
   <si>
     <t>GB</t>
   </si>
@@ -4192,6 +4192,12 @@
   </si>
   <si>
     <t>Max DOI</t>
+  </si>
+  <si>
+    <t>Aktif</t>
+  </si>
+  <si>
+    <t>Streamline</t>
   </si>
 </sst>
 </file>
@@ -8063,6 +8069,9 @@
       <c r="H2" t="s">
         <v>1276</v>
       </c>
+      <c r="I2" t="s">
+        <v>1384</v>
+      </c>
       <c r="J2">
         <v>19991</v>
       </c>
@@ -8103,6 +8112,9 @@
       <c r="H3" t="s">
         <v>1276</v>
       </c>
+      <c r="I3" t="s">
+        <v>1384</v>
+      </c>
       <c r="J3">
         <v>16662</v>
       </c>
@@ -8143,6 +8155,9 @@
       <c r="H4" t="s">
         <v>1276</v>
       </c>
+      <c r="I4" t="s">
+        <v>1384</v>
+      </c>
       <c r="J4">
         <v>19325</v>
       </c>
@@ -8183,6 +8198,9 @@
       <c r="H5" t="s">
         <v>1276</v>
       </c>
+      <c r="I5" t="s">
+        <v>1384</v>
+      </c>
       <c r="J5">
         <v>16024</v>
       </c>
@@ -8223,6 +8241,9 @@
       <c r="H6" t="s">
         <v>1277</v>
       </c>
+      <c r="I6" t="s">
+        <v>1384</v>
+      </c>
       <c r="J6">
         <v>85750</v>
       </c>
@@ -8263,6 +8284,9 @@
       <c r="H7" t="s">
         <v>1277</v>
       </c>
+      <c r="I7" t="s">
+        <v>1384</v>
+      </c>
       <c r="J7">
         <v>50000</v>
       </c>
@@ -8303,6 +8327,9 @@
       <c r="H8" t="s">
         <v>1277</v>
       </c>
+      <c r="I8" t="s">
+        <v>1384</v>
+      </c>
       <c r="J8">
         <v>5500</v>
       </c>
@@ -8342,6 +8369,9 @@
       <c r="H9" t="s">
         <v>1277</v>
       </c>
+      <c r="I9" t="s">
+        <v>1384</v>
+      </c>
       <c r="J9">
         <v>13333</v>
       </c>
@@ -8381,6 +8411,9 @@
       <c r="H10" t="s">
         <v>1277</v>
       </c>
+      <c r="I10" t="s">
+        <v>1384</v>
+      </c>
       <c r="J10">
         <v>13333</v>
       </c>
@@ -8420,6 +8453,9 @@
       <c r="H11" t="s">
         <v>1276</v>
       </c>
+      <c r="I11" t="s">
+        <v>1384</v>
+      </c>
       <c r="J11">
         <v>39734</v>
       </c>
@@ -8503,6 +8539,9 @@
       <c r="H13" t="s">
         <v>1277</v>
       </c>
+      <c r="I13" t="s">
+        <v>1384</v>
+      </c>
       <c r="J13">
         <v>2306</v>
       </c>
@@ -8542,6 +8581,9 @@
       <c r="H14" t="s">
         <v>1277</v>
       </c>
+      <c r="I14" t="s">
+        <v>1384</v>
+      </c>
       <c r="J14">
         <v>2298</v>
       </c>
@@ -8582,6 +8624,9 @@
       <c r="H15" t="s">
         <v>1277</v>
       </c>
+      <c r="I15" t="s">
+        <v>1384</v>
+      </c>
       <c r="J15">
         <v>2285</v>
       </c>
@@ -8622,6 +8667,9 @@
       <c r="H16" t="s">
         <v>1277</v>
       </c>
+      <c r="I16" t="s">
+        <v>1384</v>
+      </c>
       <c r="J16">
         <v>26080</v>
       </c>
@@ -8661,6 +8709,9 @@
       <c r="H17" t="s">
         <v>1276</v>
       </c>
+      <c r="I17" t="s">
+        <v>1384</v>
+      </c>
       <c r="J17">
         <v>98808</v>
       </c>
@@ -8701,6 +8752,9 @@
       <c r="H18" t="s">
         <v>1277</v>
       </c>
+      <c r="I18" t="s">
+        <v>1384</v>
+      </c>
       <c r="J18">
         <v>12593</v>
       </c>
@@ -8741,6 +8795,9 @@
       <c r="H19" t="s">
         <v>1277</v>
       </c>
+      <c r="I19" t="s">
+        <v>1384</v>
+      </c>
       <c r="J19">
         <v>24373</v>
       </c>
@@ -8781,6 +8838,9 @@
       <c r="H20" t="s">
         <v>1276</v>
       </c>
+      <c r="I20" t="s">
+        <v>1384</v>
+      </c>
       <c r="J20">
         <v>20053</v>
       </c>
@@ -8821,6 +8881,9 @@
       <c r="H21" t="s">
         <v>1276</v>
       </c>
+      <c r="I21" t="s">
+        <v>1384</v>
+      </c>
       <c r="J21">
         <v>16642</v>
       </c>
@@ -8861,6 +8924,9 @@
       <c r="H22" t="s">
         <v>1276</v>
       </c>
+      <c r="I22" t="s">
+        <v>1384</v>
+      </c>
       <c r="J22">
         <v>20005</v>
       </c>
@@ -8901,6 +8967,9 @@
       <c r="H23" t="s">
         <v>1276</v>
       </c>
+      <c r="I23" t="s">
+        <v>1384</v>
+      </c>
       <c r="J23">
         <v>16677</v>
       </c>
@@ -8941,6 +9010,9 @@
       <c r="H24" t="s">
         <v>1277</v>
       </c>
+      <c r="I24" t="s">
+        <v>1384</v>
+      </c>
       <c r="J24">
         <v>9201</v>
       </c>
@@ -8981,6 +9053,9 @@
       <c r="H25" t="s">
         <v>1277</v>
       </c>
+      <c r="I25" t="s">
+        <v>1384</v>
+      </c>
       <c r="J25">
         <v>32399</v>
       </c>
@@ -9021,6 +9096,9 @@
       <c r="H26" t="s">
         <v>1277</v>
       </c>
+      <c r="I26" t="s">
+        <v>1384</v>
+      </c>
       <c r="J26">
         <v>16188</v>
       </c>
@@ -9061,6 +9139,9 @@
       <c r="H27" t="s">
         <v>1277</v>
       </c>
+      <c r="I27" t="s">
+        <v>1384</v>
+      </c>
       <c r="J27">
         <v>11664</v>
       </c>
@@ -9100,6 +9181,9 @@
       <c r="H28" t="s">
         <v>1277</v>
       </c>
+      <c r="I28" t="s">
+        <v>1384</v>
+      </c>
       <c r="J28">
         <v>11664</v>
       </c>
@@ -9140,6 +9224,9 @@
       <c r="H29" t="s">
         <v>1277</v>
       </c>
+      <c r="I29" t="s">
+        <v>1385</v>
+      </c>
       <c r="J29">
         <v>8653</v>
       </c>
@@ -9179,6 +9266,9 @@
       <c r="H30" t="s">
         <v>1277</v>
       </c>
+      <c r="I30" t="s">
+        <v>1384</v>
+      </c>
       <c r="J30">
         <v>6610</v>
       </c>
@@ -9218,6 +9308,9 @@
       <c r="H31" t="s">
         <v>1277</v>
       </c>
+      <c r="I31" t="s">
+        <v>1384</v>
+      </c>
       <c r="J31">
         <v>8653</v>
       </c>
@@ -9258,6 +9351,9 @@
       <c r="H32" t="s">
         <v>1277</v>
       </c>
+      <c r="I32" t="s">
+        <v>1384</v>
+      </c>
       <c r="J32">
         <v>4840</v>
       </c>
@@ -9298,6 +9394,9 @@
       <c r="H33" t="s">
         <v>1277</v>
       </c>
+      <c r="I33" t="s">
+        <v>1384</v>
+      </c>
       <c r="J33">
         <v>6635</v>
       </c>
@@ -9338,6 +9437,9 @@
       <c r="H34" t="s">
         <v>1277</v>
       </c>
+      <c r="I34" t="s">
+        <v>1385</v>
+      </c>
       <c r="J34">
         <v>6488</v>
       </c>
@@ -9377,6 +9479,9 @@
       <c r="H35" t="s">
         <v>1277</v>
       </c>
+      <c r="I35" t="s">
+        <v>1384</v>
+      </c>
       <c r="J35">
         <v>4865</v>
       </c>
@@ -9417,6 +9522,9 @@
       <c r="H36" t="s">
         <v>1277</v>
       </c>
+      <c r="I36" t="s">
+        <v>1384</v>
+      </c>
       <c r="J36">
         <v>13651</v>
       </c>
@@ -9457,6 +9565,9 @@
       <c r="H37" t="s">
         <v>1277</v>
       </c>
+      <c r="I37" t="s">
+        <v>1384</v>
+      </c>
       <c r="J37">
         <v>12946</v>
       </c>
@@ -9497,6 +9608,9 @@
       <c r="H38" t="s">
         <v>1277</v>
       </c>
+      <c r="I38" t="s">
+        <v>1384</v>
+      </c>
       <c r="J38">
         <v>6685</v>
       </c>
@@ -9536,6 +9650,9 @@
       <c r="H39" t="s">
         <v>1277</v>
       </c>
+      <c r="I39" t="s">
+        <v>1384</v>
+      </c>
       <c r="J39">
         <v>5962</v>
       </c>
@@ -9576,6 +9693,9 @@
       <c r="H40" t="s">
         <v>1277</v>
       </c>
+      <c r="I40" t="s">
+        <v>1385</v>
+      </c>
       <c r="J40">
         <v>7707</v>
       </c>
@@ -9658,6 +9778,9 @@
       <c r="H42" t="s">
         <v>1277</v>
       </c>
+      <c r="I42" t="s">
+        <v>1384</v>
+      </c>
       <c r="J42">
         <v>5387</v>
       </c>
@@ -9698,6 +9821,9 @@
       <c r="H43" t="s">
         <v>1277</v>
       </c>
+      <c r="I43" t="s">
+        <v>1384</v>
+      </c>
       <c r="J43">
         <v>1601</v>
       </c>
@@ -9737,6 +9863,9 @@
       <c r="H44" t="s">
         <v>1277</v>
       </c>
+      <c r="I44" t="s">
+        <v>1384</v>
+      </c>
       <c r="J44">
         <v>440</v>
       </c>
@@ -9777,6 +9906,9 @@
       <c r="H45" t="s">
         <v>1276</v>
       </c>
+      <c r="I45" t="s">
+        <v>1384</v>
+      </c>
       <c r="J45">
         <v>10022</v>
       </c>
@@ -9817,6 +9949,9 @@
       <c r="H46" t="s">
         <v>1276</v>
       </c>
+      <c r="I46" t="s">
+        <v>1384</v>
+      </c>
       <c r="J46">
         <v>20034</v>
       </c>
@@ -9857,6 +9992,9 @@
       <c r="H47" t="s">
         <v>1276</v>
       </c>
+      <c r="I47" t="s">
+        <v>1384</v>
+      </c>
       <c r="J47">
         <v>4831</v>
       </c>
@@ -9897,6 +10035,9 @@
       <c r="H48" t="s">
         <v>1276</v>
       </c>
+      <c r="I48" t="s">
+        <v>1384</v>
+      </c>
       <c r="J48">
         <v>40297</v>
       </c>
@@ -9937,6 +10078,9 @@
       <c r="H49" t="s">
         <v>1276</v>
       </c>
+      <c r="I49" t="s">
+        <v>1384</v>
+      </c>
       <c r="J49">
         <v>20306</v>
       </c>
@@ -9977,6 +10121,9 @@
       <c r="H50" t="s">
         <v>1276</v>
       </c>
+      <c r="I50" t="s">
+        <v>1384</v>
+      </c>
       <c r="J50">
         <v>9732</v>
       </c>
@@ -10017,6 +10164,9 @@
       <c r="H51" t="s">
         <v>1277</v>
       </c>
+      <c r="I51" t="s">
+        <v>1384</v>
+      </c>
       <c r="J51">
         <v>2506</v>
       </c>
@@ -10057,6 +10207,9 @@
       <c r="H52" t="s">
         <v>1277</v>
       </c>
+      <c r="I52" t="s">
+        <v>1384</v>
+      </c>
       <c r="J52">
         <v>1206</v>
       </c>
@@ -10097,6 +10250,9 @@
       <c r="H53" t="s">
         <v>1277</v>
       </c>
+      <c r="I53" t="s">
+        <v>1384</v>
+      </c>
       <c r="J53">
         <v>2460</v>
       </c>
@@ -10137,6 +10293,9 @@
       <c r="H54" t="s">
         <v>1276</v>
       </c>
+      <c r="I54" t="s">
+        <v>1384</v>
+      </c>
       <c r="J54">
         <v>20306</v>
       </c>
@@ -10177,6 +10336,9 @@
       <c r="H55" t="s">
         <v>1276</v>
       </c>
+      <c r="I55" t="s">
+        <v>1384</v>
+      </c>
       <c r="J55">
         <v>42105</v>
       </c>
@@ -10217,6 +10379,9 @@
       <c r="H56" t="s">
         <v>1276</v>
       </c>
+      <c r="I56" t="s">
+        <v>1384</v>
+      </c>
       <c r="J56">
         <v>9732</v>
       </c>
@@ -10257,6 +10422,9 @@
       <c r="H57" t="s">
         <v>1276</v>
       </c>
+      <c r="I57" t="s">
+        <v>1384</v>
+      </c>
       <c r="J57">
         <v>40744</v>
       </c>
@@ -10297,6 +10465,9 @@
       <c r="H58" t="s">
         <v>1276</v>
       </c>
+      <c r="I58" t="s">
+        <v>1384</v>
+      </c>
       <c r="J58">
         <v>20270</v>
       </c>
@@ -10337,6 +10508,9 @@
       <c r="H59" t="s">
         <v>1276</v>
       </c>
+      <c r="I59" t="s">
+        <v>1384</v>
+      </c>
       <c r="J59">
         <v>9664</v>
       </c>
@@ -10377,6 +10551,9 @@
       <c r="H60" t="s">
         <v>1277</v>
       </c>
+      <c r="I60" t="s">
+        <v>1384</v>
+      </c>
       <c r="J60">
         <v>20150</v>
       </c>
@@ -10417,6 +10594,9 @@
       <c r="H61" t="s">
         <v>1277</v>
       </c>
+      <c r="I61" t="s">
+        <v>1384</v>
+      </c>
       <c r="J61">
         <v>9658</v>
       </c>
@@ -10457,6 +10637,9 @@
       <c r="H62" t="s">
         <v>1277</v>
       </c>
+      <c r="I62" t="s">
+        <v>1384</v>
+      </c>
       <c r="J62">
         <v>20214</v>
       </c>
@@ -10497,6 +10680,9 @@
       <c r="H63" t="s">
         <v>1277</v>
       </c>
+      <c r="I63" t="s">
+        <v>1384</v>
+      </c>
       <c r="J63">
         <v>9603</v>
       </c>
@@ -10537,6 +10723,9 @@
       <c r="H64" t="s">
         <v>1277</v>
       </c>
+      <c r="I64" t="s">
+        <v>1384</v>
+      </c>
       <c r="J64">
         <v>2445</v>
       </c>
@@ -10577,6 +10766,9 @@
       <c r="H65" t="s">
         <v>1277</v>
       </c>
+      <c r="I65" t="s">
+        <v>1384</v>
+      </c>
       <c r="J65">
         <v>8500</v>
       </c>
@@ -10617,6 +10809,9 @@
       <c r="H66" t="s">
         <v>1277</v>
       </c>
+      <c r="I66" t="s">
+        <v>1384</v>
+      </c>
       <c r="J66">
         <v>2750</v>
       </c>
@@ -10657,6 +10852,9 @@
       <c r="H67" t="s">
         <v>1277</v>
       </c>
+      <c r="I67" t="s">
+        <v>1384</v>
+      </c>
       <c r="J67">
         <v>4036</v>
       </c>
@@ -10697,6 +10895,9 @@
       <c r="H68" t="s">
         <v>1277</v>
       </c>
+      <c r="I68" t="s">
+        <v>1385</v>
+      </c>
       <c r="J68">
         <v>1042</v>
       </c>
@@ -10736,6 +10937,9 @@
       <c r="H69" t="s">
         <v>1277</v>
       </c>
+      <c r="I69" t="s">
+        <v>1384</v>
+      </c>
       <c r="J69">
         <v>437</v>
       </c>
@@ -10776,6 +10980,9 @@
       <c r="H70" t="s">
         <v>1277</v>
       </c>
+      <c r="I70" t="s">
+        <v>1384</v>
+      </c>
       <c r="J70">
         <v>221</v>
       </c>
@@ -10816,6 +11023,9 @@
       <c r="H71" t="s">
         <v>1277</v>
       </c>
+      <c r="I71" t="s">
+        <v>1384</v>
+      </c>
       <c r="J71">
         <v>437</v>
       </c>
@@ -10856,6 +11066,9 @@
       <c r="H72" t="s">
         <v>1277</v>
       </c>
+      <c r="I72" t="s">
+        <v>1384</v>
+      </c>
       <c r="J72">
         <v>222</v>
       </c>
@@ -10896,6 +11109,9 @@
       <c r="H73" t="s">
         <v>1277</v>
       </c>
+      <c r="I73" t="s">
+        <v>1384</v>
+      </c>
       <c r="J73">
         <v>1967</v>
       </c>
@@ -10935,6 +11151,9 @@
       <c r="H74" t="s">
         <v>1277</v>
       </c>
+      <c r="I74" t="s">
+        <v>1384</v>
+      </c>
       <c r="J74">
         <v>1965</v>
       </c>
@@ -10975,6 +11194,9 @@
       <c r="H75" t="s">
         <v>1277</v>
       </c>
+      <c r="I75" t="s">
+        <v>1384</v>
+      </c>
       <c r="J75">
         <v>953</v>
       </c>
@@ -11015,6 +11237,9 @@
       <c r="H76" t="s">
         <v>1277</v>
       </c>
+      <c r="I76" t="s">
+        <v>1384</v>
+      </c>
       <c r="J76">
         <v>1647</v>
       </c>
@@ -11054,6 +11279,9 @@
       <c r="H77" t="s">
         <v>1277</v>
       </c>
+      <c r="I77" t="s">
+        <v>1384</v>
+      </c>
       <c r="J77">
         <v>1597</v>
       </c>
@@ -11436,6 +11664,9 @@
       <c r="H86" t="s">
         <v>1277</v>
       </c>
+      <c r="I86" t="s">
+        <v>1384</v>
+      </c>
       <c r="J86">
         <v>4894</v>
       </c>
@@ -11475,6 +11706,9 @@
       <c r="H87" t="s">
         <v>1277</v>
       </c>
+      <c r="I87" t="s">
+        <v>1384</v>
+      </c>
       <c r="J87">
         <v>9657</v>
       </c>
@@ -11515,6 +11749,9 @@
       <c r="H88" t="s">
         <v>1277</v>
       </c>
+      <c r="I88" t="s">
+        <v>1384</v>
+      </c>
       <c r="J88">
         <v>2323</v>
       </c>
@@ -11554,6 +11791,9 @@
       <c r="H89" t="s">
         <v>1277</v>
       </c>
+      <c r="I89" t="s">
+        <v>1384</v>
+      </c>
       <c r="J89">
         <v>936</v>
       </c>
@@ -11594,6 +11834,9 @@
       <c r="H90" t="s">
         <v>1277</v>
       </c>
+      <c r="I90" t="s">
+        <v>1384</v>
+      </c>
       <c r="J90">
         <v>3195</v>
       </c>
@@ -11633,6 +11876,9 @@
       <c r="H91" t="s">
         <v>1277</v>
       </c>
+      <c r="I91" t="s">
+        <v>1384</v>
+      </c>
       <c r="J91">
         <v>1711</v>
       </c>
@@ -11672,6 +11918,9 @@
       <c r="H92" t="s">
         <v>1277</v>
       </c>
+      <c r="I92" t="s">
+        <v>1384</v>
+      </c>
       <c r="J92">
         <v>757</v>
       </c>
@@ -11711,6 +11960,9 @@
       <c r="H93" t="s">
         <v>1277</v>
       </c>
+      <c r="I93" t="s">
+        <v>1384</v>
+      </c>
       <c r="J93">
         <v>9888</v>
       </c>
@@ -11751,6 +12003,9 @@
       <c r="H94" t="s">
         <v>1277</v>
       </c>
+      <c r="I94" t="s">
+        <v>1384</v>
+      </c>
       <c r="J94">
         <v>25333</v>
       </c>
@@ -11791,6 +12046,9 @@
       <c r="H95" t="s">
         <v>1277</v>
       </c>
+      <c r="I95" t="s">
+        <v>1384</v>
+      </c>
       <c r="J95">
         <v>50600</v>
       </c>
@@ -11831,6 +12089,9 @@
       <c r="H96" t="s">
         <v>1277</v>
       </c>
+      <c r="I96" t="s">
+        <v>1384</v>
+      </c>
       <c r="J96">
         <v>1881</v>
       </c>
@@ -11957,6 +12218,9 @@
       <c r="H99" t="s">
         <v>1277</v>
       </c>
+      <c r="I99" t="s">
+        <v>1384</v>
+      </c>
       <c r="J99">
         <v>72215</v>
       </c>
@@ -11997,6 +12261,9 @@
       <c r="H100" t="s">
         <v>1277</v>
       </c>
+      <c r="I100" t="s">
+        <v>1384</v>
+      </c>
       <c r="J100">
         <v>12088</v>
       </c>
@@ -12037,6 +12304,9 @@
       <c r="H101" t="s">
         <v>1277</v>
       </c>
+      <c r="I101" t="s">
+        <v>1385</v>
+      </c>
       <c r="J101">
         <v>75000</v>
       </c>
@@ -12076,6 +12346,9 @@
       <c r="H102" t="s">
         <v>1277</v>
       </c>
+      <c r="I102" t="s">
+        <v>1385</v>
+      </c>
       <c r="J102">
         <v>12500</v>
       </c>
@@ -12115,6 +12388,9 @@
       <c r="H103" t="s">
         <v>1277</v>
       </c>
+      <c r="I103" t="s">
+        <v>1384</v>
+      </c>
       <c r="J103">
         <v>6495</v>
       </c>
@@ -12154,6 +12430,9 @@
       <c r="H104" t="s">
         <v>1277</v>
       </c>
+      <c r="I104" t="s">
+        <v>1384</v>
+      </c>
       <c r="J104">
         <v>1348</v>
       </c>
@@ -12193,6 +12472,9 @@
       <c r="H105" t="s">
         <v>1277</v>
       </c>
+      <c r="I105" t="s">
+        <v>1384</v>
+      </c>
       <c r="J105">
         <v>1262</v>
       </c>
@@ -12232,6 +12514,9 @@
       <c r="H106" t="s">
         <v>1277</v>
       </c>
+      <c r="I106" t="s">
+        <v>1384</v>
+      </c>
       <c r="J106">
         <v>1171</v>
       </c>
@@ -12271,6 +12556,9 @@
       <c r="H107" t="s">
         <v>1277</v>
       </c>
+      <c r="I107" t="s">
+        <v>1384</v>
+      </c>
       <c r="J107">
         <v>1511</v>
       </c>
@@ -12310,6 +12598,9 @@
       <c r="H108" t="s">
         <v>1277</v>
       </c>
+      <c r="I108" t="s">
+        <v>1384</v>
+      </c>
       <c r="J108">
         <v>1324</v>
       </c>
@@ -12349,6 +12640,9 @@
       <c r="H109" t="s">
         <v>1277</v>
       </c>
+      <c r="I109" t="s">
+        <v>1384</v>
+      </c>
       <c r="J109">
         <v>2014</v>
       </c>
@@ -12389,6 +12683,9 @@
       <c r="H110" t="s">
         <v>1277</v>
       </c>
+      <c r="I110" t="s">
+        <v>1384</v>
+      </c>
       <c r="J110">
         <v>1669</v>
       </c>
@@ -12429,6 +12726,9 @@
       <c r="H111" t="s">
         <v>1277</v>
       </c>
+      <c r="I111" t="s">
+        <v>1384</v>
+      </c>
       <c r="J111">
         <v>1695</v>
       </c>
@@ -12469,6 +12769,9 @@
       <c r="H112" t="s">
         <v>1277</v>
       </c>
+      <c r="I112" t="s">
+        <v>1384</v>
+      </c>
       <c r="J112">
         <v>1311</v>
       </c>
@@ -12509,6 +12812,9 @@
       <c r="H113" t="s">
         <v>1277</v>
       </c>
+      <c r="I113" t="s">
+        <v>1384</v>
+      </c>
       <c r="J113">
         <v>1472</v>
       </c>
@@ -12548,6 +12854,9 @@
       <c r="H114" t="s">
         <v>1277</v>
       </c>
+      <c r="I114" t="s">
+        <v>1384</v>
+      </c>
       <c r="J114">
         <v>1375</v>
       </c>
@@ -12588,6 +12897,9 @@
       <c r="H115" t="s">
         <v>1277</v>
       </c>
+      <c r="I115" t="s">
+        <v>1384</v>
+      </c>
       <c r="J115">
         <v>4896</v>
       </c>
@@ -12628,6 +12940,9 @@
       <c r="H116" t="s">
         <v>1277</v>
       </c>
+      <c r="I116" t="s">
+        <v>1384</v>
+      </c>
       <c r="J116">
         <v>1476</v>
       </c>
@@ -12667,6 +12982,9 @@
       <c r="H117" t="s">
         <v>1277</v>
       </c>
+      <c r="I117" t="s">
+        <v>1384</v>
+      </c>
       <c r="J117">
         <v>2257</v>
       </c>
@@ -12705,6 +13023,9 @@
       <c r="H118" t="s">
         <v>1277</v>
       </c>
+      <c r="I118" t="s">
+        <v>1384</v>
+      </c>
       <c r="J118">
         <v>1684</v>
       </c>
@@ -12745,6 +13066,9 @@
       <c r="H119" t="s">
         <v>1277</v>
       </c>
+      <c r="I119" t="s">
+        <v>1384</v>
+      </c>
       <c r="J119">
         <v>1673</v>
       </c>
@@ -12784,6 +13108,9 @@
       <c r="H120" t="s">
         <v>1277</v>
       </c>
+      <c r="I120" t="s">
+        <v>1384</v>
+      </c>
       <c r="J120">
         <v>1291</v>
       </c>
@@ -12824,6 +13151,9 @@
       <c r="H121" t="s">
         <v>1277</v>
       </c>
+      <c r="I121" t="s">
+        <v>1384</v>
+      </c>
       <c r="J121">
         <v>1612</v>
       </c>
@@ -12864,6 +13194,9 @@
       <c r="H122" t="s">
         <v>1277</v>
       </c>
+      <c r="I122" t="s">
+        <v>1384</v>
+      </c>
       <c r="J122">
         <v>2253</v>
       </c>
@@ -12904,6 +13237,9 @@
       <c r="H123" t="s">
         <v>1277</v>
       </c>
+      <c r="I123" t="s">
+        <v>1384</v>
+      </c>
       <c r="J123">
         <v>2019</v>
       </c>
@@ -12943,6 +13279,9 @@
       <c r="H124" t="s">
         <v>1277</v>
       </c>
+      <c r="I124" t="s">
+        <v>1384</v>
+      </c>
       <c r="J124">
         <v>26177</v>
       </c>
@@ -12982,6 +13321,9 @@
       <c r="H125" t="s">
         <v>1277</v>
       </c>
+      <c r="I125" t="s">
+        <v>1384</v>
+      </c>
       <c r="J125">
         <v>1287</v>
       </c>
@@ -13021,6 +13363,9 @@
       <c r="H126" t="s">
         <v>1277</v>
       </c>
+      <c r="I126" t="s">
+        <v>1384</v>
+      </c>
       <c r="J126">
         <v>3333</v>
       </c>
@@ -13059,6 +13404,9 @@
       <c r="H127" t="s">
         <v>1277</v>
       </c>
+      <c r="I127" t="s">
+        <v>1384</v>
+      </c>
       <c r="J127">
         <v>1239</v>
       </c>
@@ -13098,6 +13446,9 @@
       <c r="H128" t="s">
         <v>1277</v>
       </c>
+      <c r="I128" t="s">
+        <v>1384</v>
+      </c>
       <c r="J128">
         <v>1369</v>
       </c>
@@ -13138,6 +13489,9 @@
       <c r="H129" t="s">
         <v>1277</v>
       </c>
+      <c r="I129" t="s">
+        <v>1384</v>
+      </c>
       <c r="J129">
         <v>1925</v>
       </c>
@@ -13177,6 +13531,9 @@
       <c r="H130" t="s">
         <v>1277</v>
       </c>
+      <c r="I130" t="s">
+        <v>1384</v>
+      </c>
       <c r="J130">
         <v>2838</v>
       </c>
@@ -13217,6 +13574,9 @@
       <c r="H131" t="s">
         <v>1277</v>
       </c>
+      <c r="I131" t="s">
+        <v>1384</v>
+      </c>
       <c r="J131">
         <v>1701</v>
       </c>
@@ -13255,6 +13615,9 @@
       <c r="H132" t="s">
         <v>1277</v>
       </c>
+      <c r="I132" t="s">
+        <v>1384</v>
+      </c>
       <c r="J132">
         <v>1523</v>
       </c>
@@ -13295,6 +13658,9 @@
       <c r="H133" t="s">
         <v>1277</v>
       </c>
+      <c r="I133" t="s">
+        <v>1384</v>
+      </c>
       <c r="J133">
         <v>1269</v>
       </c>
@@ -13333,6 +13699,9 @@
       <c r="H134" t="s">
         <v>1277</v>
       </c>
+      <c r="I134" t="s">
+        <v>1384</v>
+      </c>
       <c r="J134">
         <v>783</v>
       </c>
@@ -13372,6 +13741,9 @@
       <c r="H135" t="s">
         <v>1277</v>
       </c>
+      <c r="I135" t="s">
+        <v>1384</v>
+      </c>
       <c r="J135">
         <v>7500</v>
       </c>
@@ -13410,6 +13782,9 @@
       <c r="H136" t="s">
         <v>1277</v>
       </c>
+      <c r="I136" t="s">
+        <v>1384</v>
+      </c>
       <c r="J136">
         <v>7500</v>
       </c>
@@ -13448,6 +13823,9 @@
       <c r="H137" t="s">
         <v>1277</v>
       </c>
+      <c r="I137" t="s">
+        <v>1384</v>
+      </c>
       <c r="J137">
         <v>7500</v>
       </c>
@@ -13487,6 +13865,9 @@
       <c r="H138" t="s">
         <v>1277</v>
       </c>
+      <c r="I138" t="s">
+        <v>1385</v>
+      </c>
       <c r="J138">
         <v>14286</v>
       </c>
@@ -13525,6 +13906,9 @@
       <c r="H139" t="s">
         <v>1277</v>
       </c>
+      <c r="I139" t="s">
+        <v>1384</v>
+      </c>
       <c r="J139">
         <v>75000</v>
       </c>
@@ -13563,6 +13947,9 @@
       <c r="H140" t="s">
         <v>1277</v>
       </c>
+      <c r="I140" t="s">
+        <v>1384</v>
+      </c>
       <c r="J140">
         <v>75000</v>
       </c>
@@ -13603,7 +13990,7 @@
         <v>1278</v>
       </c>
       <c r="I141" t="s">
-        <v>1282</v>
+        <v>1385</v>
       </c>
       <c r="J141">
         <v>2750</v>
@@ -13644,6 +14031,9 @@
       <c r="H142" t="s">
         <v>1277</v>
       </c>
+      <c r="I142" t="s">
+        <v>1384</v>
+      </c>
       <c r="J142">
         <v>3286</v>
       </c>
@@ -13683,6 +14073,9 @@
       <c r="H143" t="s">
         <v>1277</v>
       </c>
+      <c r="I143" t="s">
+        <v>1384</v>
+      </c>
       <c r="J143">
         <v>24586</v>
       </c>
@@ -13723,6 +14116,9 @@
       <c r="H144" t="s">
         <v>1277</v>
       </c>
+      <c r="I144" t="s">
+        <v>1384</v>
+      </c>
       <c r="J144">
         <v>6495</v>
       </c>
@@ -13762,6 +14158,9 @@
       <c r="H145" t="s">
         <v>1277</v>
       </c>
+      <c r="I145" t="s">
+        <v>1384</v>
+      </c>
       <c r="J145">
         <v>49164</v>
       </c>
@@ -13887,6 +14286,9 @@
       <c r="H148" t="s">
         <v>1277</v>
       </c>
+      <c r="I148" t="s">
+        <v>1384</v>
+      </c>
       <c r="J148">
         <v>12556</v>
       </c>
@@ -13927,6 +14329,9 @@
       <c r="H149" t="s">
         <v>1277</v>
       </c>
+      <c r="I149" t="s">
+        <v>1384</v>
+      </c>
       <c r="J149">
         <v>12664</v>
       </c>
@@ -13967,6 +14372,9 @@
       <c r="H150" t="s">
         <v>1277</v>
       </c>
+      <c r="I150" t="s">
+        <v>1384</v>
+      </c>
       <c r="J150">
         <v>4578</v>
       </c>
@@ -14006,6 +14414,9 @@
       <c r="H151" t="s">
         <v>1277</v>
       </c>
+      <c r="I151" t="s">
+        <v>1384</v>
+      </c>
       <c r="J151">
         <v>19259</v>
       </c>
@@ -14046,6 +14457,9 @@
       <c r="H152" t="s">
         <v>1277</v>
       </c>
+      <c r="I152" t="s">
+        <v>1384</v>
+      </c>
       <c r="J152">
         <v>9716</v>
       </c>
@@ -14085,6 +14499,9 @@
       <c r="H153" t="s">
         <v>1277</v>
       </c>
+      <c r="I153" t="s">
+        <v>1384</v>
+      </c>
       <c r="J153">
         <v>13166</v>
       </c>
@@ -14125,7 +14542,7 @@
         <v>1278</v>
       </c>
       <c r="I154" t="s">
-        <v>1282</v>
+        <v>1385</v>
       </c>
       <c r="J154">
         <v>13254</v>
@@ -14166,6 +14583,9 @@
       <c r="H155" t="s">
         <v>1277</v>
       </c>
+      <c r="I155" t="s">
+        <v>1384</v>
+      </c>
       <c r="J155">
         <v>98000</v>
       </c>
@@ -14206,6 +14626,9 @@
       <c r="H156" t="s">
         <v>1276</v>
       </c>
+      <c r="I156" t="s">
+        <v>1384</v>
+      </c>
       <c r="J156">
         <v>141323</v>
       </c>
@@ -14246,6 +14669,9 @@
       <c r="H157" t="s">
         <v>1276</v>
       </c>
+      <c r="I157" t="s">
+        <v>1385</v>
+      </c>
       <c r="J157">
         <v>141323</v>
       </c>
@@ -14285,6 +14711,9 @@
       <c r="H158" t="s">
         <v>1277</v>
       </c>
+      <c r="I158" t="s">
+        <v>1384</v>
+      </c>
       <c r="J158">
         <v>96090</v>
       </c>
@@ -14324,6 +14753,9 @@
       <c r="H159" t="s">
         <v>1277</v>
       </c>
+      <c r="I159" t="s">
+        <v>1384</v>
+      </c>
       <c r="J159">
         <v>28820</v>
       </c>
@@ -14364,6 +14796,9 @@
       <c r="H160" t="s">
         <v>1277</v>
       </c>
+      <c r="I160" t="s">
+        <v>1384</v>
+      </c>
       <c r="J160">
         <v>39000</v>
       </c>
@@ -14489,6 +14924,9 @@
       <c r="H163" t="s">
         <v>1277</v>
       </c>
+      <c r="I163" t="s">
+        <v>1384</v>
+      </c>
       <c r="J163">
         <v>9568</v>
       </c>
@@ -14529,6 +14967,9 @@
       <c r="H164" t="s">
         <v>1277</v>
       </c>
+      <c r="I164" t="s">
+        <v>1384</v>
+      </c>
       <c r="J164">
         <v>9671</v>
       </c>
@@ -14569,6 +15010,9 @@
       <c r="H165" t="s">
         <v>1277</v>
       </c>
+      <c r="I165" t="s">
+        <v>1384</v>
+      </c>
       <c r="J165">
         <v>9866</v>
       </c>
@@ -14608,6 +15052,9 @@
       <c r="H166" t="s">
         <v>1277</v>
       </c>
+      <c r="I166" t="s">
+        <v>1384</v>
+      </c>
       <c r="J166">
         <v>9849</v>
       </c>
@@ -14647,6 +15094,9 @@
       <c r="H167" t="s">
         <v>1277</v>
       </c>
+      <c r="I167" t="s">
+        <v>1384</v>
+      </c>
       <c r="J167">
         <v>2932</v>
       </c>
@@ -14686,6 +15136,9 @@
       <c r="H168" t="s">
         <v>1277</v>
       </c>
+      <c r="I168" t="s">
+        <v>1384</v>
+      </c>
       <c r="J168">
         <v>9705</v>
       </c>
@@ -14725,6 +15178,9 @@
       <c r="H169" t="s">
         <v>1277</v>
       </c>
+      <c r="I169" t="s">
+        <v>1384</v>
+      </c>
       <c r="J169">
         <v>9861</v>
       </c>
@@ -14764,6 +15220,9 @@
       <c r="H170" t="s">
         <v>1277</v>
       </c>
+      <c r="I170" t="s">
+        <v>1384</v>
+      </c>
       <c r="J170">
         <v>2943</v>
       </c>
@@ -14803,6 +15262,9 @@
       <c r="H171" t="s">
         <v>1277</v>
       </c>
+      <c r="I171" t="s">
+        <v>1384</v>
+      </c>
       <c r="J171">
         <v>9588</v>
       </c>
@@ -14843,6 +15305,9 @@
       <c r="H172" t="s">
         <v>1277</v>
       </c>
+      <c r="I172" t="s">
+        <v>1384</v>
+      </c>
       <c r="J172">
         <v>9764</v>
       </c>
@@ -14883,6 +15348,9 @@
       <c r="H173" t="s">
         <v>1277</v>
       </c>
+      <c r="I173" t="s">
+        <v>1384</v>
+      </c>
       <c r="J173">
         <v>4890</v>
       </c>
@@ -14922,6 +15390,9 @@
       <c r="H174" t="s">
         <v>1277</v>
       </c>
+      <c r="I174" t="s">
+        <v>1384</v>
+      </c>
       <c r="J174">
         <v>3286</v>
       </c>
@@ -14962,6 +15433,9 @@
       <c r="H175" t="s">
         <v>1277</v>
       </c>
+      <c r="I175" t="s">
+        <v>1384</v>
+      </c>
       <c r="J175">
         <v>9219</v>
       </c>
@@ -15001,6 +15475,9 @@
       <c r="H176" t="s">
         <v>1277</v>
       </c>
+      <c r="I176" t="s">
+        <v>1384</v>
+      </c>
       <c r="J176">
         <v>2000</v>
       </c>
@@ -15040,6 +15517,9 @@
       <c r="H177" t="s">
         <v>1277</v>
       </c>
+      <c r="I177" t="s">
+        <v>1384</v>
+      </c>
       <c r="J177">
         <v>2000</v>
       </c>
@@ -15079,6 +15559,9 @@
       <c r="H178" t="s">
         <v>1277</v>
       </c>
+      <c r="I178" t="s">
+        <v>1384</v>
+      </c>
       <c r="J178">
         <v>2000</v>
       </c>
@@ -15118,6 +15601,9 @@
       <c r="H179" t="s">
         <v>1277</v>
       </c>
+      <c r="I179" t="s">
+        <v>1384</v>
+      </c>
       <c r="J179">
         <v>2000</v>
       </c>
@@ -15157,6 +15643,9 @@
       <c r="H180" t="s">
         <v>1277</v>
       </c>
+      <c r="I180" t="s">
+        <v>1384</v>
+      </c>
       <c r="J180">
         <v>2000</v>
       </c>
@@ -15195,6 +15684,9 @@
       <c r="H181" t="s">
         <v>1277</v>
       </c>
+      <c r="I181" t="s">
+        <v>1384</v>
+      </c>
       <c r="J181">
         <v>2000</v>
       </c>
@@ -15234,6 +15726,9 @@
       <c r="H182" t="s">
         <v>1277</v>
       </c>
+      <c r="I182" t="s">
+        <v>1384</v>
+      </c>
       <c r="J182">
         <v>2000</v>
       </c>
@@ -15273,6 +15768,9 @@
       <c r="H183" t="s">
         <v>1277</v>
       </c>
+      <c r="I183" t="s">
+        <v>1384</v>
+      </c>
       <c r="J183">
         <v>2000</v>
       </c>
@@ -15312,6 +15810,9 @@
       <c r="H184" t="s">
         <v>1277</v>
       </c>
+      <c r="I184" t="s">
+        <v>1384</v>
+      </c>
       <c r="J184">
         <v>2000</v>
       </c>
@@ -15352,6 +15853,9 @@
       <c r="H185" t="s">
         <v>1277</v>
       </c>
+      <c r="I185" t="s">
+        <v>1384</v>
+      </c>
       <c r="J185">
         <v>2000</v>
       </c>
@@ -15392,6 +15896,9 @@
       <c r="H186" t="s">
         <v>1277</v>
       </c>
+      <c r="I186" t="s">
+        <v>1384</v>
+      </c>
       <c r="J186">
         <v>2000</v>
       </c>
@@ -15431,6 +15938,9 @@
       <c r="H187" t="s">
         <v>1277</v>
       </c>
+      <c r="I187" t="s">
+        <v>1384</v>
+      </c>
       <c r="J187">
         <v>2000</v>
       </c>
@@ -15471,6 +15981,9 @@
       <c r="H188" t="s">
         <v>1277</v>
       </c>
+      <c r="I188" t="s">
+        <v>1384</v>
+      </c>
       <c r="J188">
         <v>2000</v>
       </c>
@@ -15510,6 +16023,9 @@
       <c r="H189" t="s">
         <v>1277</v>
       </c>
+      <c r="I189" t="s">
+        <v>1384</v>
+      </c>
       <c r="J189">
         <v>2000</v>
       </c>
@@ -15549,6 +16065,9 @@
       <c r="H190" t="s">
         <v>1277</v>
       </c>
+      <c r="I190" t="s">
+        <v>1384</v>
+      </c>
       <c r="J190">
         <v>2000</v>
       </c>
@@ -15589,6 +16108,9 @@
       <c r="H191" t="s">
         <v>1277</v>
       </c>
+      <c r="I191" t="s">
+        <v>1384</v>
+      </c>
       <c r="J191">
         <v>2000</v>
       </c>
@@ -15628,6 +16150,9 @@
       <c r="H192" t="s">
         <v>1277</v>
       </c>
+      <c r="I192" t="s">
+        <v>1384</v>
+      </c>
       <c r="J192">
         <v>2438</v>
       </c>
@@ -15668,6 +16193,9 @@
       <c r="H193" t="s">
         <v>1277</v>
       </c>
+      <c r="I193" t="s">
+        <v>1384</v>
+      </c>
       <c r="J193">
         <v>2681</v>
       </c>
@@ -15792,6 +16320,9 @@
       <c r="H196" t="s">
         <v>1277</v>
       </c>
+      <c r="I196" t="s">
+        <v>1384</v>
+      </c>
       <c r="J196">
         <v>6966</v>
       </c>
@@ -15831,6 +16362,9 @@
       <c r="H197" t="s">
         <v>1277</v>
       </c>
+      <c r="I197" t="s">
+        <v>1384</v>
+      </c>
       <c r="J197">
         <v>7661</v>
       </c>
@@ -15870,6 +16404,9 @@
       <c r="H198" t="s">
         <v>1277</v>
       </c>
+      <c r="I198" t="s">
+        <v>1385</v>
+      </c>
       <c r="J198">
         <v>7863</v>
       </c>
@@ -15993,6 +16530,9 @@
       <c r="H201" t="s">
         <v>1277</v>
       </c>
+      <c r="I201" t="s">
+        <v>1384</v>
+      </c>
       <c r="J201">
         <v>7386</v>
       </c>
@@ -16033,6 +16573,9 @@
       <c r="H202" t="s">
         <v>1277</v>
       </c>
+      <c r="I202" t="s">
+        <v>1384</v>
+      </c>
       <c r="J202">
         <v>7539</v>
       </c>
@@ -16073,6 +16616,9 @@
       <c r="H203" t="s">
         <v>1277</v>
       </c>
+      <c r="I203" t="s">
+        <v>1384</v>
+      </c>
       <c r="J203">
         <v>15642</v>
       </c>
@@ -16155,6 +16701,9 @@
       <c r="H205" t="s">
         <v>1277</v>
       </c>
+      <c r="I205" t="s">
+        <v>1384</v>
+      </c>
       <c r="J205">
         <v>16832</v>
       </c>
@@ -16195,6 +16744,9 @@
       <c r="H206" t="s">
         <v>1277</v>
       </c>
+      <c r="I206" t="s">
+        <v>1384</v>
+      </c>
       <c r="J206">
         <v>18710</v>
       </c>
@@ -16235,6 +16787,9 @@
       <c r="H207" t="s">
         <v>1277</v>
       </c>
+      <c r="I207" t="s">
+        <v>1384</v>
+      </c>
       <c r="J207">
         <v>19099</v>
       </c>
@@ -16275,6 +16830,9 @@
       <c r="H208" t="s">
         <v>1277</v>
       </c>
+      <c r="I208" t="s">
+        <v>1384</v>
+      </c>
       <c r="J208">
         <v>7821</v>
       </c>
@@ -16358,6 +16916,9 @@
       <c r="H210" t="s">
         <v>1277</v>
       </c>
+      <c r="I210" t="s">
+        <v>1384</v>
+      </c>
       <c r="J210">
         <v>15997</v>
       </c>
@@ -16398,6 +16959,9 @@
       <c r="H211" t="s">
         <v>1277</v>
       </c>
+      <c r="I211" t="s">
+        <v>1384</v>
+      </c>
       <c r="J211">
         <v>15838</v>
       </c>
@@ -16437,6 +17001,9 @@
       <c r="H212" t="s">
         <v>1277</v>
       </c>
+      <c r="I212" t="s">
+        <v>1384</v>
+      </c>
       <c r="J212">
         <v>9355</v>
       </c>
@@ -16476,6 +17043,9 @@
       <c r="H213" t="s">
         <v>1277</v>
       </c>
+      <c r="I213" t="s">
+        <v>1384</v>
+      </c>
       <c r="J213">
         <v>9549</v>
       </c>
@@ -16516,6 +17086,9 @@
       <c r="H214" t="s">
         <v>1277</v>
       </c>
+      <c r="I214" t="s">
+        <v>1384</v>
+      </c>
       <c r="J214">
         <v>4500</v>
       </c>
@@ -16555,6 +17128,9 @@
       <c r="H215" t="s">
         <v>1277</v>
       </c>
+      <c r="I215" t="s">
+        <v>1384</v>
+      </c>
       <c r="J215">
         <v>4500</v>
       </c>
@@ -16594,6 +17170,9 @@
       <c r="H216" t="s">
         <v>1277</v>
       </c>
+      <c r="I216" t="s">
+        <v>1384</v>
+      </c>
       <c r="J216">
         <v>4698</v>
       </c>
@@ -16634,6 +17213,9 @@
       <c r="H217" t="s">
         <v>1277</v>
       </c>
+      <c r="I217" t="s">
+        <v>1384</v>
+      </c>
       <c r="J217">
         <v>4052</v>
       </c>
@@ -16674,6 +17256,9 @@
       <c r="H218" t="s">
         <v>1277</v>
       </c>
+      <c r="I218" t="s">
+        <v>1384</v>
+      </c>
       <c r="J218">
         <v>4078</v>
       </c>
@@ -16714,6 +17299,9 @@
       <c r="H219" t="s">
         <v>1277</v>
       </c>
+      <c r="I219" t="s">
+        <v>1384</v>
+      </c>
       <c r="J219">
         <v>3985</v>
       </c>
@@ -16796,6 +17384,9 @@
       <c r="H221" t="s">
         <v>1277</v>
       </c>
+      <c r="I221" t="s">
+        <v>1385</v>
+      </c>
       <c r="J221">
         <v>1495</v>
       </c>
@@ -16835,6 +17426,9 @@
       <c r="H222" t="s">
         <v>1277</v>
       </c>
+      <c r="I222" t="s">
+        <v>1385</v>
+      </c>
       <c r="J222">
         <v>1420</v>
       </c>
@@ -16874,6 +17468,9 @@
       <c r="H223" t="s">
         <v>1277</v>
       </c>
+      <c r="I223" t="s">
+        <v>1384</v>
+      </c>
       <c r="J223">
         <v>27600</v>
       </c>
@@ -16914,6 +17511,9 @@
       <c r="H224" t="s">
         <v>1277</v>
       </c>
+      <c r="I224" t="s">
+        <v>1384</v>
+      </c>
       <c r="J224">
         <v>27600</v>
       </c>
@@ -16953,6 +17553,9 @@
       <c r="H225" t="s">
         <v>1277</v>
       </c>
+      <c r="I225" t="s">
+        <v>1384</v>
+      </c>
       <c r="J225">
         <v>646</v>
       </c>
@@ -16992,6 +17595,9 @@
       <c r="H226" t="s">
         <v>1277</v>
       </c>
+      <c r="I226" t="s">
+        <v>1384</v>
+      </c>
       <c r="J226">
         <v>629</v>
       </c>
@@ -17030,6 +17636,9 @@
       <c r="H227" t="s">
         <v>1277</v>
       </c>
+      <c r="I227" t="s">
+        <v>1384</v>
+      </c>
       <c r="J227">
         <v>6468</v>
       </c>
@@ -17069,6 +17678,9 @@
       <c r="H228" t="s">
         <v>1277</v>
       </c>
+      <c r="I228" t="s">
+        <v>1384</v>
+      </c>
       <c r="J228">
         <v>6291</v>
       </c>
@@ -17108,6 +17720,9 @@
       <c r="H229" t="s">
         <v>1277</v>
       </c>
+      <c r="I229" t="s">
+        <v>1384</v>
+      </c>
       <c r="J229">
         <v>1021</v>
       </c>
@@ -17148,6 +17763,9 @@
       <c r="H230" t="s">
         <v>1277</v>
       </c>
+      <c r="I230" t="s">
+        <v>1384</v>
+      </c>
       <c r="J230">
         <v>1014</v>
       </c>
@@ -17188,6 +17806,9 @@
       <c r="H231" t="s">
         <v>1277</v>
       </c>
+      <c r="I231" t="s">
+        <v>1384</v>
+      </c>
       <c r="J231">
         <v>1023</v>
       </c>
@@ -17227,6 +17848,9 @@
       <c r="H232" t="s">
         <v>1277</v>
       </c>
+      <c r="I232" t="s">
+        <v>1384</v>
+      </c>
       <c r="J232">
         <v>5989</v>
       </c>
@@ -17266,6 +17890,9 @@
       <c r="H233" t="s">
         <v>1277</v>
       </c>
+      <c r="I233" t="s">
+        <v>1384</v>
+      </c>
       <c r="J233">
         <v>5944</v>
       </c>
@@ -17304,6 +17931,9 @@
       <c r="H234" t="s">
         <v>1277</v>
       </c>
+      <c r="I234" t="s">
+        <v>1384</v>
+      </c>
       <c r="J234">
         <v>2738</v>
       </c>
@@ -17342,6 +17972,9 @@
       <c r="H235" t="s">
         <v>1277</v>
       </c>
+      <c r="I235" t="s">
+        <v>1384</v>
+      </c>
       <c r="J235">
         <v>2717</v>
       </c>
@@ -17381,6 +18014,9 @@
       <c r="H236" t="s">
         <v>1277</v>
       </c>
+      <c r="I236" t="s">
+        <v>1385</v>
+      </c>
       <c r="J236">
         <v>12250</v>
       </c>
@@ -17420,6 +18056,9 @@
       <c r="H237" t="s">
         <v>1277</v>
       </c>
+      <c r="I237" t="s">
+        <v>1385</v>
+      </c>
       <c r="J237">
         <v>12250</v>
       </c>
@@ -17459,6 +18098,9 @@
       <c r="H238" t="s">
         <v>1277</v>
       </c>
+      <c r="I238" t="s">
+        <v>1385</v>
+      </c>
       <c r="J238">
         <v>12250</v>
       </c>
@@ -17497,6 +18139,9 @@
       <c r="H239" t="s">
         <v>1277</v>
       </c>
+      <c r="I239" t="s">
+        <v>1385</v>
+      </c>
       <c r="J239">
         <v>12250</v>
       </c>
@@ -17579,6 +18224,9 @@
       <c r="H241" t="s">
         <v>1277</v>
       </c>
+      <c r="I241" t="s">
+        <v>1384</v>
+      </c>
       <c r="J241">
         <v>19128</v>
       </c>
@@ -17619,6 +18267,9 @@
       <c r="H242" t="s">
         <v>1277</v>
       </c>
+      <c r="I242" t="s">
+        <v>1384</v>
+      </c>
       <c r="J242">
         <v>21833</v>
       </c>
@@ -17659,6 +18310,9 @@
       <c r="H243" t="s">
         <v>1277</v>
       </c>
+      <c r="I243" t="s">
+        <v>1384</v>
+      </c>
       <c r="J243">
         <v>21289</v>
       </c>
@@ -17699,6 +18353,9 @@
       <c r="H244" t="s">
         <v>1277</v>
       </c>
+      <c r="I244" t="s">
+        <v>1384</v>
+      </c>
       <c r="J244">
         <v>21781</v>
       </c>
@@ -17739,6 +18396,9 @@
       <c r="H245" t="s">
         <v>1277</v>
       </c>
+      <c r="I245" t="s">
+        <v>1384</v>
+      </c>
       <c r="J245">
         <v>8092</v>
       </c>
@@ -17779,6 +18439,9 @@
       <c r="H246" t="s">
         <v>1277</v>
       </c>
+      <c r="I246" t="s">
+        <v>1385</v>
+      </c>
       <c r="J246">
         <v>7245</v>
       </c>
@@ -17818,6 +18481,9 @@
       <c r="H247" t="s">
         <v>1277</v>
       </c>
+      <c r="I247" t="s">
+        <v>1384</v>
+      </c>
       <c r="J247">
         <v>7482</v>
       </c>
@@ -17900,6 +18566,9 @@
       <c r="H249" t="s">
         <v>1277</v>
       </c>
+      <c r="I249" t="s">
+        <v>1384</v>
+      </c>
       <c r="J249">
         <v>13308</v>
       </c>
@@ -17940,6 +18609,9 @@
       <c r="H250" t="s">
         <v>1277</v>
       </c>
+      <c r="I250" t="s">
+        <v>1384</v>
+      </c>
       <c r="J250">
         <v>16072</v>
       </c>
@@ -17980,6 +18652,9 @@
       <c r="H251" t="s">
         <v>1277</v>
       </c>
+      <c r="I251" t="s">
+        <v>1384</v>
+      </c>
       <c r="J251">
         <v>13857</v>
       </c>
@@ -18020,6 +18695,9 @@
       <c r="H252" t="s">
         <v>1277</v>
       </c>
+      <c r="I252" t="s">
+        <v>1384</v>
+      </c>
       <c r="J252">
         <v>17082</v>
       </c>
@@ -18059,6 +18737,9 @@
       <c r="H253" t="s">
         <v>1277</v>
       </c>
+      <c r="I253" t="s">
+        <v>1384</v>
+      </c>
       <c r="J253">
         <v>15974</v>
       </c>
@@ -18099,6 +18780,9 @@
       <c r="H254" t="s">
         <v>1277</v>
       </c>
+      <c r="I254" t="s">
+        <v>1384</v>
+      </c>
       <c r="J254">
         <v>17250</v>
       </c>
@@ -18139,6 +18823,9 @@
       <c r="H255" t="s">
         <v>1277</v>
       </c>
+      <c r="I255" t="s">
+        <v>1384</v>
+      </c>
       <c r="J255">
         <v>10249</v>
       </c>
@@ -18177,6 +18864,9 @@
       <c r="H256" t="s">
         <v>1277</v>
       </c>
+      <c r="I256" t="s">
+        <v>1384</v>
+      </c>
       <c r="J256">
         <v>9477</v>
       </c>
@@ -18216,6 +18906,9 @@
       <c r="H257" t="s">
         <v>1277</v>
       </c>
+      <c r="I257" t="s">
+        <v>1384</v>
+      </c>
       <c r="J257">
         <v>10290</v>
       </c>
@@ -18255,6 +18948,9 @@
       <c r="H258" t="s">
         <v>1277</v>
       </c>
+      <c r="I258" t="s">
+        <v>1384</v>
+      </c>
       <c r="J258">
         <v>7985</v>
       </c>
@@ -18294,6 +18990,9 @@
       <c r="H259" t="s">
         <v>1277</v>
       </c>
+      <c r="I259" t="s">
+        <v>1384</v>
+      </c>
       <c r="J259">
         <v>9643</v>
       </c>
@@ -18334,6 +19033,9 @@
       <c r="H260" t="s">
         <v>1277</v>
       </c>
+      <c r="I260" t="s">
+        <v>1384</v>
+      </c>
       <c r="J260">
         <v>9177</v>
       </c>
@@ -18373,6 +19075,9 @@
       <c r="H261" t="s">
         <v>1277</v>
       </c>
+      <c r="I261" t="s">
+        <v>1384</v>
+      </c>
       <c r="J261">
         <v>10407</v>
       </c>
@@ -18413,6 +19118,9 @@
       <c r="H262" t="s">
         <v>1277</v>
       </c>
+      <c r="I262" t="s">
+        <v>1384</v>
+      </c>
       <c r="J262">
         <v>8314</v>
       </c>
@@ -18452,6 +19160,9 @@
       <c r="H263" t="s">
         <v>1277</v>
       </c>
+      <c r="I263" t="s">
+        <v>1385</v>
+      </c>
       <c r="J263">
         <v>8243</v>
       </c>
@@ -18491,6 +19202,9 @@
       <c r="H264" t="s">
         <v>1277</v>
       </c>
+      <c r="I264" t="s">
+        <v>1385</v>
+      </c>
       <c r="J264">
         <v>17630</v>
       </c>
@@ -18530,6 +19244,9 @@
       <c r="H265" t="s">
         <v>1277</v>
       </c>
+      <c r="I265" t="s">
+        <v>1384</v>
+      </c>
       <c r="J265">
         <v>1</v>
       </c>
@@ -18570,6 +19287,9 @@
       <c r="H266" t="s">
         <v>1277</v>
       </c>
+      <c r="I266" t="s">
+        <v>1384</v>
+      </c>
       <c r="J266">
         <v>4588</v>
       </c>
@@ -18610,6 +19330,9 @@
       <c r="H267" t="s">
         <v>1277</v>
       </c>
+      <c r="I267" t="s">
+        <v>1384</v>
+      </c>
       <c r="J267">
         <v>5494</v>
       </c>
@@ -18650,6 +19373,9 @@
       <c r="H268" t="s">
         <v>1277</v>
       </c>
+      <c r="I268" t="s">
+        <v>1384</v>
+      </c>
       <c r="J268">
         <v>910</v>
       </c>
@@ -18689,6 +19415,9 @@
       <c r="H269" t="s">
         <v>1277</v>
       </c>
+      <c r="I269" t="s">
+        <v>1384</v>
+      </c>
       <c r="J269">
         <v>4586</v>
       </c>
@@ -18729,6 +19458,9 @@
       <c r="H270" t="s">
         <v>1277</v>
       </c>
+      <c r="I270" t="s">
+        <v>1384</v>
+      </c>
       <c r="J270">
         <v>5494</v>
       </c>
@@ -18769,6 +19501,9 @@
       <c r="H271" t="s">
         <v>1277</v>
       </c>
+      <c r="I271" t="s">
+        <v>1384</v>
+      </c>
       <c r="J271">
         <v>922</v>
       </c>
@@ -18809,6 +19544,9 @@
       <c r="H272" t="s">
         <v>1277</v>
       </c>
+      <c r="I272" t="s">
+        <v>1384</v>
+      </c>
       <c r="J272">
         <v>1</v>
       </c>
@@ -18848,6 +19586,9 @@
       <c r="H273" t="s">
         <v>1277</v>
       </c>
+      <c r="I273" t="s">
+        <v>1384</v>
+      </c>
       <c r="J273">
         <v>2648</v>
       </c>
@@ -18888,6 +19629,9 @@
       <c r="H274" t="s">
         <v>1277</v>
       </c>
+      <c r="I274" t="s">
+        <v>1384</v>
+      </c>
       <c r="J274">
         <v>2648</v>
       </c>
@@ -18927,6 +19671,9 @@
       <c r="H275" t="s">
         <v>1277</v>
       </c>
+      <c r="I275" t="s">
+        <v>1384</v>
+      </c>
       <c r="J275">
         <v>2648</v>
       </c>
@@ -18966,6 +19713,9 @@
       <c r="H276" t="s">
         <v>1277</v>
       </c>
+      <c r="I276" t="s">
+        <v>1384</v>
+      </c>
       <c r="J276">
         <v>2663</v>
       </c>
@@ -19006,6 +19756,9 @@
       <c r="H277" t="s">
         <v>1277</v>
       </c>
+      <c r="I277" t="s">
+        <v>1384</v>
+      </c>
       <c r="J277">
         <v>2648</v>
       </c>
@@ -19046,6 +19799,9 @@
       <c r="H278" t="s">
         <v>1277</v>
       </c>
+      <c r="I278" t="s">
+        <v>1384</v>
+      </c>
       <c r="J278">
         <v>2648</v>
       </c>
@@ -19086,6 +19842,9 @@
       <c r="H279" t="s">
         <v>1277</v>
       </c>
+      <c r="I279" t="s">
+        <v>1384</v>
+      </c>
       <c r="J279">
         <v>2648</v>
       </c>
@@ -19126,6 +19885,9 @@
       <c r="H280" t="s">
         <v>1277</v>
       </c>
+      <c r="I280" t="s">
+        <v>1384</v>
+      </c>
       <c r="J280">
         <v>2656</v>
       </c>
@@ -19166,6 +19928,9 @@
       <c r="H281" t="s">
         <v>1277</v>
       </c>
+      <c r="I281" t="s">
+        <v>1384</v>
+      </c>
       <c r="J281">
         <v>2679</v>
       </c>
@@ -19292,6 +20057,9 @@
       <c r="H284" t="s">
         <v>1276</v>
       </c>
+      <c r="I284" t="s">
+        <v>1384</v>
+      </c>
       <c r="J284">
         <v>3170</v>
       </c>
@@ -19331,6 +20099,9 @@
       <c r="H285" t="s">
         <v>1277</v>
       </c>
+      <c r="I285" t="s">
+        <v>1384</v>
+      </c>
       <c r="J285">
         <v>3070</v>
       </c>
@@ -19371,6 +20142,9 @@
       <c r="H286" t="s">
         <v>1277</v>
       </c>
+      <c r="I286" t="s">
+        <v>1384</v>
+      </c>
       <c r="J286">
         <v>3066</v>
       </c>
@@ -19411,6 +20185,9 @@
       <c r="H287" t="s">
         <v>1276</v>
       </c>
+      <c r="I287" t="s">
+        <v>1384</v>
+      </c>
       <c r="J287">
         <v>793</v>
       </c>
@@ -19451,6 +20228,9 @@
       <c r="H288" t="s">
         <v>1276</v>
       </c>
+      <c r="I288" t="s">
+        <v>1384</v>
+      </c>
       <c r="J288">
         <v>3170</v>
       </c>
@@ -19491,6 +20271,9 @@
       <c r="H289" t="s">
         <v>1276</v>
       </c>
+      <c r="I289" t="s">
+        <v>1384</v>
+      </c>
       <c r="J289">
         <v>3170</v>
       </c>
@@ -19530,6 +20313,9 @@
       <c r="H290" t="s">
         <v>1276</v>
       </c>
+      <c r="I290" t="s">
+        <v>1384</v>
+      </c>
       <c r="J290">
         <v>1981</v>
       </c>
@@ -19570,6 +20356,9 @@
       <c r="H291" t="s">
         <v>1277</v>
       </c>
+      <c r="I291" t="s">
+        <v>1384</v>
+      </c>
       <c r="J291">
         <v>1919</v>
       </c>
@@ -19609,6 +20398,9 @@
       <c r="H292" t="s">
         <v>1277</v>
       </c>
+      <c r="I292" t="s">
+        <v>1385</v>
+      </c>
       <c r="J292">
         <v>1920</v>
       </c>
@@ -19648,6 +20440,9 @@
       <c r="H293" t="s">
         <v>1277</v>
       </c>
+      <c r="I293" t="s">
+        <v>1385</v>
+      </c>
       <c r="J293">
         <v>1920</v>
       </c>
@@ -19730,6 +20525,9 @@
       <c r="H295" t="s">
         <v>1277</v>
       </c>
+      <c r="I295" t="s">
+        <v>1385</v>
+      </c>
       <c r="J295">
         <v>2937</v>
       </c>
@@ -19769,6 +20567,9 @@
       <c r="H296" t="s">
         <v>1277</v>
       </c>
+      <c r="I296" t="s">
+        <v>1385</v>
+      </c>
       <c r="J296">
         <v>734</v>
       </c>
@@ -19808,6 +20609,9 @@
       <c r="H297" t="s">
         <v>1277</v>
       </c>
+      <c r="I297" t="s">
+        <v>1384</v>
+      </c>
       <c r="J297">
         <v>2959</v>
       </c>
@@ -19848,6 +20652,9 @@
       <c r="H298" t="s">
         <v>1277</v>
       </c>
+      <c r="I298" t="s">
+        <v>1385</v>
+      </c>
       <c r="J298">
         <v>3980</v>
       </c>
@@ -20057,6 +20864,9 @@
       <c r="H303" t="s">
         <v>1277</v>
       </c>
+      <c r="I303" t="s">
+        <v>1384</v>
+      </c>
       <c r="J303">
         <v>2614</v>
       </c>
@@ -20097,6 +20907,9 @@
       <c r="H304" t="s">
         <v>1277</v>
       </c>
+      <c r="I304" t="s">
+        <v>1384</v>
+      </c>
       <c r="J304">
         <v>2612</v>
       </c>
@@ -20137,6 +20950,9 @@
       <c r="H305" t="s">
         <v>1277</v>
       </c>
+      <c r="I305" t="s">
+        <v>1384</v>
+      </c>
       <c r="J305">
         <v>2492</v>
       </c>
@@ -20177,6 +20993,9 @@
       <c r="H306" t="s">
         <v>1277</v>
       </c>
+      <c r="I306" t="s">
+        <v>1384</v>
+      </c>
       <c r="J306">
         <v>2614</v>
       </c>
@@ -20216,6 +21035,9 @@
       <c r="H307" t="s">
         <v>1279</v>
       </c>
+      <c r="I307" t="s">
+        <v>1384</v>
+      </c>
       <c r="J307">
         <v>316</v>
       </c>
@@ -20256,6 +21078,9 @@
       <c r="H308" t="s">
         <v>1279</v>
       </c>
+      <c r="I308" t="s">
+        <v>1384</v>
+      </c>
       <c r="J308">
         <v>313</v>
       </c>
@@ -20296,6 +21121,9 @@
       <c r="H309" t="s">
         <v>1279</v>
       </c>
+      <c r="I309" t="s">
+        <v>1384</v>
+      </c>
       <c r="J309">
         <v>313</v>
       </c>
@@ -20336,6 +21164,9 @@
       <c r="H310" t="s">
         <v>1279</v>
       </c>
+      <c r="I310" t="s">
+        <v>1384</v>
+      </c>
       <c r="J310">
         <v>310</v>
       </c>
@@ -20376,6 +21207,9 @@
       <c r="H311" t="s">
         <v>1279</v>
       </c>
+      <c r="I311" t="s">
+        <v>1384</v>
+      </c>
       <c r="J311">
         <v>304</v>
       </c>
@@ -20416,6 +21250,9 @@
       <c r="H312" t="s">
         <v>1277</v>
       </c>
+      <c r="I312" t="s">
+        <v>1384</v>
+      </c>
       <c r="J312">
         <v>6650</v>
       </c>
@@ -20456,6 +21293,9 @@
       <c r="H313" t="s">
         <v>1277</v>
       </c>
+      <c r="I313" t="s">
+        <v>1384</v>
+      </c>
       <c r="J313">
         <v>6650</v>
       </c>
@@ -20496,6 +21336,9 @@
       <c r="H314" t="s">
         <v>1277</v>
       </c>
+      <c r="I314" t="s">
+        <v>1384</v>
+      </c>
       <c r="J314">
         <v>6773</v>
       </c>
@@ -20578,6 +21421,9 @@
       <c r="H316" t="s">
         <v>1277</v>
       </c>
+      <c r="I316" t="s">
+        <v>1384</v>
+      </c>
       <c r="J316">
         <v>3014</v>
       </c>
@@ -20618,6 +21464,9 @@
       <c r="H317" t="s">
         <v>1277</v>
       </c>
+      <c r="I317" t="s">
+        <v>1384</v>
+      </c>
       <c r="J317">
         <v>6883</v>
       </c>
@@ -20658,6 +21507,9 @@
       <c r="H318" t="s">
         <v>1277</v>
       </c>
+      <c r="I318" t="s">
+        <v>1384</v>
+      </c>
       <c r="J318">
         <v>6680</v>
       </c>
@@ -20698,6 +21550,9 @@
       <c r="H319" t="s">
         <v>1277</v>
       </c>
+      <c r="I319" t="s">
+        <v>1384</v>
+      </c>
       <c r="J319">
         <v>1634</v>
       </c>
@@ -20738,6 +21593,9 @@
       <c r="H320" t="s">
         <v>1277</v>
       </c>
+      <c r="I320" t="s">
+        <v>1385</v>
+      </c>
       <c r="J320">
         <v>2867</v>
       </c>
@@ -20778,6 +21636,9 @@
       <c r="H321" t="s">
         <v>1277</v>
       </c>
+      <c r="I321" t="s">
+        <v>1385</v>
+      </c>
       <c r="J321">
         <v>3035</v>
       </c>
@@ -20817,6 +21678,9 @@
       <c r="H322" t="s">
         <v>1277</v>
       </c>
+      <c r="I322" t="s">
+        <v>1384</v>
+      </c>
       <c r="J322">
         <v>3021</v>
       </c>
@@ -20857,6 +21721,9 @@
       <c r="H323" t="s">
         <v>1277</v>
       </c>
+      <c r="I323" t="s">
+        <v>1385</v>
+      </c>
       <c r="J323">
         <v>2758</v>
       </c>
@@ -20938,6 +21805,9 @@
       <c r="H325" t="s">
         <v>1277</v>
       </c>
+      <c r="I325" t="s">
+        <v>1384</v>
+      </c>
       <c r="J325">
         <v>8031</v>
       </c>
@@ -20978,6 +21848,9 @@
       <c r="H326" t="s">
         <v>1277</v>
       </c>
+      <c r="I326" t="s">
+        <v>1384</v>
+      </c>
       <c r="J326">
         <v>8010</v>
       </c>
@@ -21060,6 +21933,9 @@
       <c r="H328" t="s">
         <v>1277</v>
       </c>
+      <c r="I328" t="s">
+        <v>1385</v>
+      </c>
       <c r="J328">
         <v>19</v>
       </c>
@@ -21185,6 +22061,9 @@
       <c r="H331" t="s">
         <v>1280</v>
       </c>
+      <c r="I331" t="s">
+        <v>1385</v>
+      </c>
       <c r="J331">
         <v>19</v>
       </c>
@@ -21224,6 +22103,9 @@
       <c r="H332" t="s">
         <v>1280</v>
       </c>
+      <c r="I332" t="s">
+        <v>1384</v>
+      </c>
       <c r="J332">
         <v>781</v>
       </c>
@@ -21263,6 +22145,9 @@
       <c r="H333" t="s">
         <v>1280</v>
       </c>
+      <c r="I333" t="s">
+        <v>1384</v>
+      </c>
       <c r="J333">
         <v>300</v>
       </c>
@@ -21386,6 +22271,9 @@
       <c r="H336" t="s">
         <v>1280</v>
       </c>
+      <c r="I336" t="s">
+        <v>1384</v>
+      </c>
       <c r="J336">
         <v>1932</v>
       </c>
@@ -21425,6 +22313,9 @@
       <c r="H337" t="s">
         <v>1280</v>
       </c>
+      <c r="I337" t="s">
+        <v>1384</v>
+      </c>
       <c r="J337">
         <v>3000</v>
       </c>
@@ -21465,6 +22356,9 @@
       <c r="H338" t="s">
         <v>1280</v>
       </c>
+      <c r="I338" t="s">
+        <v>1384</v>
+      </c>
       <c r="J338">
         <v>1896</v>
       </c>
@@ -21505,6 +22399,9 @@
       <c r="H339" t="s">
         <v>1280</v>
       </c>
+      <c r="I339" t="s">
+        <v>1384</v>
+      </c>
       <c r="J339">
         <v>16012</v>
       </c>
@@ -21544,6 +22441,9 @@
       <c r="H340" t="s">
         <v>1280</v>
       </c>
+      <c r="I340" t="s">
+        <v>1384</v>
+      </c>
       <c r="J340">
         <v>1253</v>
       </c>
@@ -21626,6 +22526,9 @@
       <c r="H342" t="s">
         <v>1280</v>
       </c>
+      <c r="I342" t="s">
+        <v>1384</v>
+      </c>
       <c r="J342">
         <v>4200</v>
       </c>
@@ -21708,6 +22611,9 @@
       <c r="H344" t="s">
         <v>1280</v>
       </c>
+      <c r="I344" t="s">
+        <v>1384</v>
+      </c>
       <c r="J344">
         <v>726</v>
       </c>
@@ -21747,6 +22653,9 @@
       <c r="H345" t="s">
         <v>1280</v>
       </c>
+      <c r="I345" t="s">
+        <v>1384</v>
+      </c>
       <c r="J345">
         <v>4114</v>
       </c>
@@ -21786,6 +22695,9 @@
       <c r="H346" t="s">
         <v>1280</v>
       </c>
+      <c r="I346" t="s">
+        <v>1384</v>
+      </c>
       <c r="J346">
         <v>4700</v>
       </c>
@@ -21826,6 +22738,9 @@
       <c r="H347" t="s">
         <v>1280</v>
       </c>
+      <c r="I347" t="s">
+        <v>1384</v>
+      </c>
       <c r="J347">
         <v>9398</v>
       </c>
@@ -21864,6 +22779,9 @@
       <c r="H348" t="s">
         <v>1280</v>
       </c>
+      <c r="I348" t="s">
+        <v>1384</v>
+      </c>
       <c r="J348">
         <v>6400</v>
       </c>
@@ -21946,6 +22864,9 @@
       <c r="H350" t="s">
         <v>1280</v>
       </c>
+      <c r="I350" t="s">
+        <v>1384</v>
+      </c>
       <c r="J350">
         <v>1213</v>
       </c>
@@ -21985,6 +22906,9 @@
       <c r="H351" t="s">
         <v>1280</v>
       </c>
+      <c r="I351" t="s">
+        <v>1384</v>
+      </c>
       <c r="J351">
         <v>2941</v>
       </c>
@@ -22024,6 +22948,9 @@
       <c r="H352" t="s">
         <v>1280</v>
       </c>
+      <c r="I352" t="s">
+        <v>1384</v>
+      </c>
       <c r="J352">
         <v>426</v>
       </c>
@@ -22064,6 +22991,9 @@
       <c r="H353" t="s">
         <v>1280</v>
       </c>
+      <c r="I353" t="s">
+        <v>1384</v>
+      </c>
       <c r="J353">
         <v>1056</v>
       </c>
@@ -22103,6 +23033,9 @@
       <c r="H354" t="s">
         <v>1280</v>
       </c>
+      <c r="I354" t="s">
+        <v>1384</v>
+      </c>
       <c r="J354">
         <v>1530</v>
       </c>
@@ -22184,6 +23117,9 @@
       <c r="H356" t="s">
         <v>1280</v>
       </c>
+      <c r="I356" t="s">
+        <v>1384</v>
+      </c>
       <c r="J356">
         <v>1044</v>
       </c>
@@ -22223,6 +23159,9 @@
       <c r="H357" t="s">
         <v>1280</v>
       </c>
+      <c r="I357" t="s">
+        <v>1384</v>
+      </c>
       <c r="J357">
         <v>2317</v>
       </c>
@@ -22262,6 +23201,9 @@
       <c r="H358" t="s">
         <v>1280</v>
       </c>
+      <c r="I358" t="s">
+        <v>1384</v>
+      </c>
       <c r="J358">
         <v>4000</v>
       </c>
@@ -22472,6 +23414,9 @@
       <c r="H363" t="s">
         <v>1280</v>
       </c>
+      <c r="I363" t="s">
+        <v>1385</v>
+      </c>
       <c r="J363">
         <v>862</v>
       </c>
@@ -22511,6 +23456,9 @@
       <c r="H364" t="s">
         <v>1280</v>
       </c>
+      <c r="I364" t="s">
+        <v>1385</v>
+      </c>
       <c r="J364">
         <v>861</v>
       </c>
@@ -22550,6 +23498,9 @@
       <c r="H365" t="s">
         <v>1280</v>
       </c>
+      <c r="I365" t="s">
+        <v>1384</v>
+      </c>
       <c r="J365">
         <v>1951</v>
       </c>
@@ -22717,6 +23668,9 @@
       <c r="H369" t="s">
         <v>1280</v>
       </c>
+      <c r="I369" t="s">
+        <v>1384</v>
+      </c>
       <c r="J369">
         <v>4847</v>
       </c>
@@ -22756,6 +23710,9 @@
       <c r="H370" t="s">
         <v>1280</v>
       </c>
+      <c r="I370" t="s">
+        <v>1385</v>
+      </c>
       <c r="J370">
         <v>2900</v>
       </c>
@@ -22795,6 +23752,9 @@
       <c r="H371" t="s">
         <v>1280</v>
       </c>
+      <c r="I371" t="s">
+        <v>1384</v>
+      </c>
       <c r="J371">
         <v>4167</v>
       </c>
@@ -22835,6 +23795,9 @@
       <c r="H372" t="s">
         <v>1280</v>
       </c>
+      <c r="I372" t="s">
+        <v>1384</v>
+      </c>
       <c r="J372">
         <v>18845</v>
       </c>
@@ -22874,6 +23837,9 @@
       <c r="H373" t="s">
         <v>1280</v>
       </c>
+      <c r="I373" t="s">
+        <v>1384</v>
+      </c>
       <c r="J373">
         <v>3225</v>
       </c>
@@ -22913,6 +23879,9 @@
       <c r="H374" t="s">
         <v>1280</v>
       </c>
+      <c r="I374" t="s">
+        <v>1384</v>
+      </c>
       <c r="J374">
         <v>4181</v>
       </c>
@@ -22952,6 +23921,9 @@
       <c r="H375" t="s">
         <v>1280</v>
       </c>
+      <c r="I375" t="s">
+        <v>1384</v>
+      </c>
       <c r="J375">
         <v>647</v>
       </c>
@@ -22991,6 +23963,9 @@
       <c r="H376" t="s">
         <v>1280</v>
       </c>
+      <c r="I376" t="s">
+        <v>1384</v>
+      </c>
       <c r="J376">
         <v>5261</v>
       </c>
@@ -23030,6 +24005,9 @@
       <c r="H377" t="s">
         <v>1280</v>
       </c>
+      <c r="I377" t="s">
+        <v>1384</v>
+      </c>
       <c r="J377">
         <v>478</v>
       </c>
@@ -23070,6 +24048,9 @@
       <c r="H378" t="s">
         <v>1280</v>
       </c>
+      <c r="I378" t="s">
+        <v>1384</v>
+      </c>
       <c r="J378">
         <v>6408</v>
       </c>
@@ -23110,6 +24091,9 @@
       <c r="H379" t="s">
         <v>1280</v>
       </c>
+      <c r="I379" t="s">
+        <v>1384</v>
+      </c>
       <c r="J379">
         <v>4120</v>
       </c>
@@ -23149,6 +24133,9 @@
       <c r="H380" t="s">
         <v>1280</v>
       </c>
+      <c r="I380" t="s">
+        <v>1384</v>
+      </c>
       <c r="J380">
         <v>3360</v>
       </c>
@@ -23231,6 +24218,9 @@
       <c r="H382" t="s">
         <v>1280</v>
       </c>
+      <c r="I382" t="s">
+        <v>1384</v>
+      </c>
       <c r="J382">
         <v>1839</v>
       </c>
@@ -23270,6 +24260,9 @@
       <c r="H383" t="s">
         <v>1280</v>
       </c>
+      <c r="I383" t="s">
+        <v>1384</v>
+      </c>
       <c r="J383">
         <v>2484</v>
       </c>
@@ -23310,6 +24303,9 @@
       <c r="H384" t="s">
         <v>1280</v>
       </c>
+      <c r="I384" t="s">
+        <v>1384</v>
+      </c>
       <c r="J384">
         <v>3152</v>
       </c>
@@ -23350,6 +24346,9 @@
       <c r="H385" t="s">
         <v>1280</v>
       </c>
+      <c r="I385" t="s">
+        <v>1384</v>
+      </c>
       <c r="J385">
         <v>3135</v>
       </c>
@@ -23389,6 +24388,9 @@
       <c r="H386" t="s">
         <v>1280</v>
       </c>
+      <c r="I386" t="s">
+        <v>1384</v>
+      </c>
       <c r="J386">
         <v>3653</v>
       </c>
@@ -23428,6 +24430,9 @@
       <c r="H387" t="s">
         <v>1280</v>
       </c>
+      <c r="I387" t="s">
+        <v>1384</v>
+      </c>
       <c r="J387">
         <v>4733</v>
       </c>
@@ -23467,6 +24472,9 @@
       <c r="H388" t="s">
         <v>1280</v>
       </c>
+      <c r="I388" t="s">
+        <v>1384</v>
+      </c>
       <c r="J388">
         <v>1587</v>
       </c>
@@ -23506,6 +24514,9 @@
       <c r="H389" t="s">
         <v>1280</v>
       </c>
+      <c r="I389" t="s">
+        <v>1384</v>
+      </c>
       <c r="J389">
         <v>3285</v>
       </c>
@@ -23545,6 +24556,9 @@
       <c r="H390" t="s">
         <v>1280</v>
       </c>
+      <c r="I390" t="s">
+        <v>1384</v>
+      </c>
       <c r="J390">
         <v>3700</v>
       </c>
@@ -23584,6 +24598,9 @@
       <c r="H391" t="s">
         <v>1280</v>
       </c>
+      <c r="I391" t="s">
+        <v>1385</v>
+      </c>
       <c r="J391">
         <v>6800</v>
       </c>
@@ -23624,6 +24641,9 @@
       <c r="H392" t="s">
         <v>1280</v>
       </c>
+      <c r="I392" t="s">
+        <v>1385</v>
+      </c>
       <c r="J392">
         <v>545</v>
       </c>
@@ -23663,6 +24683,9 @@
       <c r="H393" t="s">
         <v>1280</v>
       </c>
+      <c r="I393" t="s">
+        <v>1384</v>
+      </c>
       <c r="J393">
         <v>9571</v>
       </c>
@@ -23702,6 +24725,9 @@
       <c r="H394" t="s">
         <v>1280</v>
       </c>
+      <c r="I394" t="s">
+        <v>1384</v>
+      </c>
       <c r="J394">
         <v>676</v>
       </c>
@@ -23742,6 +24768,9 @@
       <c r="H395" t="s">
         <v>1280</v>
       </c>
+      <c r="I395" t="s">
+        <v>1384</v>
+      </c>
       <c r="J395">
         <v>1600</v>
       </c>
@@ -23781,6 +24810,9 @@
       <c r="H396" t="s">
         <v>1280</v>
       </c>
+      <c r="I396" t="s">
+        <v>1384</v>
+      </c>
       <c r="J396">
         <v>4607</v>
       </c>
@@ -23821,6 +24853,9 @@
       <c r="H397" t="s">
         <v>1280</v>
       </c>
+      <c r="I397" t="s">
+        <v>1384</v>
+      </c>
       <c r="J397">
         <v>3942</v>
       </c>
@@ -23861,6 +24896,9 @@
       <c r="H398" t="s">
         <v>1280</v>
       </c>
+      <c r="I398" t="s">
+        <v>1384</v>
+      </c>
       <c r="J398">
         <v>6750</v>
       </c>
@@ -23901,6 +24939,9 @@
       <c r="H399" t="s">
         <v>1280</v>
       </c>
+      <c r="I399" t="s">
+        <v>1384</v>
+      </c>
       <c r="J399">
         <v>6400</v>
       </c>
@@ -23940,6 +24981,9 @@
       <c r="H400" t="s">
         <v>1280</v>
       </c>
+      <c r="I400" t="s">
+        <v>1384</v>
+      </c>
       <c r="J400">
         <v>1692</v>
       </c>
@@ -24022,6 +25066,9 @@
       <c r="H402" t="s">
         <v>1280</v>
       </c>
+      <c r="I402" t="s">
+        <v>1384</v>
+      </c>
       <c r="J402">
         <v>5133</v>
       </c>
@@ -24062,6 +25109,9 @@
       <c r="H403" t="s">
         <v>1280</v>
       </c>
+      <c r="I403" t="s">
+        <v>1384</v>
+      </c>
       <c r="J403">
         <v>1603</v>
       </c>
@@ -24101,6 +25151,9 @@
       <c r="H404" t="s">
         <v>1280</v>
       </c>
+      <c r="I404" t="s">
+        <v>1384</v>
+      </c>
       <c r="J404">
         <v>1</v>
       </c>
@@ -24227,6 +25280,9 @@
       <c r="H407" t="s">
         <v>1280</v>
       </c>
+      <c r="I407" t="s">
+        <v>1384</v>
+      </c>
       <c r="J407">
         <v>213</v>
       </c>
@@ -24480,6 +25536,9 @@
       <c r="H413" t="s">
         <v>1280</v>
       </c>
+      <c r="I413" t="s">
+        <v>1384</v>
+      </c>
       <c r="J413">
         <v>1520</v>
       </c>
@@ -24519,6 +25578,9 @@
       <c r="H414" t="s">
         <v>1280</v>
       </c>
+      <c r="I414" t="s">
+        <v>1384</v>
+      </c>
       <c r="J414">
         <v>2866</v>
       </c>
@@ -24685,6 +25747,9 @@
       <c r="H418" t="s">
         <v>1280</v>
       </c>
+      <c r="I418" t="s">
+        <v>1384</v>
+      </c>
       <c r="J418">
         <v>1500</v>
       </c>
@@ -24724,6 +25789,9 @@
       <c r="H419" t="s">
         <v>1280</v>
       </c>
+      <c r="I419" t="s">
+        <v>1384</v>
+      </c>
       <c r="J419">
         <v>2667</v>
       </c>
@@ -24819,7 +25887,7 @@
         <v>30</v>
       </c>
       <c r="M421" s="1">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="422" spans="1:13" x14ac:dyDescent="0.3">
@@ -24861,7 +25929,7 @@
         <v>30</v>
       </c>
       <c r="M422" s="1">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Set standard Understock DOI Min threshold to 45 days and Normal range from 45 days to DOI Max
</commit_message>
<xml_diff>
--- a/Master produk.xlsx
+++ b/Master produk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Argo\Project AI\DOI BULANAN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753BFE91-A066-4629-BFFD-A2ADF2C3197E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1954BFE6-1B86-4D5B-A82B-C88019E20311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7A4E4CA0-3C41-4699-9069-61742CAEF447}"/>
   </bookViews>
@@ -4569,7 +4569,7 @@
     <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="58.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -4952,7 +4952,7 @@
         <v>30</v>
       </c>
       <c r="M9" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -4994,7 +4994,7 @@
         <v>30</v>
       </c>
       <c r="M10" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -5078,7 +5078,7 @@
         <v>30</v>
       </c>
       <c r="M12" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -5120,7 +5120,7 @@
         <v>30</v>
       </c>
       <c r="M13" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
@@ -5162,7 +5162,7 @@
         <v>30</v>
       </c>
       <c r="M14" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -5204,7 +5204,7 @@
         <v>30</v>
       </c>
       <c r="M15" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
@@ -5246,7 +5246,7 @@
         <v>32</v>
       </c>
       <c r="M16" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -5287,7 +5287,7 @@
         <v>31</v>
       </c>
       <c r="M17" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
@@ -5539,7 +5539,7 @@
         <v>30</v>
       </c>
       <c r="M23" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
@@ -5707,7 +5707,7 @@
         <v>30</v>
       </c>
       <c r="M27" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
@@ -5749,7 +5749,7 @@
         <v>31</v>
       </c>
       <c r="M28" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
@@ -6168,7 +6168,7 @@
         <v>30</v>
       </c>
       <c r="M38" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
@@ -6336,7 +6336,7 @@
         <v>33</v>
       </c>
       <c r="M42" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
@@ -7637,7 +7637,7 @@
         <v>30</v>
       </c>
       <c r="M73" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.3">
@@ -8183,7 +8183,7 @@
         <v>30</v>
       </c>
       <c r="M86" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.3">
@@ -8225,7 +8225,7 @@
         <v>30</v>
       </c>
       <c r="M87" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.3">
@@ -10976,7 +10976,7 @@
         <v>30</v>
       </c>
       <c r="M153" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="154" spans="1:13" x14ac:dyDescent="0.3">
@@ -11186,7 +11186,7 @@
         <v>30</v>
       </c>
       <c r="M158" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="159" spans="1:13" x14ac:dyDescent="0.3">
@@ -11312,7 +11312,7 @@
         <v>30</v>
       </c>
       <c r="M161" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="162" spans="1:13" x14ac:dyDescent="0.3">
@@ -11354,7 +11354,7 @@
         <v>30</v>
       </c>
       <c r="M162" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="163" spans="1:13" x14ac:dyDescent="0.3">
@@ -11480,7 +11480,7 @@
         <v>34</v>
       </c>
       <c r="M165" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="166" spans="1:13" x14ac:dyDescent="0.3">
@@ -11816,7 +11816,7 @@
         <v>30</v>
       </c>
       <c r="M173" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="174" spans="1:13" x14ac:dyDescent="0.3">
@@ -12068,7 +12068,7 @@
         <v>30</v>
       </c>
       <c r="M179" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="180" spans="1:13" x14ac:dyDescent="0.3">
@@ -12151,7 +12151,7 @@
         <v>30</v>
       </c>
       <c r="M181" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="182" spans="1:13" x14ac:dyDescent="0.3">
@@ -12235,7 +12235,7 @@
         <v>30</v>
       </c>
       <c r="M183" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="184" spans="1:13" x14ac:dyDescent="0.3">
@@ -12403,7 +12403,7 @@
         <v>30</v>
       </c>
       <c r="M187" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="188" spans="1:13" x14ac:dyDescent="0.3">
@@ -12613,7 +12613,7 @@
         <v>31</v>
       </c>
       <c r="M192" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="193" spans="1:13" x14ac:dyDescent="0.3">
@@ -13449,7 +13449,7 @@
         <v>30</v>
       </c>
       <c r="M212" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="213" spans="1:13" x14ac:dyDescent="0.3">
@@ -13616,7 +13616,7 @@
         <v>34</v>
       </c>
       <c r="M216" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="217" spans="1:13" x14ac:dyDescent="0.3">
@@ -13658,7 +13658,7 @@
         <v>33</v>
       </c>
       <c r="M217" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="218" spans="1:13" x14ac:dyDescent="0.3">
@@ -13993,7 +13993,7 @@
         <v>30</v>
       </c>
       <c r="M225" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="226" spans="1:13" x14ac:dyDescent="0.3">
@@ -14035,7 +14035,7 @@
         <v>30</v>
       </c>
       <c r="M226" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="227" spans="1:13" x14ac:dyDescent="0.3">
@@ -14160,7 +14160,7 @@
         <v>32</v>
       </c>
       <c r="M229" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="230" spans="1:13" x14ac:dyDescent="0.3">
@@ -14202,7 +14202,7 @@
         <v>30</v>
       </c>
       <c r="M230" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="231" spans="1:13" x14ac:dyDescent="0.3">
@@ -14244,7 +14244,7 @@
         <v>30</v>
       </c>
       <c r="M231" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="232" spans="1:13" x14ac:dyDescent="0.3">
@@ -14285,7 +14285,7 @@
         <v>31</v>
       </c>
       <c r="M232" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="233" spans="1:13" x14ac:dyDescent="0.3">
@@ -14367,7 +14367,7 @@
         <v>30</v>
       </c>
       <c r="M234" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="235" spans="1:13" x14ac:dyDescent="0.3">
@@ -14408,7 +14408,7 @@
         <v>30</v>
       </c>
       <c r="M235" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="236" spans="1:13" x14ac:dyDescent="0.3">
@@ -14743,7 +14743,7 @@
         <v>30</v>
       </c>
       <c r="M243" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="244" spans="1:13" x14ac:dyDescent="0.3">
@@ -14785,7 +14785,7 @@
         <v>30</v>
       </c>
       <c r="M244" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="245" spans="1:13" x14ac:dyDescent="0.3">
@@ -14827,7 +14827,7 @@
         <v>33</v>
       </c>
       <c r="M245" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="246" spans="1:13" x14ac:dyDescent="0.3">
@@ -14995,7 +14995,7 @@
         <v>32</v>
       </c>
       <c r="M249" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="250" spans="1:13" x14ac:dyDescent="0.3">
@@ -15037,7 +15037,7 @@
         <v>34</v>
       </c>
       <c r="M250" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="251" spans="1:13" x14ac:dyDescent="0.3">
@@ -15079,7 +15079,7 @@
         <v>32</v>
       </c>
       <c r="M251" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="252" spans="1:13" x14ac:dyDescent="0.3">
@@ -15121,7 +15121,7 @@
         <v>33</v>
       </c>
       <c r="M252" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="253" spans="1:13" x14ac:dyDescent="0.3">
@@ -15162,7 +15162,7 @@
         <v>32</v>
       </c>
       <c r="M253" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="254" spans="1:13" x14ac:dyDescent="0.3">
@@ -15204,7 +15204,7 @@
         <v>32</v>
       </c>
       <c r="M254" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="255" spans="1:13" x14ac:dyDescent="0.3">
@@ -15246,7 +15246,7 @@
         <v>30</v>
       </c>
       <c r="M255" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="256" spans="1:13" x14ac:dyDescent="0.3">
@@ -15287,7 +15287,7 @@
         <v>30</v>
       </c>
       <c r="M256" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="257" spans="1:13" x14ac:dyDescent="0.3">
@@ -15329,7 +15329,7 @@
         <v>30</v>
       </c>
       <c r="M257" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="258" spans="1:13" x14ac:dyDescent="0.3">
@@ -15371,7 +15371,7 @@
         <v>30</v>
       </c>
       <c r="M258" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="259" spans="1:13" x14ac:dyDescent="0.3">
@@ -15665,7 +15665,7 @@
         <v>30</v>
       </c>
       <c r="M265" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="266" spans="1:13" x14ac:dyDescent="0.3">
@@ -15791,7 +15791,7 @@
         <v>30</v>
       </c>
       <c r="M268" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="269" spans="1:13" x14ac:dyDescent="0.3">
@@ -16043,7 +16043,7 @@
         <v>30</v>
       </c>
       <c r="M274" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="275" spans="1:13" x14ac:dyDescent="0.3">
@@ -16085,7 +16085,7 @@
         <v>30</v>
       </c>
       <c r="M275" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="276" spans="1:13" x14ac:dyDescent="0.3">
@@ -16127,7 +16127,7 @@
         <v>30</v>
       </c>
       <c r="M276" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="277" spans="1:13" x14ac:dyDescent="0.3">
@@ -16169,7 +16169,7 @@
         <v>31</v>
       </c>
       <c r="M277" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="278" spans="1:13" x14ac:dyDescent="0.3">
@@ -16211,7 +16211,7 @@
         <v>30</v>
       </c>
       <c r="M278" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="279" spans="1:13" x14ac:dyDescent="0.3">
@@ -16253,7 +16253,7 @@
         <v>31</v>
       </c>
       <c r="M279" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="280" spans="1:13" x14ac:dyDescent="0.3">
@@ -16295,7 +16295,7 @@
         <v>31</v>
       </c>
       <c r="M280" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="281" spans="1:13" x14ac:dyDescent="0.3">
@@ -16337,7 +16337,7 @@
         <v>32</v>
       </c>
       <c r="M281" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="282" spans="1:13" x14ac:dyDescent="0.3">
@@ -16421,7 +16421,7 @@
         <v>30</v>
       </c>
       <c r="M283" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="284" spans="1:13" x14ac:dyDescent="0.3">
@@ -16463,7 +16463,7 @@
         <v>30</v>
       </c>
       <c r="M284" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="285" spans="1:13" x14ac:dyDescent="0.3">
@@ -16505,7 +16505,7 @@
         <v>30</v>
       </c>
       <c r="M285" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="286" spans="1:13" x14ac:dyDescent="0.3">
@@ -16589,7 +16589,7 @@
         <v>33</v>
       </c>
       <c r="M287" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="288" spans="1:13" x14ac:dyDescent="0.3">
@@ -16631,7 +16631,7 @@
         <v>33</v>
       </c>
       <c r="M288" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="289" spans="1:13" x14ac:dyDescent="0.3">
@@ -16673,7 +16673,7 @@
         <v>30</v>
       </c>
       <c r="M289" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="290" spans="1:13" x14ac:dyDescent="0.3">
@@ -16715,7 +16715,7 @@
         <v>30</v>
       </c>
       <c r="M290" s="1">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="291" spans="1:13" x14ac:dyDescent="0.3">
@@ -16757,7 +16757,7 @@
         <v>30</v>
       </c>
       <c r="M291" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="292" spans="1:13" x14ac:dyDescent="0.3">
@@ -16883,7 +16883,7 @@
         <v>34</v>
       </c>
       <c r="M294" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="295" spans="1:13" x14ac:dyDescent="0.3">
@@ -17429,7 +17429,7 @@
         <v>31</v>
       </c>
       <c r="M307" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="308" spans="1:13" x14ac:dyDescent="0.3">
@@ -17471,7 +17471,7 @@
         <v>33</v>
       </c>
       <c r="M308" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="309" spans="1:13" x14ac:dyDescent="0.3">
@@ -17513,7 +17513,7 @@
         <v>33</v>
       </c>
       <c r="M309" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="310" spans="1:13" x14ac:dyDescent="0.3">
@@ -17555,7 +17555,7 @@
         <v>33</v>
       </c>
       <c r="M310" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="311" spans="1:13" x14ac:dyDescent="0.3">
@@ -17639,7 +17639,7 @@
         <v>32</v>
       </c>
       <c r="M312" s="1">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="313" spans="1:13" x14ac:dyDescent="0.3">
@@ -17681,7 +17681,7 @@
         <v>33</v>
       </c>
       <c r="M313" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="314" spans="1:13" x14ac:dyDescent="0.3">
@@ -17723,7 +17723,7 @@
         <v>34</v>
       </c>
       <c r="M314" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="315" spans="1:13" x14ac:dyDescent="0.3">
@@ -17891,7 +17891,7 @@
         <v>31</v>
       </c>
       <c r="M318" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="319" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Apply conditional Min DOI rule: 0 if Master Min is 0 else 45, and DOI Max from Master
</commit_message>
<xml_diff>
--- a/Master produk.xlsx
+++ b/Master produk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Argo\Project AI\DOI BULANAN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1954BFE6-1B86-4D5B-A82B-C88019E20311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{237D098F-2282-4402-8231-B2CBD4E2FD19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7A4E4CA0-3C41-4699-9069-61742CAEF447}"/>
   </bookViews>
@@ -15067,7 +15067,7 @@
         <v>1276</v>
       </c>
       <c r="I251" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
       <c r="J251">
         <v>13857</v>
@@ -15076,10 +15076,10 @@
         <v>1334</v>
       </c>
       <c r="L251" s="1">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="M251" s="1">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="252" spans="1:13" x14ac:dyDescent="0.3">
@@ -21112,7 +21112,7 @@
         <v>1279</v>
       </c>
       <c r="I395" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
       <c r="J395">
         <v>1600</v>
@@ -21121,10 +21121,10 @@
         <v>1328</v>
       </c>
       <c r="L395" s="1">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="M395" s="1">
-        <v>106</v>
+        <v>0</v>
       </c>
     </row>
     <row r="396" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>